<commit_message>
feat: upgrade reading creator agent with unified threaded scenario, 16:9 2D flat vector image standard, and interactive code sandboxes
</commit_message>
<xml_diff>
--- a/output/pms/Lập_trình_Python/Session 02 - Môi trường Python 3.12 và Cú pháp cơ bản/Session02._Quizz_Cuoi_Gio_Tổng_quan_về_ngôn_ngữ_Python_3_12.xlsx
+++ b/output/pms/Lập_trình_Python/Session 02 - Môi trường Python 3.12 và Cú pháp cơ bản/Session02._Quizz_Cuoi_Gio_Tổng_quan_về_ngôn_ngữ_Python_3_12.xlsx
@@ -539,59 +539,56 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>Cho đoạn mã nguồn Python sau đây thực hiện tính toán giá trị biểu thức toán tử:
+          <t>Một lập trình viên thực hiện nhập dữ liệu từ bàn phím qua console để tính tuổi cho năm sau bằng đoạn mã Python 3.12 như sau:
 ```python
-base_num = 2
-exp_num = 3
-factor_val = 4
-result_val = -base_num ** exp_num + factor_val * 3 // 2
-print(result_val)
+age_str = input("Nhập tuổi: ")
+next_age = age_str + 1
 ```
-Kết quả hiển thị ra màn hình sau khi chương trình thực thi là bao nhiêu?</t>
+Khi chạy chương trình, hệ thống phát sinh lỗi `TypeError`. Cách xử lý nào đúng nhất để chuyển đổi kiểu dữ liệu thành công?</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>Thực hiện ép kiểu bằng từ khóa `var age_str` ngay khi nhận dữ liệu để Python tự chuyển thành kiểu số nguyên.</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>Đáp án B sai. Đây là kết quả xuất phát từ suy luận sai lầm rằng toán tử đổi dấu `-` có độ ưu tiên cao hơn toán tử lũy thừa `**`, dẫn đến việc tính `(-2) ** 3 = -8`. Sau đó, người học nhầm dấu âm hoặc tính sai tổng `8 + 6 = 14`. Trong thực tế chuẩn của Python 3.12, lũy thừa `**` luôn được ưu tiên tính trước toán tử đổi dấu đơn thể.</t>
+          <t>Python không sử dụng từ khóa `var` để khai báo biến hay ép kiểu dữ liệu. Cú pháp này không tồn tại trong Python và sẽ gây lỗi cú pháp `SyntaxError`.</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>Sử dụng hàm `int(age_str)` để chuyển đổi chuỗi nhập từ console thành kiểu số nguyên trước khi thực hiện phép cộng số học.</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>Đáp án D sai. Kết quả này do áp dụng sai thứ tự tính toán từ trái sang phải mà không tuân theo bảng độ ưu tiên toán tử của Python, hoặc tính nhầm biểu thức lũy thừa kết hợp phép cộng `(-2) ** (3 + 4)`, dẫn tới giá trị tính toán sai hoàn toàn so với nguyên lý thực thi của ngôn ngữ.</t>
+          <t>Hàm `input()` trong Python luôn trả về dữ liệu thuộc kiểu chuỗi (`str`). Không thể thực hiện phép cộng trực tiếp giữa chuỗi và số nguyên (`int`). Việc dùng `int(age_str)` sẽ chuyển đổi chuỗi chữ số thành kiểu số nguyên hợp lệ để tính toán.</t>
         </is>
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
-          <t>-2</t>
+          <t>Thực hiện đổi tên biến `age_str` thành `age_int` để trình thông dịch Python tự động nhận diện thành kiểu số nguyên.</t>
         </is>
       </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
-          <t>Đáp án A đúng. Trong Python, toán tử lũy thừa `**` có độ ưu tiên cao hơn toán tử đổi dấu `-` (unary minus), nên biểu thức `-base_num ** exp_num` được đánh giá thành `-(2 ** 3) = -8`. Tiếp theo, các toán tử nhân `*` và chia lấy phần nguyên `//` có cùng mức ưu tiên và thực hiện theo thứ tự từ trái sang phải: `factor_val * 3` thành `4 * 3 = 12`, sau đó `12 // 2` thu được `6`. Cuối cùng, thực hiện toán tử cộng `+`: `-8 + 6 = -2` thuộc kiểu số nguyên `int`.</t>
+          <t>Đổi tên biến chỉ có tác dụng thay đổi định danh hiển thị trong mã nguồn, không ảnh hưởng đến kiểu dữ liệu thực tế của giá trị do hàm `input()` trả về.</t>
         </is>
       </c>
       <c r="I2" s="3" t="inlineStr">
         <is>
-          <t>-2.0</t>
+          <t>Sử dụng hàm `float(1)` để chuyển đổi số nguyên thành kiểu chuỗi ký tự trước khi thực hiện phép cộng nối chuỗi.</t>
         </is>
       </c>
       <c r="J2" s="3" t="inlineStr">
         <is>
-          <t>Đáp án C sai. Đây là bẫy nhầm lẫn về kiểu dữ liệu đầu ra. Người học cho rằng phép chia trong Python luôn trả về số thực kiểu `float`. Tuy nhiên, toán tử `//` là phép chia lấy phần nguyên (floor division). Khi cả hai toán hạng `12` và `2` đều là số nguyên kiểu `int`, kết quả phép chia trả về là `6` kiểu `int`, làm cho kết quả cuối cùng là `-2` kiểu `int` chứ không phải `-2.0` kiểu `float`.</t>
+          <t>Hàm `float(1)` trả về số thực `1.0` chứ không phải kiểu chuỗi ký tự (`str`), do đó phép cộng giữa chuỗi `age_str` và số thực vẫn gây ra lỗi `TypeError`.</t>
         </is>
       </c>
       <c r="K2" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L2" s="2" t="n">
         <v>6</v>
@@ -608,56 +605,47 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Cho đoạn mã Python thực hiện các toán tử số học chia lấy phần nguyên và chia lấy phần dư với số âm như sau:
-```python
-val_a = -15
-val_b = 4
-quotient_val = val_a // val_b
-remainder_val = val_a % val_b
-result_val = quotient_val + remainder_val
-print(result_val)
-```
-Giá trị của `result_val` được in ra màn hình console là bao nhiêu?</t>
+          <t>Khi phát triển một ứng dụng bằng Python 3.12, người lập trình cần tạo biến để lưu trữ điểm số của sinh viên đầu tiên. Tên biến nào sau đây tuân thủ đúng quy tắc đặt tên định danh (identifier) của Python?</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>`class` vì đây là từ khóa ngắn gọn và mô tả chính xác lớp học của sinh viên trong chương trình.</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>Đáp án D sai. Đây là lỗi khi người học áp dụng sai quy tắc dấu của toán tử chia lấy phần dư `%`, cho rằng phần dư mang dấu của số bị chia (`remainder_val = -3`) và kết hợp với việc làm tròn lên của thương (`quotient_val = -3`), dẫn đến tổng `-3 + 3 = 0`.</t>
+          <t>`class` là từ khóa dành riêng (reserved keyword) trong ngôn ngữ Python dùng để định nghĩa lớp, do đó không thể dùng làm tên biến.</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>-2</t>
+          <t>`1st_student_score` vì tên biến được phép bắt đầu bằng chữ số để thể hiện thứ tự của sinh viên.</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>Đáp án C sai. Nguyên nhân là do người học tính đúng `quotient_val = -4` nhưng lại hiểu sai cơ chế toán tử `%` với số chia dương, lầm tưởng số dư của phép chia `-15` cho `4` là `2` hoặc `-2`, dẫn đến kết quả tổng tính ra bị sai thành `-2`.</t>
+          <t>Tên biến `1st_student_score` vi phạm quy tắc đặt tên vì bắt đầu bằng chữ số `1`, dẫn đến lỗi cú pháp `SyntaxError` khi trình thông dịch xử lý.</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>-6</t>
+          <t>`student-score-1` vì tên biến cho phép sử dụng dấu gạch ngang để phân tách các từ trong tên.</t>
         </is>
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t>Đáp án B sai. Người học mắc phải bẫy tư duy từ các ngôn ngữ như C/C++ hay Java khi cho rằng phép chia lấy phần nguyên `//` sẽ cắt bỏ phần thập phân tiến về số 0 (truncate towards zero), coi `-15 // 4` bằng `-3`. Khi đó tính sai `remainder_val = -15 - (-3 * 4) = -3`, dẫn tới tổng `-3 + (-3) = -6`. Đây không phải cơ chế hoạt động của toán tử số học trong Python.</t>
+          <t>Tên biến `student-score-1` vi phạm quy tắc vì chứa ký tự gạch ngang (`-`), trình thông dịch Python sẽ hiểu nhầm đây là toán tử trừ số học.</t>
         </is>
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>-3</t>
+          <t>`student_score_1` vì tên biến chỉ chứa chữ cái, chữ số, dấu gạch dưới và không bắt đầu bằng chữ số.</t>
         </is>
       </c>
       <c r="J3" s="3" t="inlineStr">
         <is>
-          <t>Đáp án A đúng. Trong Python, toán tử chia lấy phần nguyên `//` thực hiện làm tròn xuống số nguyên gần nhất theo hướng âm vô cực (floor). Ta có `-15 / 4 = -3.75`, làm tròn xuống thành `-4`, nên `quotient_val = -4`. Toán tử chia lấy phần dư `%` được tính theo công thức `r = a - (a // b) * b`, tức là `remainder_val = -15 - (-4 * 4) = -15 - (-16) = 1`. Do đó, `result_val = quotient_val + remainder_val = -4 + 1 = -3`.</t>
+          <t>Trong Python, tên biến hợp lệ chỉ được bao gồm các chữ cái (a-z, A-Z), chữ số (0-9) và dấu gạch dưới (`_`), đồng thời tuyệt đối không được bắt đầu bằng chữ số.</t>
         </is>
       </c>
       <c r="K3" s="2" t="n">
@@ -678,59 +666,53 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Phân tích đoạn mã Python sử dụng chuỗi các toán tử gán phức hợp (compound assignment operators) dưới đây:
+          <t>Khi thực thi đoạn mã Python 3.12 để khởi tạo và kiểm tra kiểu dữ liệu cơ sở như sau:
 ```python
-total_score = 10
-multiplier_val = 3
-total_score += 5 * 2
-total_score //= multiplier_val
-total_score **= 2
-print(total_score)
+is_active = True
+total_price = 99.5
+print(type(is_active), type(total_price))
 ```
-Giá trị cuối cùng của `total_score` hiển thị ra màn hình là bao nhiêu?</t>
+Kết quả hiển thị chính xác trên màn hình console là gì?</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>`&lt;class 'boolean'&gt; &lt;class 'double'&gt;` đại diện cho kiểu dữ liệu luận lý (Boolean) và kiểu số thực.</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>Đáp án D sai. Người học mắc bẫy khi bỏ qua tác động của toán tử gán phức hợp chia lấy phần nguyên `total_score //= multiplier_val` hoặc tính nhầm `20 // 3` thành `10`, dẫn tới bước cuối cùng tính toán `10 ** 2 = 100`.</t>
+          <t>Python không sử dụng tên kiểu dữ liệu `boolean` hay `double` như một số ngôn ngữ khác, mà tên kiểu dữ liệu chuẩn là `bool` và `float`.</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>36.0</t>
+          <t>`&lt;class 'int'&gt; &lt;class 'decimal'&gt;` đại diện cho kiểu dữ liệu số nguyên và kiểu số thập phân chính xác.</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>Đáp án B sai. Đây là lỗi nhầm lẫn về kiểu dữ liệu (data type). Người học lầm tưởng rằng việc sử dụng các toán tử gán phức hợp như `//=` hay `**=` sẽ tự động ép kiểu biến sang số thực `float`. Vì tất cả các toán hạng tham gia trong chuỗi tính toán đều là kiểu số nguyên `int`, giá trị kết quả giữ nguyên kiểu `int` là `36` chứ không phải `36.0`.</t>
+          <t>Giá trị `True` được xác định là kiểu `bool` chứ không phải `int`, và `99.5` là kiểu số thực `float` cơ bản chứ không phải lớp `decimal`.</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>36</t>
+          <t>`&lt;class 'bool'&gt; &lt;class 'float'&gt;` đại diện cho kiểu dữ liệu luận lý (Boolean) và kiểu số thực.</t>
         </is>
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>Đáp án A đúng. Tiến trình biến đổi giá trị của biến `total_score` qua các toán tử gán phức hợp như sau:
-1. `total_score += 5 * 2`: Biểu thức vế phải `5 * 2 = 10` được tính trước, sau đó thực hiện cộng tích lũy `total_score = 10 + 10 = 20`.
-2. `total_score //= multiplier_val`: Thực hiện phép chia lấy phần nguyên `20 // 3 = 6` kết quả kiểu `int`.
-3. `total_score **= 2`: Thực hiện toán tử lũy thừa `6 ** 2 = 36` kết quả kiểu `int`.</t>
+          <t>Trong Python 3.12, giá trị `True` thuộc kiểu dữ liệu luận lý `bool` và số `99.5` chứa phần thập phân thuộc kiểu số thực `float`.</t>
         </is>
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>`&lt;class 'str'&gt; &lt;class 'float'&gt;` đại diện cho kiểu dữ liệu chuỗi ký tự và kiểu số thực trong Python.</t>
         </is>
       </c>
       <c r="J4" s="3" t="inlineStr">
         <is>
-          <t>Đáp án C sai. Lỗi này xảy ra khi người học tính toán sai câu lệnh `total_score += 5 * 2` do thực hiện phép cộng trước từ trái sang phải `(10 + 5) * 2 = 30`, từ đó dẫn tới các bước tính toán tiếp theo bị sai lệch hoàn toàn so với thứ tự ưu tiên toán tử chuẩn.</t>
+          <t>Giá trị `True` là một hằng số Boolean nguyên bản, không phải chuỗi ký tự (`str`) vì không được đặt trong cặp dấu báo chuỗi (dấu ngoặc đơn hoặc ngoặc kép).</t>
         </is>
       </c>
       <c r="K4" s="2" t="n">
@@ -751,60 +733,47 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Cho đoạn mã Python thực thi các toán tử số học cơ bản để tính toán mã số định danh như sau:
-```python
-total_items = 27
-box_capacity = 4
-full_boxes = total_items // box_capacity
-remaining_items = total_items % box_capacity
-result_code = remaining_items ** 3 + full_boxes
-print(result_code)
-```
-Kết quả in ra màn hình console là bao nhiêu?</t>
+          <t>Trong ngôn ngữ lập trình Python, khi khởi tạo biến để lưu trữ điểm số của người dùng, tên biến nào sau đây là hợp lệ và không gây ra lỗi cú pháp (`SyntaxError`)?</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>216</t>
+          <t>`user score 2024`</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>Bẫy tư duy sai lầm: Học viên vi phạm quy tắc độ ưu tiên toán tử (Operator Precedence). Nhầm tưởng phép cộng `+` được thực hiện trước lũy thừa `**` theo thứ tự từ trái sang phải thành `3 ** (3 + 6) = 3 ** 9` hoặc thực hiện nhân/lũy thừa sai thứ tự biến. Theo chuẩn Python, toán tử lũy thừa `**` luôn được ưu tiên tính trước toán tử cộng `+`.</t>
+          <t>Tên biến `user score 2024` không hợp lệ vì chứa khoảng trắng, vi phạm quy tắc tên biến phải là một chuỗi ký tự liền mạch.</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>`_user_score_2024`</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>Đáp án đúng. Phân tích chi tiết từng bước toán tử trong đoạn mã:
-1. `total_items // box_capacity` thực hiện toán tử chia lấy phần nguyên: `27 // 4 = 6` (gán cho `full_boxes`).
-2. `total_items % box_capacity` thực hiện toán tử chia lấy phần dư: `27 % 4 = 3` (gán cho `remaining_items`).
-3. Toán tử lũy thừa `**` có độ ưu tiên cao hơn toán tử cộng `+`. Do đó, `remaining_items ** 3` được tính trước: `3 ** 3 = 27`.
-4. Sau đó thực hiện phép cộng với `full_boxes`: `27 + 6 = 33`.</t>
+          <t>Tên biến `_user_score_2024` hợp lệ theo đúng quy tắc đặt tên của Python vì tên biến có thể bắt đầu bằng dấu gạch dưới (`_`) và theo sau bởi các chữ cái, chữ số hoặc dấu gạch dưới.</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>12.75</t>
+          <t>`2024_user_score`</t>
         </is>
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>Bẫy tư duy sai lầm: Học viên nhầm lẫn toán tử chia lấy phần nguyên `//` và chia lấy phần dư `%` với toán tử chia thực `/`. Nếu tính `27 / 4 = 6.75`, dẫn đến xác định sai giá trị kiểu số nguyên của `full_boxes` và `remaining_items`, tạo ra kết quả dạng số thực `float` thay vì số nguyên `int`.</t>
+          <t>Tên biến `2024_user_score` không hợp lệ vì cú pháp ngôn ngữ Python quy định tên biến không được phép bắt đầu bằng chữ số, vi phạm quy tắc sẽ dẫn đến lỗi `SyntaxError`.</t>
         </is>
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>`user-score-2024`</t>
         </is>
       </c>
       <c r="J5" s="3" t="inlineStr">
         <is>
-          <t>Bẫy tư duy sai lầm: Học viên nhầm lẫn toán tử lũy thừa `**` với phép nhân `*`. Nếu hiểu nhầm `3 ** 3` thành `3 * 3 = 9`, thì phép tính trở thành `9 + 6 = 15`. Trong Python, `**` đại diện cho lũy thừa (số mũ), còn `*` mới là phép nhân.</t>
+          <t>Tên biến `user-score-2024` không hợp lệ vì dấu gạch ngang (`-`) được trình biên dịch/thông dịch hiểu là toán tử số học trừ chứ không phải ký tự hợp lệ trong tên biến.</t>
         </is>
       </c>
       <c r="K5" s="2" t="n">
@@ -825,64 +794,55 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Cho đoạn mã Python sử dụng toán tử nhân `*` và cộng `+` kết hợp ép kiểu dữ liệu như sau:
+          <t>Một chương trình Python nhận dữ liệu từ bàn phím thông qua đoạn mã sau:
 ```python
-unit_code = "5"
-repeat_count = 3
-calculated_val = int(unit_code) * repeat_count
-raw_pattern = unit_code * repeat_count
-output_result = int(raw_pattern) + calculated_val
-print(output_result)
+age_input = input("Nhập số tuổi: ")
 ```
-Kết quả in ra màn hình console là bao nhiêu?</t>
+Khi người dùng nhập vào chuỗi `"25"`, giá trị biến `age_input` có kiểu dữ liệu mặc định là `str`. Câu lệnh nào sau đây chuyển đổi giá trị của `age_input` thành số nguyên để lưu vào biến `age` một cách chính xác?</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>55515</t>
+          <t>`age = str(age_input)`</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>Bẫy tư duy sai lầm: Học viên nghĩ rằng biểu thức `output_result` thực hiện toán tử nối chuỗi (string concatenation) do không chú ý hàm `int(raw_pattern)` đã chuyển đổi `raw_pattern` về kiểu `int`. Nếu nối chuỗi `"555" + "15"` sẽ ra `"55515"`, nhưng ở đây cả 2 vế đều là số nguyên `int` nên thực hiện phép cộng số học.</t>
+          <t>Hàm `str()` thực hiện chuyển đổi thành kiểu chuỗi ký tự, giữ nguyên biến `age` ở kiểu `str` chứ không chuyển đổi về số nguyên.</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>555</t>
+          <t>`age = float(age_input)`</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>Bẫy tư duy sai lầm: Học viên bỏ sót biểu thức cộng `+ calculated_val` ở dòng gán `output_result` hoặc hiểu nhầm rằng phép chuyển đổi `int(raw_pattern)` đè lên kết quả tính toán trước đó, dẫn đến chỉ lấy giá trị `555`.</t>
+          <t>Hàm `float()` chuyển đổi chuỗi thành số thực (`25.0`) thuộc kiểu `float`, không tạo ra số nguyên thuộc kiểu `int`.</t>
         </is>
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>570</t>
+          <t>`age = type(age_input)`</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
-          <t>Đáp án đúng. Phân tích chi tiết luồng xử lý toán tử:
-1. `int(unit_code)` ép chuỗi `"5"` thành số nguyên `5`. Sau đó `5 * 3` thực hiện toán tử nhân số học cho ra `calculated_val = 15`.
-2. `unit_code * repeat_count` thực hiện toán tử lặp chuỗi (string repetition): `"5" * 3` cho ra chuỗi `"555"` (gán cho `raw_pattern`).
-3. `int(raw_pattern)` ép chuỗi `"555"` thành số nguyên `555`.
-4. `555 + 15` thực hiện toán tử cộng số học thu được kết quả `570`.</t>
+          <t>Hàm `type()` dùng để kiểm tra kiểu dữ liệu của đối tượng và trả về `&lt;class 'str'&gt;` chứ không có chức năng ép kiểu dữ liệu của giá trị.</t>
         </is>
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>`age = int(age_input)`</t>
         </is>
       </c>
       <c r="J6" s="3" t="inlineStr">
         <is>
-          <t>Bẫy tư duy sai lầm: Học viên nhầm lẫn hành vi của toán tử `*` khi làm việc với kiểu chuỗi `str`. Nhầm tưởng `"5" * 3` cũng thực hiện phép nhân số học ra `15`, dẫn đến `raw_pattern = 15` và phép cộng cuối cùng là `15 + 15 = 30`. Trong Python, toán tử `*` giữa `str` và `int` thực hiện lặp chuỗi chứ không nhân giá trị số.</t>
+          <t>Hàm `int()` nhận đối số là một chuỗi ký tự biểu diễn số nguyên (như `"25"`) và thực hiện ép kiểu thành số nguyên `25` chính xác.</t>
         </is>
       </c>
       <c r="K6" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L6" s="2" t="n">
         <v>6</v>
@@ -899,64 +859,51 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Cho đoạn mã Python sử dụng các toán tử gán kết hợp (Compound Assignment Operators) và toán tử số học như sau:
-```python
-base_score = 10
-bonus_multiplier = 2
-base_score += 5 * bonus_multiplier
-base_score *= 2
-base_score -= 4 // 2
-print(base_score)
-```
-Kết quả hiển thị trên màn hình console là gì?</t>
+          <t>Ngôn ngữ Python 3.12 áp dụng cơ chế định kiểu động (dynamic typing). Cơ chế này thể hiện qua đặc điểm nào sau đây khi khai báo và gán giá trị cho biến?</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>38</t>
+          <t>Kiểu dữ liệu của biến phụ thuộc vào cách đặt tên biến chứ không liên quan đến đối tượng giá trị được gán cho biến.</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>Đáp án đúng. Phân tích từng bước thay đổi giá trị biến qua các toán tử gán phức hợp:
-1. `base_score += 5 * bonus_multiplier`: Phép nhân `5 * 2 = 10` được tính trước. Sau đó `base_score = 10 + 10 = 20`.
-2. `base_score *= 2`: Nhân đôi giá trị hiện tại `base_score = 20 * 2 = 40`.
-3. `base_score -= 4 // 2`: Phép chia lấy phần nguyên `4 // 2 = 2` được thực hiện trước. Sau đó `base_score = 40 - 2 = 38`.
-Kết quả cuối cùng thu được số nguyên `38`.</t>
+          <t>Quy tắc đặt tên biến không quyết định kiểu dữ liệu của biến; kiểu dữ liệu hoàn toàn do đối tượng giá trị mà biến đang tham chiếu quyết định.</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>Kiểu dữ liệu của biến phải được khai báo cố định trước khi gán và không thể gán giá trị thuộc kiểu dữ liệu khác trong suốt chương trình.</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>Bẫy tư duy sai lầm: Học viên tính toán sai bước `base_score += 5 * bonus_multiplier` khi quên cộng giá trị ban đầu của `base_score` (10), mà lại gán trực tiếp `base_score = 5 * 2 = 10`. Từ đó `10 * 2 = 20` và `20 - 2 = 18` hoặc tính sai thứ tự gán ở các dòng sau dẫn tới giá trị `28`.</t>
+          <t>Đây là đặc điểm của các ngôn ngữ định kiểu tĩnh (static typing) như C, C++ hoặc Java, không phải đặc điểm định kiểu động của Python.</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t>58</t>
+          <t>Kiểu dữ liệu của biến chỉ được kiểm tra duy nhất một lần ở giai đoạn biên dịch trước khi chương trình được mã hóa thành tệp nhị phân.</t>
         </is>
       </c>
       <c r="H7" s="3" t="inlineStr">
         <is>
-          <t>Bẫy tư duy sai lầm: Học viên vi phạm độ ưu tiên toán tử số học khi tính dòng `base_score += 5 * bonus_multiplier`. Nhầm tưởng phép cộng được tính trước: `(10 + 5) * 2 = 30`, từ đó `base_score` thành `30`. Tiếp tục `30 * 2 = 60` và `60 - 2 = 58`. Quy tắc Python bắt buộc thực hiện phép nhân `5 * 2` trước phép gán cộng `+=`.</t>
+          <t>Python kiểm tra và xử lý kiểu dữ liệu trực tiếp trong quá trình thực thi (runtime) thay vì bắt buộc kiểm tra cố định ở bước biên dịch trước.</t>
         </is>
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>38.0</t>
+          <t>Kiểu dữ liệu của biến được tự động xác định dựa trên giá trị được gán tại thời điểm thực thi mà không cần khai báo trước kiểu dữ liệu.</t>
         </is>
       </c>
       <c r="J7" s="3" t="inlineStr">
         <is>
-          <t>Bẫy tư duy sai lầm: Học viên nhầm lẫn giữa toán tử chia thực `/` và toán tử chia lấy phần nguyên `//`. Nếu sử dụng `/`, phép tính `4 / 2` trả về số thực `2.0` làm cho `base_score` chuyển thành kiểu `float` (`38.0`). Tuy nhiên, toán tử `//` giữa 2 số nguyên trả về kiểu `int` (`2`), giữ nguyên kiểu số nguyên cho `base_score`.</t>
+          <t>Trong cơ chế định kiểu động của Python, lập trình viên không cần khai báo kiểu dữ liệu cho biến trước; kiểu dữ liệu của biến được hệ thống tự động nhận diện dựa vào giá trị mà biến đó tham chiếu tới tại thời điểm runtime.</t>
         </is>
       </c>
       <c r="K7" s="2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="L7" s="2" t="n">
         <v>6</v>
@@ -973,59 +920,56 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Trong một hệ thống quản lý kho hàng, lập trình viên thực thi đoạn mã Python 3.12 sau để tính số lượng thùng hàng nguyên chiếc và số sản phẩm lẻ còn dư:
+          <t>Khi thực thi một chương trình Python 3.12 xử lý dữ liệu nhập từ người dùng với đoạn mã dưới đây, kết quả hiển thị ra màn hình console là gì nếu người dùng nhập vào giá trị `20`?
 ```python
-total_items = 27
-box_capacity = 4
-full_boxes = total_items // box_capacity
-remaining_items = total_items % box_capacity
-print(full_boxes, remaining_items)
-```
-Kết quả hiển thị trên màn hình console là gì?</t>
+user_data = input("Nhập dữ liệu: ")
+result = int(user_data) + 10
+print(type(user_data), type(result))
+```</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>6.75 3</t>
+          <t>&lt;class 'int'&gt; &lt;class 'int'&gt;</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>Sai. Đáp án này nhầm lẫn toán tử chia lấy phần nguyên `//` với toán tử chia số thực `/`. Phép tính `27 / 4` mới trả về `6.75` (kiểu `float`), trong khi toán tử `//` cắt bỏ hoàn toàn phần thập phân và trả về số nguyên `6` (kiểu `int`).</t>
+          <t>Phân tích sai vì hàm `input()` không tự động chuyển đổi chuỗi chữ số nhập vào thành kiểu số nguyên `int` nếu không gọi hàm chuyển kiểu dữ liệu.</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>6 3</t>
+          <t>&lt;class 'int'&gt; &lt;class 'str'&gt;</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>Đúng. Toán tử chia lấy phần nguyên `//` thực hiện `27 // 4` cho kết quả kiểu số nguyên là `6` (số thùng hàng hoàn chỉnh). Toán tử chia lấy phần dư `%` thực hiện `27 % 4` cho kết quả là `3` (số sản phẩm còn dư). Hàm `print` mặc định phân tách các tham số bằng một khoảng trắng nên in ra `6 3`.</t>
+          <t>Phân tích sai vì xác định ngược kiểu dữ liệu của biến `user_data` và biến `result`.</t>
         </is>
       </c>
       <c r="G8" s="3" t="inlineStr">
         <is>
-          <t>6.75 0.75</t>
+          <t>&lt;class 'str'&gt; &lt;class 'str'&gt;</t>
         </is>
       </c>
       <c r="H8" s="3" t="inlineStr">
         <is>
-          <t>Sai. Đáp án này nhầm lẫn hoàn toàn chức năng của cả hai toán tử `//` và `%` với phép chia thập phân thông thường. Toán tử `//` trả về kết quả số nguyên `6` và toán tử `%` trả về số dư nguyên `3`, không tạo ra bất kỳ giá trị số thực nào trong đoạn mã này.</t>
+          <t>Phân tích sai vì phép toán `int(user_data) + 10` tạo ra một số nguyên, hàm `int()` không giữ nguyên kiểu chuỗi ban đầu của dữ liệu.</t>
         </is>
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>6 0.75</t>
+          <t>&lt;class 'str'&gt; &lt;class 'int'&gt;</t>
         </is>
       </c>
       <c r="J8" s="3" t="inlineStr">
         <is>
-          <t>Sai. Đáp án này hiểu sai bản chất của toán tử chia lấy phần dư `%`. Toán tử `%` trả về số dư nguyên còn lại sau phép chia nguyên (ở đây là `3`), chứ không phải phần thập phân thu được từ phép chia số thực (`0.75`).</t>
+          <t>Hàm `input()` trong Python 3.12 luôn trả về dữ liệu thuộc kiểu chuỗi ký tự (`str`), do đó `type(user_data)` trả về `&lt;class 'str'&gt;`. Sau khi sử dụng hàm `int()` để chuyển đổi kiểu dữ liệu thành công, biến `result` chứa số nguyên `30` nên `type(result)` trả về `&lt;class 'int'&gt;`.</t>
         </is>
       </c>
       <c r="K8" s="2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L8" s="2" t="n">
         <v>6</v>
@@ -1042,57 +986,51 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Cho đoạn mã Python 3.12 thực hiện tính toán biểu thức dưới đây:
-```python
-base_val = 2
-result_val = 10 + 3 * base_val ** 3 // 4
-print(result_val)
-```
-Giá trị của biến `result_val` được in ra màn hình console là bao nhiêu?</t>
+          <t>Trong quá trình thiết kế mã nguồn Python 3.12 để lưu trữ thông tin ứng dụng, việc khởi tạo biến cần đảm bảo quy tắc đặt tên hợp lệ theo chuẩn ngôn ngữ. Tên biến nào sau đây là hợp lệ?</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>Biến _total_amount_2024 (bắt đầu bằng dấu gạch dưới, kết hợp chữ cái và chữ số).</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>Sai. Đáp án này mắc bẫy nhầm lẫn độ ưu tiên giữa toán tử nhân `*` và lũy thừa `**`. Lỗi này xảy ra nếu lấy `3 * base_val` (`3 * 2 = 6`) trước, rồi mới tính lũy thừa 3 (`6 ** 3 = 216`), dẫn đến phép tính `10 + 216 // 4 = 64` hoặc các sai sót tính toán khác.</t>
+          <t>Tên biến trong Python hợp lệ khi bắt đầu bằng một chữ cái hoặc dấu gạch dưới (`_`), theo sau là chữ cái, chữ số hoặc dấu gạch dưới. Biến `_total_amount_2024` tuân thủ đầy đủ quy tắc này.</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>52</t>
+          <t>Biến total amount 2024 (bắt đầu bằng chữ cái, chứa khoảng trắng giữa các từ).</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>Sai. Đáp án này mắc bẫy thực hiện các phép tính tuần tự từ trái sang phải mà bỏ qua thứ tự ưu tiên toán tử. Lỗi này xảy ra nếu lấy `(10 + 3) * 2` trước (= `26`), sau đó lấy `26 ** 3 // 4` dẫn tới kết quả hoàn toàn sai lệch.</t>
+          <t>Tên biến `total amount 2024` không hợp lệ vì chứa khoảng trắng giữa các từ, gây lỗi cú pháp khi phân tích mã nguồn.</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>16.0</t>
+          <t>Biến total-amount-2024 (bắt đầu bằng chữ cái, kết hợp dấu gạch ngang và chữ số).</t>
         </is>
       </c>
       <c r="H9" s="3" t="inlineStr">
         <is>
-          <t>Sai. Đáp án này mắc bẫy kiểu dữ liệu trả về. Phép chia lấy phần nguyên `//` giữa hai số nguyên (`24 // 4`) trả về kết quả là số nguyên `6` (kiểu `int`), do đó phép cộng `10 + 6` cho ra số nguyên `16`, không phải số thực `16.0` (kiểu `float`). Phép chia số thực `/` mới trả về kiểu `float`.</t>
+          <t>Tên biến `total-amount-2024` không hợp lệ vì chứa ký tự gạch ngang (`-`), ký tự này bị trình biên dịch Python nhận diện là toán tử trừ.</t>
         </is>
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>Biến 2024_total_amount (bắt đầu bằng chữ số, kết hợp dấu gạch dưới và chữ cái).</t>
         </is>
       </c>
       <c r="J9" s="3" t="inlineStr">
         <is>
-          <t>Đúng. Theo quy tắc thứ tự ưu tiên toán tử trong Python: (1) Toán tử lũy thừa `**` có độ ưu tiên cao nhất: `base_val ** 3` = `2 ** 3` = `8`. (2) Toán tử nhân `*` và chia lấy phần nguyên `//` có cùng độ ưu tiên, thực hiện lần lượt từ trái sang phải: `3 * 8` = `24`, sau đó `24 // 4` = `6`. (3) Toán tử cộng `+` có độ ưu tiên thấp nhất: `10 + 6` = `16` (kiểu số nguyên `int`).</t>
+          <t>Tên biến `2024_total_amount` không hợp lệ vì cú pháp Python cấm đặt tên biến bắt đầu bằng ký tự chữ số.</t>
         </is>
       </c>
       <c r="K9" s="2" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="L9" s="2" t="n">
         <v>6</v>
@@ -1109,58 +1047,59 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Trong Python 3.12, toán tử `*` và `+` có thể được áp dụng trên kiểu dữ liệu chuỗi (`str`). Hãy xác định kết quả in ra của đoạn mã sau:
+          <t>Khi thực thi đoạn mã nguồn Python 3.12 dưới đây trong ứng dụng xử lý dữ liệu:
 ```python
-prefix_code = "PY"
-repeat_count = 3
-suffix_code = "312"
-formatted_text = prefix_code * repeat_count + suffix_code
-print(formatted_text)
-```</t>
+num_a = "20"
+num_b = "30"
+combined = num_a + num_b
+total = int(num_a) + int(num_b)
+print(combined, total)
+```
+Kết quả hiển thị ra màn hình console là gì?</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>PY333312</t>
+          <t>Dòng chữ "2030 50" (chuỗi "2030" ghép từ hai chuỗi và số 50 từ tổng số nguyên).</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>Sai. Đáp án này hiểu sai cơ chế lặp của toán tử `*`. Toán tử `*` nhân bản toàn bộ nội dung của chuỗi `prefix_code` (`"PY"`) đúng `repeat_count` (`3`) lần để thành `"PYPYPY"`, chứ không phải chỉ lặp ký tự cuối hoặc nhân số vào sau chuỗi.</t>
+          <t>Toán tử `+` khi thao tác trên hai chuỗi ký tự (`"20"` và `"30"`) sẽ thực hiện phép nối chuỗi tạo thành `"2030"`. Khi ép kiểu hai biến về số nguyên bằng `int()`, toán tử `+` thực hiện phép cộng số học giữa `20` và `30` tạo thành kết quả `50`.</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>Báo lỗi TypeError: can't multiply sequence by non-int</t>
+          <t>Dòng chữ "2030 2030" (hàm int() không làm thay đổi kết quả của phép cộng chuỗi ban đầu).</t>
         </is>
       </c>
       <c r="F10" s="3" t="inlineStr">
         <is>
-          <t>Sai. Đáp án này hiểu sai rằng toán tử `*` không thể áp dụng cho chuỗi. Trong Python, nhân chuỗi (`str`) với một số nguyên (`int`) là cú pháp hoàn toàn hợp lệ dùng để nhân bản chuỗi. Ngoại lệ `TypeError` chỉ xuất hiện nếu nhân chuỗi với số thực `float` hoặc nhân hai chuỗi với nhau.</t>
+          <t>Phân tích sai vì hàm `int()` đã chuyển đổi thành công hai chuỗi số thành kiểu số nguyên, làm cho phép cộng `int(num_a) + int(num_b)` trả về kết quả số học `50` chứ không phải chuỗi ghép.</t>
         </is>
       </c>
       <c r="G10" s="3" t="inlineStr">
         <is>
-          <t>PYPYPY 312</t>
+          <t>Dòng chữ "50 2030" (phép cộng chuỗi tạo ra số 50 và phép ép kiểu int() tạo ra chuỗi ghép).</t>
         </is>
       </c>
       <c r="H10" s="3" t="inlineStr">
         <is>
-          <t>Sai. Đáp án này mắc bẫy ký tự khoảng trắng. Toán tử cộng chuỗi `+` trong Python ghép nối trực tiếp các ký tự của hai chuỗi liền kề nhau mà không tự động thêm bất kỳ khoảng trắng nào vào giữa.</t>
+          <t>Phân tích sai vì đệm ngược vị trí giữa kết quả của phép nối chuỗi (`combined`) và kết quả của phép cộng số nguyên (`total`).</t>
         </is>
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>PYPYPY312</t>
+          <t>Dòng chữ "50 50" (cả hai biến tự động chuyển sang kiểu số nguyên để thực hiện phép cộng).</t>
         </is>
       </c>
       <c r="J10" s="3" t="inlineStr">
         <is>
-          <t>Đúng. Trong Python, toán tử `*` giữa một chuỗi (`str`) và một số nguyên (`int`) thực hiện phép lặp chuỗi (`"PY" * 3` tạo ra `"PYPYPY"`). Tiếp theo, toán tử `+` thực hiện phép nối hai chuỗi (`"PYPYPY" + "312"`), tạo ra chuỗi kết quả cuối cùng là `"PYPYPY312"`.</t>
+          <t>Phân tích sai vì Python không tự động chuyển kiểu chuỗi thành số nguyên trong phép cộng hai chuỗi `num_a` và `num_b`.</t>
         </is>
       </c>
       <c r="K10" s="2" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="L10" s="2" t="n">
         <v>6</v>
@@ -1177,56 +1116,47 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>Cho đoạn mã Python thực thi các toán tử số học cơ bản như sau:
-```python
-total_items = 25
-items_per_box = 4
-full_boxes = total_items // items_per_box
-remaining_items = total_items % items_per_box
-result_summary = full_boxes + remaining_items / 2
-print(result_summary)
-```
-Giá trị được in ra màn hình console sau khi chạy đoạn mã trên là bao nhiêu?</t>
+          <t>Trong quá trình khởi tạo các biến lưu trữ thông tin nhân sự trên Python 3.12, khai báo nào sau đây tuân thủ đúng quy tắc đặt tên biến (variable naming convention) và không gây ra lỗi cú pháp (`SyntaxError`)?</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>`7`</t>
+          <t>`employee@id = 101`</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>Sai do nhầm lẫn toán tử chia số nguyên: Học viên hiểu nhầm toán tử `//` sẽ làm tròn lên (rounding up) kết quả chia `25 / 4` thành `7` thay vì lấy phần nguyên `6`.</t>
+          <t>Tên biến `employee@id` không hợp lệ vì chứa ký tự đặc biệt `@`, đây là ký tự không được phép sử dụng trong tên định danh của Python.</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>`6.5`</t>
+          <t>`_employee_id = 101`</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>Đúng vì toán tử `//` thực hiện chia lấy phần nguyên (`25 // 4` ra `6`), toán tử `%` lấy phần dư (`25 % 4` ra `1`). Trong Python, toán tử chia `/` giữa hai số nguyên (`1 / 2`) luôn trả về kết quả kiểu `float` là `0.5`. Phép cộng `6 + 0.5` cho kết quả cuối cùng là `6.5` kiểu số thực (`float`).</t>
+          <t>Tên biến `_employee_id` hợp lệ vì trong Python, tên biến có thể bắt đầu bằng chữ cái hoặc dấu gạch dưới (`_`), theo sau là các chữ cái, chữ số hoặc dấu gạch dưới.</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
         <is>
-          <t>`6`</t>
+          <t>`employee-id = 101`</t>
         </is>
       </c>
       <c r="H11" s="3" t="inlineStr">
         <is>
-          <t>Sai do bẫy tư duy toán tử chia trong một số ngôn ngữ lập trình khác: Học viên nhầm tưởng toán tử chia `/` giữa hai số nguyên `1 / 2` sẽ làm tròn xuống lấy số nguyên `0`, dẫn đến kết quả `6 + 0 = 6`.</t>
+          <t>Tên biến `employee-id` không hợp lệ vì dấu gạch nối (`-`) không được chấp nhận trong tên biến và trình biên dịch sẽ hiểu lầm đây là phép toán trừ.</t>
         </is>
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>`6.0`</t>
+          <t>`2nd_employee_id = 101`</t>
         </is>
       </c>
       <c r="J11" s="3" t="inlineStr">
         <is>
-          <t>Sai do tính toán sai phần dư: Học viên xác định đúng kết quả trả về mang kiểu `float` nhưng lại tính nhầm phép chia phần dư `remaining_items` bằng `0`, từ đó tính `6 + 0.0 = 6.0`.</t>
+          <t>Tên biến `2nd_employee_id` không hợp lệ vì cú pháp Python cấm đặt tên biến bắt đầu bằng một chữ số, dẫn đến lỗi `SyntaxError` khi thực thi.</t>
         </is>
       </c>
       <c r="K11" s="2" t="n">
@@ -1247,55 +1177,47 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>Xem xét đoạn mã Python sử dụng toán tử trên chuỗi và số nguyên dưới đây:
-```python
-prefix = "Py"
-count = 2
-suffix = "3"
-result_text = prefix * count + suffix * (count + 1)
-print(result_text)
-```
-Kết quả hiển thị trên màn hình console sau khi thực thi là gì?</t>
+          <t>Khi thực hiện nhận số lượng sản phẩm nhập từ bàn phím bằng hàm `input()` trong Python để phục vụ tính toán số học, đoạn mã nào sau đây chuyển đổi kiểu dữ liệu sang số nguyên (`int`) đúng cú pháp?</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>`"PyPy333"`</t>
+          <t>`quantity = int(input("Nhập số lượng: "))`</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>Đúng vì toán tử `*` giữa một chuỗi (`str`) và một số nguyên (`int`) hoạt động như toán tử lặp chuỗi. Biểu thức `prefix * 2` tạo ra `"PyPy"`. Biểu thức `count + 1` bằng `3` nên `suffix * 3` (tức `"3" * 3`) tạo ra `"333"`. Toán tử `+` thực hiện nối hai chuỗi lại thành `"PyPy333"`.</t>
+          <t>Hàm `input()` luôn trả về dữ liệu kiểu chuỗi (`str`), do đó việc bọc hàm `input()` bên trong hàm khởi tạo `int()` là cách chính xác để chuyển đổi dữ liệu nhập vào thành kiểu số nguyên.</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>`"Py233"`</t>
+          <t>`quantity = (int)input("Nhập số lượng: ")`</t>
         </is>
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>Sai do nhầm lẫn chức năng toán tử: Học viên lầm tưởng toán tử `*` khi dùng với chuỗi `prefix` và biến `count` sẽ chuyển số `2` thành chuỗi và ghép trực tiếp thành `"Py2"`.</t>
+          <t>Cú pháp ép kiểu dạng `(int)` là cú pháp của các ngôn ngữ khác như C/C++ hoặc Java, không phải cú pháp hợp lệ của Python và sẽ gây ra lỗi `SyntaxError`.</t>
         </is>
       </c>
       <c r="G12" s="3" t="inlineStr">
         <is>
-          <t>`TypeError`</t>
+          <t>`quantity = input("Nhập số lượng: ").to_int()`</t>
         </is>
       </c>
       <c r="H12" s="3" t="inlineStr">
         <is>
-          <t>Sai do hiểu sai quy tắc syntax trong Python: Học viên nghĩ rằng không thể dùng toán tử `*` giữa dữ liệu kiểu `str` và `int` nên trình biên dịch/thông dịch sẽ báo lỗi kiểu dữ liệu `TypeError`.</t>
+          <t>Phương thức `.to_int()` không tồn tại đối với đối tượng chuỗi (`str`) trong Python, việc gọi phương thức này sẽ làm phát sinh lỗi `AttributeError`.</t>
         </is>
       </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t>`"PyPy9"`</t>
+          <t>`quantity = integer(input("Nhập số lượng: "))`</t>
         </is>
       </c>
       <c r="J12" s="3" t="inlineStr">
         <is>
-          <t>Sai do nhầm lẫn ép kiểu tự động: Học viên cho rằng toán tử `*` khi gặp chuỗi chữ số `"3"` sẽ tự động ép kiểu thành số nguyên `3` để tính phép nhân `3 * 3 = 9`, tạo ra chuỗi `"PyPy9"`.</t>
+          <t>Python không định nghĩa tên hàm chuyển đổi kiểu dữ liệu là `integer`, sử dụng tên này sẽ làm phát sinh lỗi `NameError` do tên hàm không tồn tại.</t>
         </is>
       </c>
       <c r="K12" s="2" t="n">
@@ -1316,58 +1238,51 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Cho đoạn mã Python thực hiện biểu thức số học như sau:
-```python
-base_value = 2
-exponent = 3
-result_val = -base_value ** exponent + 10
-print(result_val)
-```
-Giá trị của biến `result_val` được in ra màn hình console là bao nhiêu?</t>
+          <t>Khi thực hiện gán lại giá trị cho một biến trong Python với các kiểu dữ liệu khác nhau trong cùng một chương trình (ví dụ: gán `data = 100` sau đó gán `data = "Rikkei"`), hành vi nào sau đây mô tả đúng nhất cơ chế xử lý kiểu dữ liệu của Python?</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>`-18`</t>
+          <t>Python tự động thay đổi kiểu dữ liệu của biến `data` từ `int` sang `str` theo giá trị mới nhờ cơ chế kiểu dữ liệu động (dynamic typing).</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>Sai do nhầm lẫn dấu phép toán: Học viên tính đúng `-2 ** 3 = -8` nhưng lại thực hiện nhầm phép cộng với `10` thành phép trừ `-8 - 10`, dẫn đến kết quả `-18`.</t>
+          <t>Python là ngôn ngữ có cơ chế kiểu dữ liệu động (dynamic typing), cho phép một biến liên kết với các giá trị thuộc những kiểu dữ liệu khác nhau tại các thời điểm thực thi khác nhau.</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>`18`</t>
+          <t>Python phát sinh lỗi `TypeError` vì biến sau khi khởi tạo với kiểu `int` thì không thể tiếp nhận giá trị mới mang kiểu `str`.</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>Sai do bẫy độ ưu tiên toán tử: Học viên lầm tưởng toán tử âm một ngôi `-` thực hiện trước toán tử lũy thừa `**`, dẫn đến phép tính `(-2) ** 3` và nhầm dấu thành số dương `8`, sau đó lấy `8 + 10 = 18`.</t>
+          <t>Quy tắc bắt buộc cố định kiểu dữ liệu chỉ xuất hiện ở các ngôn ngữ kiểm tra kiểu tĩnh (static typing), không phải là hành vi mặc định của Python.</t>
         </is>
       </c>
       <c r="G13" s="3" t="inlineStr">
         <is>
-          <t>`4`</t>
+          <t>Python giữ nguyên kiểu `int` cho biến `data` và tự động chuyển đổi chuỗi `"Rikkei"` về giá trị số nguyên 0.</t>
         </is>
       </c>
       <c r="H13" s="3" t="inlineStr">
         <is>
-          <t>Sai do nhầm lẫn toán tử lũy thừa: Học viên nhầm toán tử lũy thừa `**` thành toán tử nhân thông thường `*`, thực hiện tính `-2 * 3 = -6`, sau đó lấy `-6 + 10 = 4`.</t>
+          <t>Python không tự động thực hiện ép kiểu chuỗi chữ cái không chứa số về số nguyên 0 khi thực hiện phép gán giá trị mới cho biến.</t>
         </is>
       </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>`2`</t>
+          <t>Python bắt buộc phải khai báo lại tên biến bằng từ khóa tạo biến mới trước khi gán giá trị thuộc kiểu dữ liệu khác.</t>
         </is>
       </c>
       <c r="J13" s="3" t="inlineStr">
         <is>
-          <t>Đúng vì theo độ ưu tiên toán tử trong Python (Operator Precedence), toán tử lũy thừa `**` có độ ưu tiên cao hơn toán tử âm một ngôi `-`. Do đó, biểu thức `-2 ** 3` sẽ được tính là `-(2 ** 3) = -8`. Tiếp tục thực hiện phép cộng `-8 + 10` cho kết quả chính xác là `2`.</t>
+          <t>Python không yêu cầu hay cung cấp từ khóa khai báo lại biến khi thay đổi kiểu giá trị gán, việc gán trực tiếp giá trị mới hoàn toàn hợp lệ.</t>
         </is>
       </c>
       <c r="K13" s="2" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="L13" s="2" t="n">
         <v>6</v>
@@ -1384,54 +1299,67 @@
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>Cho đoạn mã Python thực hiện các thao tác với toán tử số học cơ bản như sau:
-```python
-first_num = 17
-second_num = 5
-result = first_num // second_num + first_num % second_num * 2
-print(result)
-```
-Kết quả in ra màn hình console là bao nhiêu?</t>
+          <t>Trong Python 3.12, một lập trình viên thực hiện khai báo các biến lưu trữ thông tin của một sản phẩm phần mềm bao gồm: tên sản phẩm, phiên bản (dạng số thực), số lượng tồn kho và trạng thái có sẵn. Đoạn mã nào dưới đây tuân thủ đúng cú pháp và quy tắc đặt tên biến (identifier)?</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>```python
+1st_product_name = "Laptop"
+release-version = 2.5
+stock_quantity = 100
+is_available = True
+```</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>Đáp án sai. Lựa chọn này do tính sai kết quả của toán tử lấy số dư `%` (cho rằng `17 % 5 = 1` thay vì `2`), từ đó thực hiện phép tính `3 + 1 * 2 = 5`. Trong Python, `17 % 5` trả về số dư chính xác là `2` vì `17 = 5 * 3 + 2`.</t>
+          <t>Đoạn mã vi phạm quy tắc đặt tên biến: tên biến `1st_product_name` bắt đầu bằng chữ số và `release-version` chứa dấu gạch nối `-` (Python sẽ hiểu nhầm là phép trừ).</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>```python
+product_name = "Laptop"
+release_version = 2.5
+stock_quantity = 100
+is_available = true
+```</t>
         </is>
       </c>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t>Đáp án sai. Lựa chọn này xuất phát từ lỗi thực hiện tính toán từ trái sang phải mà bỏ qua độ ưu tiên toán tử: lấy `17 // 5` được `3`, cộng với `17 % 5` được `2` ra tổng là `5`, rồi mới nhân cho `2` (`5 * 2 = 10`). Trong Python, toán tử nhân `*` có độ ưu tiên cao hơn toán tử cộng `+` nên phép nhân phải được thực hiện trước.</t>
+          <t>Đoạn mã bị lỗi cú pháp do giá trị Boolean `true` viết thường. Trong Python 3.12, giá trị đúng sai bắt buộc phải viết hoa chữ cái đầu (`True` hoặc `False`).</t>
         </is>
       </c>
       <c r="G14" s="3" t="inlineStr">
         <is>
-          <t>7.4</t>
+          <t>```python
+product_name = "Laptop"
+release_version = 2.5
+stock quantity = 100
+is_available = True
+```</t>
         </is>
       </c>
       <c r="H14" s="3" t="inlineStr">
         <is>
-          <t>Đáp án sai. Lựa chọn này xuất phát từ sự nhầm lẫn giữa toán tử chia lấy phần nguyên `//` và toán tử chia số thực `/`. Nếu sử dụng `17 / 5`, kết quả trả về sẽ là kiểu số thực `3.4`, cộng với `4` sẽ ra `7.4`. Tuy nhiên, toán tử `//` (floor division) thực hiện làm tròn xuống số nguyên gần nhất nên `17 // 5` trả về số nguyên `3`.</t>
+          <t>Đoạn mã bị lỗi cú pháp do tên biến `stock quantity` chứa khoảng trắng phân cách giữa các từ, vi phạm quy tắc khai báo định danh trong Python.</t>
         </is>
       </c>
       <c r="I14" s="3" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>```python
+product_name = "Laptop"
+release_version = 2.5
+stock_quantity = 100
+is_available = True
+```</t>
         </is>
       </c>
       <c r="J14" s="3" t="inlineStr">
         <is>
-          <t>Đáp án đúng. Theo thứ tự ưu tiên của toán tử trong Python, các toán tử chia lấy phần nguyên `//`, chia lấy số dư `%` và toán tử nhân `*` có cùng độ ưu tiên và cao hơn toán tử cộng `+`. Khi các toán tử cùng độ ưu tiên đứng cạnh nhau, Python thực thi từ trái sang phải: đầu tiên `17 // 5` trả về `3` (phần nguyên), tiếp theo `17 % 5` trả về `2` (phần dư). Sau đó thực hiện phép nhân `2 * 2 = 4`. Cuối cùng thực hiện phép cộng `3 + 4 = 7`.</t>
+          <t>Đoạn mã khai báo đúng cú pháp Python 3.12. Tên các biến tuân thủ quy tắc đặt tên định danh (chỉ gồm chữ cái, chữ số và dấu gạch dưới `_`, không bắt đầu bằng chữ số, không chứa khoảng trắng hay dấu gạch nối). Giá trị kiểu Boolean `True` được viết hoa chữ cái đầu đúng quy định.</t>
         </is>
       </c>
       <c r="K14" s="2" t="n">
@@ -1452,59 +1380,57 @@
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>Xem xét đoạn mã Python xử lý dữ liệu nhập từ người dùng và thực hiện toán tử trên chuỗi dưới đây:
+          <t>Một ứng dụng Python 3.12 thực hiện nhận dữ liệu đầu vào từ người dùng qua console và ép kiểu như sau:
 ```python
-raw_count = "3"
-unit_symbol = "A"
-total_items = int(raw_count) + 2
-display_pattern = unit_symbol * total_items
-print(display_pattern)
+raw_data = input()
+converted_data = int(raw_data)
+print(type(converted_data))
 ```
-Kết quả xuất ra màn hình console là gì?</t>
+Nếu người dùng nhập vào chuỗi chữ số `"25"`, kết quả hiển thị trên màn hình console là gì?</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>A5</t>
+          <t>Kiểu dữ liệu `&lt;class 'float'&gt;` vì dữ liệu số nhập từ bàn phím tự động ép kiểu thành số thực.</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>Đáp án sai. Lựa chọn này do nhầm lẫn toán tử nhân chuỗi `*` thành toán tử nối chuỗi `+` và suy luận sai rằng Python tự động ép kiểu số `5` thành chuỗi `"5"` để nối đằng sau chữ `"A"`. Toán tử `*` trong ngữ cảnh này là toán tử lặp chuỗi chứ không nối ký tự.</t>
+          <t>Đáp án này sai vì Python không tự động ép kiểu sang `float` khi dùng hàm `int()`. Muốn thu được kiểu số thực phải dùng hàm `float()`.</t>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>AAAAA</t>
+          <t>Kiểu dữ liệu `&lt;class 'bool'&gt;` vì giá trị chuỗi không rỗng tự động biến đổi thành kiểu đúng sai.</t>
         </is>
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>Đáp án đúng. Biến `raw_count` chứa chuỗi `"3"` được chuyển đổi thành số nguyên `3` bằng hàm `int(raw_count)`. Sau đó thực hiện phép cộng số học `3 + 2 = 5`, gán cho `total_items`. Khi sử dụng toán tử nhân `*` giữa một chuỗi (`"A"`) và một số nguyên (`5`), Python sẽ thực hiện lặp lại chuỗi đó `5` lần, tạo ra chuỗi kết quả `"AAAAA"`.</t>
+          <t>Đáp án này sai vì hàm `int()` thực hiện chuyển đổi chuỗi chữ số thành số nguyên chứ không chuyển thành kiểu dữ liệu đúng sai (`bool`).</t>
         </is>
       </c>
       <c r="G15" s="3" t="inlineStr">
         <is>
-          <t>Báo lỗi TypeError vì không thể nhân chuỗi với số nguyên</t>
+          <t>Kiểu dữ liệu `&lt;class 'str'&gt;` vì hàm `input()` luôn giữ nguyên kiểu dữ liệu chuỗi ban đầu chưa qua ép kiểu.</t>
         </is>
       </c>
       <c r="H15" s="3" t="inlineStr">
         <is>
-          <t>Đáp án sai. Lựa chọn này xuất phát từ việc hiểu sai quy tắc toán tử chuỗi trong Python. Python cho phép sử dụng toán tử nhân `*` giữa một `str` và một `int` để lặp lại chuỗi. Lỗi `TypeError` chỉ xuất hiện khi cố gắng nhân hai chuỗi với nhau hoặc nhân chuỗi với số thực `float`.</t>
+          <t>Đáp án này sai vì biến `raw_data` đã được ép kiểu thành công thông qua hàm `int(raw_data)` trước khi truyền vào hàm `print(type(...))`.</t>
         </is>
       </c>
       <c r="I15" s="3" t="inlineStr">
         <is>
-          <t>AAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAA</t>
+          <t>Kiểu dữ liệu `&lt;class 'int'&gt;` vì hàm `int()` đã chuyển đổi thành công chuỗi chữ số thành số nguyên.</t>
         </is>
       </c>
       <c r="J15" s="3" t="inlineStr">
         <is>
-          <t>Đáp án sai. Lựa chọn này xảy ra khi học viên mắc lỗi tư duy nhầm lẫn rằng `raw_count` không được chuyển kiểu dữ liệu và thực hiện phép cộng chuỗi `"3" + "2" = "32"`, dẫn đến phép lặp chuỗi `"A" * 32` tạo ra 32 chữ `A`. Thực tế hàm `int(raw_count)` đã ép kiểu về số nguyên `3` trước khi thực hiện phép cộng số học.</t>
+          <t>Hàm `input()` mặc định nhận dữ liệu đầu vào ở kiểu chuỗi (`str`). Khi gọi `int("25")`, chuỗi `"25"` được chuyển đổi thành số nguyên `25`. Do đó, kết quả kiểm tra bằng hàm `type()` sẽ trả về kết quả `&lt;class 'int'&gt;`.</t>
         </is>
       </c>
       <c r="K15" s="2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L15" s="2" t="n">
         <v>6</v>
@@ -1521,59 +1447,51 @@
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>Đoạn mã Python dưới đây sử dụng toán tử lũy thừa và toán tử gán kết hợp để tính toán giá trị:
-```python
-base_value = 2
-power_factor = 3
-calculated_result = base_value ** power_factor ** 2
-calculated_result -= 10
-print(calculated_result)
-```
-Giá trị của `calculated_result` được in ra màn hình là bao nhiêu?</t>
+          <t>Cho biến `user_input = "18.5"` nhận giá trị dữ liệu nhập vào từ console dưới dạng chuỗi có chứa dấu chấm thập phân. Đoạn mã nào dưới đây thực hiện ép kiểu thành công giá trị này sang số nguyên trong Python 3.12 mà không gây ra lỗi?</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>54</t>
+          <t>Dùng `age = integer(user_input)` để dùng hàm `integer()` mặc định nhằm làm tròn chuỗi về dạng số nguyên.</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>Đáp án sai. Lựa chọn này do mắc bẫy tư duy khi giả định toán tử lũy thừa `**` thực thi từ trái sang phải như các toán tử số học thông thường. Nếu tính từ trái sang phải: `(2 ** 3) ** 2 = 8 ** 2 = 64`, sau đó trừ `10` ra `54`. Đây là lỗi sai phổ biến do không nắm rõ quy tắc kết hợp từ phải sang trái của toán tử `**`.</t>
+          <t>Đáp án này sai vì ngôn ngữ Python 3.12 không có hàm built-in nào tên là `integer()`. Gọi hàm không tồn tại sẽ phát sinh lỗi `NameError`.</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>512</t>
+          <t>Dùng `age = int(float(user_input))` để chuyển chuỗi thành số thực trước rồi mới ép thành số nguyên.</t>
         </is>
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>Đáp án sai. Lựa chọn này xảy ra khi tính chính xác giá trị của biểu thức lũy thừa `2 ** (3 ** 2) = 512`, nhưng bỏ sót câu lệnh tiếp theo chứa toán tử gán kết hợp `calculated_result -= 10` nên chưa trừ đi 10.</t>
+          <t>Trong Python 3.12, hàm `int()` không thể trực tiếp xử lý chuỗi ký tự chứa dấu chấm thập phân như `"18.5"`. Cần ép kiểu chuỗi về dạng số thực bằng `float("18.5")` thu được `18.5`, sau đó mới ép sang `int(18.5)` để lấy phần nguyên là `18`.</t>
         </is>
       </c>
       <c r="G16" s="3" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>Dùng `age = str(int(user_input))` để ép kiểu trực tiếp chuỗi thập phân sang số nguyên rồi đổi thành chuỗi.</t>
         </is>
       </c>
       <c r="H16" s="3" t="inlineStr">
         <is>
-          <t>Đáp án sai. Lựa chọn này xuất phát từ việc nhầm lẫn toán tử lũy thừa `**` thành toán tử nhân `*`. Nếu tính `2 * 3 * 2 = 12`, sau đó thực hiện `12 -= 10` sẽ cho ra kết quả bằng `2`. Trong Python, `**` đại diện cho phép tính lũy thừa.</t>
+          <t>Đáp án này sai vì biểu thức bên trong `int(user_input)` sẽ phát sinh lỗi `ValueError` trước khi hàm `str()` ở bên ngoài kịp thực thi.</t>
         </is>
       </c>
       <c r="I16" s="3" t="inlineStr">
         <is>
-          <t>502</t>
+          <t>Dùng `age = int(user_input)` để trực tiếp chuyển đổi chuỗi chứa ký tự thập phân sang kiểu số nguyên.</t>
         </is>
       </c>
       <c r="J16" s="3" t="inlineStr">
         <is>
-          <t>Đáp án đúng. Toán tử lũy thừa `**` trong Python có tính kết hợp từ phải sang trái (right-to-left associativity). Do đó, biểu thức `2 ** 3 ** 2` được tính theo thứ tự `2 ** (3 ** 2) = 2 ** 9 = 512`. Tiếp theo, toán tử gán kết hợp `calculated_result -= 10` tương đương với `calculated_result = calculated_result - 10`, dẫn đến `512 - 10 = 502`.</t>
+          <t>Đáp án này sai vì việc truyền trực tiếp chuỗi ký tự chứa dấu chấm thập phân `"18.5"` vào hàm `int()` sẽ gây lỗi `ValueError` tại thời điểm chạy chương trình.</t>
         </is>
       </c>
       <c r="K16" s="2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L16" s="2" t="n">
         <v>6</v>
@@ -1590,54 +1508,47 @@
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>Cho đoạn mã Python 3.12 xử lý tính toán số lượng trang hiển thị như sau:
-```python
-total_products = 53
-items_per_page = 10
-total_pages = total_products // items_per_page + (total_products % items_per_page &gt; 0)
-print(total_pages)
-```
-Giá trị in ra màn hình console sau khi thực thi đoạn mã trên là bao nhiêu?</t>
+          <t>Trong ngôn ngữ Python 3.12, quy tắc đặt tên biến nào dưới đây là đúng cú pháp và không gây ra lỗi `SyntaxError` khi khai báo biến?</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>`TypeError: unsupported operand type(s) for +: 'int' and 'bool'`</t>
+          <t>Tên biến có thể bắt đầu bằng chữ số từ 0 đến 9 nhưng không được chứa các khoảng trắng giữa các từ.</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>Đáp án sai. Học viên lầm tưởng rằng Python sẽ phát sinh lỗi `TypeError` khi cộng trực tiếp số nguyên `int` với giá trị `bool`. Tuy nhiên, trong Python, `bool` là lớp con của `int` nên phép cộng `5 + True` hoàn toàn hợp lệ.</t>
+          <t>Tên biến bắt đầu bằng chữ số vi phạm cú pháp của Python và sẽ gây ra lỗi `SyntaxError` ngay khi trình thông dịch phân tích mã.</t>
         </is>
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>`5.3`</t>
+          <t>Tên biến bắt buộc phải viết hoa toàn bộ các chữ cái và không được sử dụng dấu gạch dưới (`_`).</t>
         </is>
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>Đáp án sai. Người học thường nhầm lẫn giữa toán tử chia lấy phần nguyên `//` và toán tử chia số thực `/`. Nếu dùng `total_products / items_per_page`, kết quả sẽ là `5.3`, nhưng toán tử `//` ép kết quả về số nguyên `5` trước khi thực hiện phép cộng phía sau.</t>
+          <t>Python không bắt buộc tên biến phải viết hoa toàn bộ; việc dùng dấu gạch dưới (`_`) là hoàn toàn hợp lệ và khuyến khích theo quy chuẩn `snake_case`.</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr">
         <is>
-          <t>`5`</t>
+          <t>Tên biến có thể chứa các ký tự toán học như `-` hoặc `+` miễn là từ đầu tiên bắt đầu bằng chữ thường.</t>
         </is>
       </c>
       <c r="H17" s="3" t="inlineStr">
         <is>
-          <t>Đáp án sai. Bẫy tư duy xảy ra khi học viên bỏ qua hoặc cho rằng biểu thức so sánh `(total_products % items_per_page &gt; 0)` trả về kiểu `bool` nên không thể tham gia vào phép cộng số học với số nguyên, dẫn đến việc chỉ lấy kết quả của `53 // 10 = 5`.</t>
+          <t>Các ký tự toán học như `-` hay `+` là các toán tử trong Python nên không thể dùng trong tên biến vì làm trình thông dịch hiểu nhầm thành phép toán.</t>
         </is>
       </c>
       <c r="I17" s="3" t="inlineStr">
         <is>
-          <t>`6`</t>
+          <t>Tên biến chỉ bao gồm chữ cái, chữ số, dấu gạch dưới (`_`) và không được bắt đầu bằng chữ số.</t>
         </is>
       </c>
       <c r="J17" s="3" t="inlineStr">
         <is>
-          <t>Đáp án đúng. Phép toán `total_products // items_per_page` sử dụng toán tử chia lấy phần nguyên `//` cho kết quả `53 // 10 = 5`. Phép so sánh `total_products % items_per_page &gt; 0` cho kết quả `3 &gt; 0` là `True`. Trong Python, kiểu `bool` kế thừa từ `int` (với `True` tương đương `1` và `False` tương đương `0`). Khi thực hiện phép cộng `5 + True`, Python tự động coi `True` là `1`, dẫn đến kết quả `5 + 1 = 6`.</t>
+          <t>Trong Python, tên biến hợp lệ phải bắt đầu bằng một chữ cái hoặc dấu gạch dưới (`_`), không được bắt đầu bằng chữ số và không chứa các ký tự đặc biệt ngoài `_`.</t>
         </is>
       </c>
       <c r="K17" s="2" t="n">
@@ -1658,55 +1569,52 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>Cho đoạn mã Python 3.12 thực hiện cập nhật chuỗi mã định danh như sau:
+          <t>Xét đoạn mã xử lý dữ liệu nhập vào từ người dùng trong Python 3.12 dưới đây:
 ```python
-unit_code = "A"
-repeat_count = 3
-multiplier = 2
-unit_code *= repeat_count + multiplier
-print(unit_code)
+data = input("Nhập đơn giá: ")
+result = data * 2
 ```
-Kết quả hiển thị trên màn hình console là gì?</t>
+Nếu người dùng nhập chuỗi `"500"` từ console, biến `result` nhận giá trị và kiểu dữ liệu nào?</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>`"AAAA"`</t>
+          <t>Chương trình dừng và báo lỗi `TypeError` ngay tại dòng lệnh `result = data * 2` vì không cho phép nhân chuỗi với số.</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>Đáp án sai. Học viên tính nhầm thứ tự ưu tiên hoặc tính sai phép cộng vế phải `3 + 2`, dẫn đến kết quả chuỗi chỉ gồm 4 ký tự `"AAAA"`.</t>
+          <t>Phép nhân giữa một chuỗi (`str`) và một số nguyên (`int`) là cú pháp hoàn toàn hợp lệ trong Python (toán tử lặp chuỗi), không gây lỗi `TypeError`.</t>
         </is>
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>`"AAA2"`</t>
+          <t>Giá trị `1000.0` với kiểu dữ liệu `float` do trình thông dịch mặc định tự ép kiểu dữ liệu nhập vào thành số thực.</t>
         </is>
       </c>
       <c r="F18" s="3" t="inlineStr">
         <is>
-          <t>Đáp án sai. Học viên suy luận sai rằng phép cộng `+ multiplier` sẽ tự động chuyển số `2` thành chuỗi và nối vào sau chuỗi đã nhân bản `"AAA"` để thành `"AAA2"`.</t>
+          <t>Python không tự động chuyển kiểu chuỗi thu được từ `input()` sang `float` nếu không gọi hàm ép kiểu `float()` một cách tường minh.</t>
         </is>
       </c>
       <c r="G18" s="3" t="inlineStr">
         <is>
-          <t>`"AAAAA"`</t>
+          <t>Giá trị `"500500"` với kiểu dữ liệu `str` do hàm `input()` luôn trả về chuỗi và toán tử `*` thực hiện lặp chuỗi.</t>
         </is>
       </c>
       <c r="H18" s="3" t="inlineStr">
         <is>
-          <t>Đáp án đúng. Trong Python, biểu thức vế phải của toán tử gán phức hợp (như `*=`) luôn được ưu tiên tính toán trước. Biểu thức `repeat_count + multiplier` được thực hiện trước cho kết quả `3 + 2 = 5`. Sau đó toán tử `unit_code *= 5` được thực thi, thực hiện nhân bản chuỗi `"A"` lên 5 lần, tạo ra kết quả `"AAAAA"`.</t>
+          <t>Hàm `input()` mặc định trả về kiểu chuỗi (`str`). Khi áp dụng toán tử `*` giữa chuỗi `"500"` và số nguyên `2`, Python thực hiện phép nhân bản chuỗi để tạo ra chuỗi `"500500"`.</t>
         </is>
       </c>
       <c r="I18" s="3" t="inlineStr">
         <is>
-          <t>`TypeError: can only concatenate str (not "int") to str`</t>
+          <t>Giá trị `1000` với kiểu dữ liệu `int` do Python tự động chuyển đổi chuỗi số sang số nguyên khi tính toán.</t>
         </is>
       </c>
       <c r="J18" s="3" t="inlineStr">
         <is>
-          <t>Đáp án sai. Học viên lầm tưởng toán tử `*=` có độ ưu tiên cao hơn phép cộng `+` nên chương trình sẽ thực hiện `unit_code = unit_code * repeat_count` trước (cho ra `"AAA"`), sau đó thực hiện `"AAA" + 2` (cộng chuỗi với số nguyên), dẫn đến suy đoán phát sinh lỗi `TypeError`. Thực tế vế phải `3 + 2` được tính toán xong trước rồi mới nhân chuỗi.</t>
+          <t>Python là ngôn ngữ ép kiểu động nhưng không tự động chuyển đổi kiểu dữ liệu chuỗi sang số nguyên khi dùng toán tử `*` với một số nguyên.</t>
         </is>
       </c>
       <c r="K18" s="2" t="n">
@@ -1727,57 +1635,47 @@
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>Cho đoạn mã Python 3.12 thực hiện các phép toán chia và so sánh như sau:
-```python
-number_a = 10
-number_b = 4
-result_1 = number_a / number_b
-result_2 = number_a // number_b
-is_equal = result_1 == result_2
-output_val = result_1 * is_equal + result_2
-print(output_val)
-```
-Kết quả hiển thị trên màn hình console là bao nhiêu?</t>
+          <t>Khi thu thập một giá trị số thực từ console dưới dạng chuỗi `val_str = "18.5"`, đoạn mã nào dưới đây chuyển đổi kiểu dữ liệu sang số thực (`float`) một cách tường minh và đúng cú pháp trong Python 3.12?</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>`TypeError: unsupported operand type(s) for *: 'float' and 'bool'`</t>
+          <t>`val_num = (float)val_str` - Sử dụng ép kiểu cú pháp đóng mở ngoặc đơn đứng trước tên biến.</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>Đáp án sai. Học viên nhầm lẫn rằng phép nhân giữa một số thực `float` (`2.5`) với một giá trị `bool` (`False`) sẽ gây ra lỗi `TypeError`. Trong Python, `bool` tham gia vào các phép tính số học bình thường với giá trị `1` (`True`) hoặc `0` (`False`).</t>
+          <t>Cú pháp ép kiểu `(float)variable` thuộc các ngôn ngữ như C/C++/Java và không hợp lệ trong Python 3.12, sẽ gây ra lỗi `SyntaxError`.</t>
         </is>
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>`4.5`</t>
+          <t>`val_num = parse_float(val_str)` - Sử dụng hàm toàn cục `parse_float()` có sẵn của ngôn ngữ.</t>
         </is>
       </c>
       <c r="F19" s="3" t="inlineStr">
         <is>
-          <t>Đáp án sai. Bẫy tư duy xảy ra khi học viên cho rằng `2.5` và `2` bằng nhau trong phép so sánh `==` dẫn tới `is_equal` nhận giá trị `True` (tương đương `1`). Khi đó phép tính trở thành `2.5 * 1 + 2 = 4.5`.</t>
+          <t>Python không cung cấp sẵn hàm toàn cục tên là `parse_float()`, việc gọi hàm không tồn tại trong môi trường mặc định sẽ phát sinh lỗi `NameError`.</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
         <is>
-          <t>`2.0`</t>
+          <t>`val_num = float(val_str)` - Gọi hàm built-in `float()` để chuyển đổi chuỗi hợp lệ thành số thực.</t>
         </is>
       </c>
       <c r="H19" s="3" t="inlineStr">
         <is>
-          <t>Đáp án đúng. Phép chia `/` luôn trả về số thực `float` (`10 / 4 = 2.5`), trong khi chia lấy phần nguyên `//` trả về số nguyên `int` (`10 // 4 = 2`). Phép so sánh `2.5 == 2` cho kết quả `False`. Trong phép tính số học, `False` tương đương giá trị `0`. Do đó `2.5 * False` trở thành `2.5 * 0 = 0.0` (kiểu `float`). Cuối cùng phép cộng `0.0 + 2` giữa số thực và số nguyên trả về số thực `2.0`.</t>
+          <t>Trong Python, hàm khởi tạo kiểu `float()` được sử dụng trực tiếp để ép kiểu dữ liệu từ chuỗi chứa định dạng số hợp lệ sang số thực.</t>
         </is>
       </c>
       <c r="I19" s="3" t="inlineStr">
         <is>
-          <t>`2`</t>
+          <t>`val_num = val_str.to_float()` - Gọi phương thức chuyển đổi `to_float()` trực tiếp từ đối tượng chuỗi.</t>
         </is>
       </c>
       <c r="J19" s="3" t="inlineStr">
         <is>
-          <t>Đáp án sai. Học viên không chú ý đến kiểu dữ liệu số thực `float` xuất hiện từ phép nhân `2.5 * 0 = 0.0`. Khi thực hiện phép cộng giữa `0.0` (float) và `2` (int), Python tự động chuyển kết quả về kiểu `float` là `2.0` chứ không phải số nguyên `2`.</t>
+          <t>Đối tượng kiểu chuỗi (`str`) trong Python không có phương thức nội tại tên là `to_float()`, câu lệnh này sẽ phát sinh lỗi `AttributeError`.</t>
         </is>
       </c>
       <c r="K19" s="2" t="n">
@@ -1798,58 +1696,57 @@
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>Trong một hệ thống tính toán chỉ số hiệu năng, lập trình viên gặp lỗi sai số logic khi thực thi đoạn mã Python 3 xử lý toán tử số học với số âm như sau:
+          <t>Cho đoạn mã Python thực thi thao tác xử lý dữ liệu nhập từ console như sau:
 ```python
-val_x = -5
-val_y = 2
-result = -val_x ** 2 // val_y
-print(result)
+data = input("Nhập số lượng: ")
+result = data * 2
+print(result, type(result))
 ```
-Hãy phân tích thứ tự ưu tiên của toán tử và xác định kết quả được in ra console của biến `result`:</t>
+Khi người dùng nhập vào ký tự `3` từ màn hình console, kết quả hiển thị ra màn hình và kiểu dữ liệu của biến `result` là gì?</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>`result` có giá trị `12`</t>
+          <t>Màn hình hiển thị `33 &lt;class 'str'&gt;` vì hàm `input()` luôn trả về kiểu chuỗi nên phép `*` đóng vai trò nhân bản chuỗi.</t>
         </is>
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>Đáp án sai. Người học mắc sai lầm khi cho rằng toán tử đổi dấu `-` ở đầu biểu thức `-val_x` sẽ biến `val_x = -5` thành `5`, sau đó `5 ** 2 = 25` và `25 // 2 = 12`. Đây là tư duy sai vì toán tử lũy thừa `**` liên kết chặt hơn toán tử đổi dấu `-` đứng trước biến.</t>
+          <t>Hàm `input()` trong Python luôn nhận dữ liệu đầu vào dưới dạng chuỗi ký tự (`str`). Khi áp dụng toán tử `*` giữa một chuỗi ký tự và một số nguyên `2`, Python thực thi hành vi nhân bản chuỗi (string repetition) tạo thành chuỗi `'33'`. Do đó `type(result)` trả về `&lt;class 'str'&gt;`.</t>
         </is>
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>`result` có giá trị `13`</t>
+          <t>Màn hình hiển thị `6 &lt;class 'int'&gt;` vì Python tự động nhận diện giá trị nhập vào là chữ số và ép kiểu sang số nguyên.</t>
         </is>
       </c>
       <c r="F20" s="3" t="inlineStr">
         <is>
-          <t>Đáp án sai. Đây là kết quả xuất phát từ hai sai lầm kết hợp: nhầm lẫn toán tử đổi dấu `-val_x` thành dương `5` và đồng thời làm tròn lên kết quả `12.5` thành `13`. Trong thực tế cú pháp Python không hoạt động theo cơ chế này.</t>
+          <t>Python là ngôn ngữ định kiểu động nhưng không tự động chuyển đổi kiểu dữ liệu chuỗi từ `input()` sang số nguyên khi chưa qua các hàm ép kiểu rõ ràng như `int()`.</t>
         </is>
       </c>
       <c r="G20" s="3" t="inlineStr">
         <is>
-          <t>`result` có giá trị `-12`</t>
+          <t>Màn hình hiển thị `32 &lt;class 'str'&gt;` vì toán tử `*` với chuỗi ký tự hoạt động tương tự như phép nối chuỗi với ký tự `2`.</t>
         </is>
       </c>
       <c r="H20" s="3" t="inlineStr">
         <is>
-          <t>Đáp án sai. Học viên phân tích đúng thứ tự ưu tiên để ra `-25`, nhưng nhầm lẫn cơ chế chia phần nguyên `//` của Python với phép chia cắt bỏ phần thập phân (truncate toward zero) trong C/C++ hoặc Java. Phép chia `-25 / 2 = -12.5` khi làm tròn xuống (floor) trong Python phải thu được `-13`, không phải `-12`.</t>
+          <t>Toán tử `*` thực hiện lặp lại chuỗi `data` theo số lần là `2` (tạo thành `'3'` + `'3'` = `'33'`), chứ không ghép ký tự `'2'` vào cuối chuỗi `data`.</t>
         </is>
       </c>
       <c r="I20" s="3" t="inlineStr">
         <is>
-          <t>`result` có giá trị `-13`</t>
+          <t>Chương trình phát sinh lỗi `TypeError` vì Python không cho phép thực hiện phép toán nhân giữa kiểu chuỗi và kiểu số nguyên.</t>
         </is>
       </c>
       <c r="J20" s="3" t="inlineStr">
         <is>
-          <t>Đáp án đúng. Trong Python, toán tử lũy thừa `**` có độ ưu tiên cao hơn toán tử đổi dấu (phủ định số học `-`). Do đó, `val_x ** 2` được thực hiện trước: `(-5) ** 2 = 25`. Tiếp theo toán tử đổi dấu đổi `25` thành `-25`. Cuối cùng, toán tử chia lấy phần nguyên `//` thực hiện phép tính `-25 // 2`. Khác với một số ngôn ngữ làm tròn về `0`, toán tử `//` trong Python luôn làm tròn xuống (floor) về phía âm vô cùng, khiến `-12.5` bị làm tròn xuống `-13`.</t>
+          <t>Trong Python, phép nhân giữa một chuỗi (`str`) và một số nguyên (`int`) là hợp lệ và được dùng để lặp lại chuỗi đó theo số lần tương ứng chứ không gây lỗi kiểu dữ liệu.</t>
         </is>
       </c>
       <c r="K20" s="2" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="L20" s="2" t="n">
         <v>10</v>
@@ -1866,61 +1763,53 @@
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>Một mô đun tính toán mã kiểm tra dữ liệu gặp sự cố tính sai giá trị đầu ra. Đoạn mã nguồn Python 3 được thu hẹp về các toán tử cốt lõi như sau:
+          <t>Xét đoạn mã Python thực hiện khởi tạo và gán giá trị cho các biến như sau:
 ```python
-val_a = 23
-val_b = 5
-val_c = 2
-output_val = val_a % val_b * val_c ** 3 // 4
-print(output_val)
+User_Age = 25
+user_age = "25"
+print(User_Age, type(user_age))
 ```
-Hãy phân tích thứ tự kết hợp và độ ưu tiên toán tử để xác định giá trị đúng của biến `output_val` khi in ra console:</t>
+Kết quả xuất ra màn hình console của đoạn mã trên là gì?</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>`output_val` có giá trị `0`</t>
+          <t>Chương trình phát sinh lỗi `NameError` do cú pháp khai báo hai biến có cùng tên gọi chỉ khác biệt về chữ hoa và chữ thường.</t>
         </is>
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>Đáp án sai. Đây là sai lầm khi học viên cho rằng toán tử chia phần nguyên `//` được thực thi trước phép nhân, khiến `8 // 4 = 2`, sau đó tính `5 * 2 = 10` rồi `23 % 10` hoặc tính sai thứ tự nhóm phép chia tạo ra kết quả `0`.</t>
+          <t>Khai báo các biến chỉ khác nhau về ký tự viết hoa/viết thường là hợp lệ trong Python, không vi phạm quy tắc đặt tên biến và không gây lỗi `NameError`.</t>
         </is>
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>`output_val` có giá trị `6`</t>
+          <t>Màn hình hiển thị `25 &lt;class 'str'&gt;` do Python phân biệt chữ hoa chữ thường nên đây là hai biến hoàn toàn riêng biệt.</t>
         </is>
       </c>
       <c r="F21" s="3" t="inlineStr">
         <is>
-          <t>Đáp án đúng. Thứ tự thực thi toán tử trong biểu thức được Python xử lý như sau:
-1. Toán tử lũy thừa `**` có độ ưu tiên cao nhất: `val_c ** 3` -&gt; `2 ** 3 = 8`. Biểu thức trở thành `23 % 5 * 8 // 4`.
-2. Các toán tử `%`, `*`, và `//` có cùng cấp độ ưu tiên và được thực thi lần lượt từ trái sang phải:
-   - `23 % 5 = 3` (lấy số dư)
-   - `3 * 8 = 24` (phép nhân)
-   - `24 // 4 = 6` (chia lấy phần nguyên).
-Do đó `output_val` nhận giá trị chuẩn xác là `6`.</t>
+          <t>Python có tính chất phân biệt chữ hoa chữ thường (case-sensitive). Biến `User_Age` và `user_age` được lưu trữ ở hai vùng nhớ khác nhau. Giá trị của `User_Age` là `25` (kiểu `int`), còn `type(user_age)` truy xuất kiểu dữ liệu của `user_age` mang giá trị `"25"` nên trả về `&lt;class 'str'&gt;`.</t>
         </is>
       </c>
       <c r="G21" s="3" t="inlineStr">
         <is>
-          <t>`output_val` có giá trị `24`</t>
+          <t>Màn hình hiển thị `"25" &lt;class 'str'&gt;` do biến `User_Age` bị tự động ép kiểu và đồng bộ dữ liệu theo biến `user_age`.</t>
         </is>
       </c>
       <c r="H21" s="3" t="inlineStr">
         <is>
-          <t>Đáp án sai. Kết quả này xảy ra khi học viên bỏ sót bước thực hiện toán tử chia lấy phần nguyên `// 4` ở cuối biểu thức, dừng lại sau bước tính phép nhân `3 * 8 = 24`.</t>
+          <t>Python không tự động đồng bộ hay ép kiểu dữ liệu giữa các biến có tên gọi tương tự nhau. `User_Age` vẫn giữ nguyên giá trị số nguyên `25` ban đầu.</t>
         </is>
       </c>
       <c r="I21" s="3" t="inlineStr">
         <is>
-          <t>`output_val` có giá trị `3`</t>
+          <t>Màn hình hiển thị `25 &lt;class 'int'&gt;` do biến `user_age` viết sau đã đè lên giá trị và kiểu dữ liệu của biến `User_Age` trước đó.</t>
         </is>
       </c>
       <c r="J21" s="3" t="inlineStr">
         <is>
-          <t>Đáp án sai. Học viên mắc bẫy khi lầm tưởng toán tử nhân `*` và chia nguyên `//` có độ ưu tiên cao hơn toán tử chia lấy dư `%`. Khi đó học viên tính `5 * 8 // 4 = 10`, sau đó lấy `23 % 10 = 3`. Thực tế trong Python, `%`, `*` và `//` cùng cấp độ ưu tiên nên phải tính từ trái sang phải.</t>
+          <t>Biến `user_age` không ghi đè lên `User_Age` vì Python phân biệt chữ hoa chữ thường. Việc khai báo `user_age` tạo ra một biến mới độc lập chứ không thay đổi giá trị của `User_Age`.</t>
         </is>
       </c>
       <c r="K21" s="2" t="n">
@@ -1941,64 +1830,57 @@
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>Trong chương trình xử lý chuỗi và số nguyên cơ bản, lập trình viên viết đoạn mã để sinh chuỗi ký tự lặp lại như sau:
+          <t>Xét đoạn mã xử lý ép kiểu dữ liệu cơ sở và xuất kết quả ra màn hình console như sau:
 ```python
-raw_input_1 = "10"
-raw_input_2 = "2"
-val_num = int(raw_input_1)
-calc_res = val_num / int(raw_input_2) + val_num % int(raw_input_2)
-output_data = str(calc_res) * int(raw_input_2)
-print(output_data)
+val_a = float(10)
+val_b = int(3.9)
+print(val_a, val_b, sep=" | ")
 ```
-Hãy phân tích kiểu dữ liệu tạo ra từ các toán tử và xác định kết quả in ra màn hình console của biến `output_data`:</t>
+Kết quả hiển thị chính xác trên màn hình console là gì?</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>`output_data` có giá trị `"55"`</t>
+          <t>Màn hình hiển thị `10.0 | 4` do hàm `int(3.9)` thực hiện quy tắc làm tròn số thực lên giá trị số nguyên lớn hơn.</t>
         </is>
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>Đáp án sai. Học viên mắc sai lầm phổ biến khi nghĩ rằng toán tử chia `/` đối với hai số nguyên chia hết (`10 / 2`) sẽ trả về số nguyên `5` (như trong C/Java hoặc Python 2). Nếu `calc_res = 5`, `str(5) * 2` sẽ ra `"55"`. Tuy nhiên trong Python 3, `/` luôn trả về `float`.</t>
+          <t>Hàm `int()` không làm tròn số (rounding) mà chỉ đơn thuần cắt bỏ phần thập phân. Do đó `int(3.9)` cho ra kết quả `3` chứ không phải `4`.</t>
         </is>
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>`output_data` có giá trị `"5.05.0"`</t>
+          <t>Màn hình hiển thị `10 | 4` do hàm `float()` tự động rút gọn dấu thập phân và hàm `int()` làm tròn tiến lên số nguyên gần nhất.</t>
         </is>
       </c>
       <c r="F22" s="3" t="inlineStr">
         <is>
-          <t>Đáp án đúng. Phân tích tiến trình thực thi:
-1. Phép chia `/` trong Python 3 luôn trả về kiểu `float` (kể cả chia hết): `10 / 2 = 5.0`.
-2. Phép chia lấy dư `10 % 2 = 0`. Tổng `calc_res = 5.0 + 0 = 5.0` (kiểu `float`).
-3. `str(calc_res)` chuyển số thực `5.0` thành chuỗi `"5.0"`.
-4. Toán tử nhân chuỗi với số nguyên `"5.0" * 2` thực hiện lặp lại chuỗi 2 lần, tạo ra kết quả `"5.05.0"`.</t>
+          <t>Hàm `float(10)` biểu diễn giá trị dưới dạng số thực `10.0` chứ không mất phần thập phân `.0`. Hàm `int()` trích xuất phần nguyên chứ không thực hiện quy tắc làm tròn số.</t>
         </is>
       </c>
       <c r="G22" s="3" t="inlineStr">
         <is>
-          <t>`output_data` có giá trị `"10.0"`</t>
+          <t>Màn hình hiển thị `10.0 | 3` do hàm `float()` chuyển số nguyên thành số thực và `int()` cắt bỏ hoàn toàn phần thập phân.</t>
         </is>
       </c>
       <c r="H22" s="3" t="inlineStr">
         <is>
-          <t>Đáp án sai. Sai lầm này xảy ra khi học viên nhầm lẫn toán tử nhân chuỗi `*` thành phép nhân số học giữa hai số `5.0 * 2 = 10.0`, thay vì nhận biết `str(calc_res)` đã ép kiểu thành chuỗi khiến toán tử `*` trở thành toán tử lặp chuỗi (string replication).</t>
+          <t>Hàm `float(10)` chuyển đổi số nguyên `10` thành số thực `10.0`. Hàm `int(3.9)` thực hiện chuyển đổi số thực thành số nguyên bằng cách lấy phần nguyên (cắt bỏ phần thập phân `.9`, không làm tròn). Tham số `sep=" | "` nối hai giá trị bằng chuỗi `" | "`, tạo ra kết quả `10.0 | 3`.</t>
         </is>
       </c>
       <c r="I22" s="3" t="inlineStr">
         <is>
-          <t>`output_data` có giá trị `"5.0"`</t>
+          <t>Màn hình hiển thị `10 | 3` do hàm `print()` tự động loại bỏ phần thập phân `.0` của các giá trị số thực khi xuất dữ liệu.</t>
         </is>
       </c>
       <c r="J22" s="3" t="inlineStr">
         <is>
-          <t>Đáp án sai. Học viên hiểu đúng kiểu `float` `5.0` nhưng quên không tính đến toán tử nhân chuỗi `* int(raw_input_2)` ở bước gán cho `output_data`, dẫn đến việc không lặp lại chuỗi.</t>
+          <t>Hàm `print()` giữ nguyên định dạng hiển thị của kiểu dữ liệu `float`. Giá trị `10.0` sẽ được in ra đầy đủ cả phần số thập phân chứ không bị lược bỏ thành `10`.</t>
         </is>
       </c>
       <c r="K22" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L22" s="2" t="n">
         <v>10</v>
@@ -2015,57 +1897,58 @@
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>Trong Python 3.12, một lập trình viên thực hiện đoạn mã xử lý toán tử số học và định dạng f-string như sau:
+          <t>Xét đoạn mã nguồn thực thi khởi tạo biến trong Python 3.12 bên dưới:
 ```python
-x = -3 ** 2 + 15 // 4 * 2
-y = (-3) ** 2 + 15 % 4 * 2
-result = f"{x = }, {y = }"
+x = 100
+x = "Python 3.12"
+type_x = type(x)
+print(type_x)
 ```
-Kết quả của biến `result` sau khi đoạn mã trên thực thi là gì và nguyên nhân do đâu toán tử `**` lại cho ra kết quả khác biệt giữa `x` và `y`?</t>
+Kết quả hiển thị trên màn hình console và đặc tính cơ bản nào của ngôn ngữ được phản ánh?</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>`result` có giá trị là `"x = 15, y = 15"`. Nguyên nhân do toán tử âm một ngôi `-` có độ ưu tiên cao hơn toán tử lũy thừa `**`, làm cho `-3 ** 2` được tính thành `(-3) ** 2 = 9`.</t>
+          <t>Chương trình in ra `&lt;class 'int'&gt;`, vì biến `x` đã được cố định kiểu dữ liệu ngay từ lần khởi tạo đầu tiên và không thể thay đổi giá trị thành chuỗi.</t>
         </is>
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>Phân tích sai lầm: Đáp án này phản ánh lỗi tư duy phổ biến khi lập trình viên nhầm tưởng dấu âm `-` dính liền vào số `3` sẽ tạo thành số âm nguyên khối trước khi thực hiện lũy thừa. Thực tế trong cú pháp của trình biên dịch Python, toán tử unary `-` có độ ưu tiên thấp hơn toán tử `**`, nên không thể tạo ra kết quả `9` cho `x`.</t>
+          <t>Khái niệm cố định kiểu dữ liệu từ lần khởi tạo đầu tiên thuộc về các ngôn ngữ tĩnh (static typing); Python cho phép thay đổi kiểu dữ liệu của biến một cách linh hoạt trong suốt quá trình thực thi.</t>
         </is>
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>`result` có giá trị là `"x = -3, y = 15"`. Nguyên nhân do toán tử lũy thừa `**` có độ ưu tiên cao hơn toán tử âm một ngôi `-`, làm cho `-3 ** 2` được tính thành `-(3 ** 2) = -9`.</t>
+          <t>Chương trình xuất hiện lỗi cú pháp (`SyntaxError`) vì Python là ngôn ngữ tĩnh (static typing), yêu cầu khai báo rõ kiểu dữ liệu trước khi gán.</t>
         </is>
       </c>
       <c r="F23" s="3" t="inlineStr">
         <is>
-          <t>Đáp án đúng. Trong bảng độ ưu tiên toán tử của Python, toán tử lũy thừa `**` có độ ưu tiên cao hơn toán tử dấu âm một ngôi (unary minus `-`). Do đó, biểu thức `-3 ** 2` được giải mã thành `-(3 ** 2) = -9`. Tiếp theo, toán tử chia lấy phần nguyên `//` và nhân `*` có cùng cấp độ ưu tiên nên tính từ trái sang phải: `15 // 4` cho `3`, rồi `3 * 2 = 6`. Do đó `x = -9 + 6 = -3`. Ở biến `y`, ngoặc đơn `(-3)` thay đổi thứ tự ưu tiên làm cho `(-3) ** 2 = 9`. Phép `%` và `*` tính từ trái sang phải: `15 % 4 = 3`, rồi `3 * 2 = 6`. Do đó `y = 9 + 6 = 15`. Đặc tả f-string debug `f"{x = }, {y = }"` xuất ra chuỗi `"x = -3, y = 15"`.</t>
+          <t>Python là ngôn ngữ được thiết kế với cơ chế kiểu dữ liệu động chứ không phải kiểu tĩnh, do đó việc gán lại giá trị khác kiểu dữ liệu hoàn toàn hợp lệ và không gây ra lỗi cú pháp.</t>
         </is>
       </c>
       <c r="G23" s="3" t="inlineStr">
         <is>
-          <t>`result` có giá trị là `"x = 3, y = 15"`. Nguyên nhân do phép tính `15 // 4 * 2` được thực hiện từ phải sang trái thành `15 // (4 * 2) = 1`.</t>
+          <t>Chương trình in ra `&lt;class 'str'&gt;`, thể hiện đặc tính cơ chế kiểu dữ liệu động (dynamic typing) cho phép biến `x` thay đổi kiểu dữ liệu linh hoạt từ số nguyên sang chuỗi ký tự.</t>
         </is>
       </c>
       <c r="H23" s="3" t="inlineStr">
         <is>
-          <t>Phân tích sai lầm: Đáp án này sai do áp dụng sai tính kết hợp (associativity). Các toán tử `//` và `*` kết hợp từ trái sang phải, nên `15 // 4 * 2` phải thực hiện `(15 // 4)` trước ra `3`, sau đó lấy `3 * 2` ra `6`. Nếu thực hiện từ phải sang trái sẽ ra `15 // 8 = 1` dẫn đến `x = -9 + 1 = -8` (hoặc `3` nếu tính nhầm toán tử âm), là cách tính sai quy chuẩn Python.</t>
+          <t>Trong Python 3.12, biến sở hữu đặc tính kiểu dữ liệu động (dynamic typing). Khi biến `x` được gán lại bằng chuỗi `"Python 3.12"`, kiểu dữ liệu của biến sẽ tự động chuyển thành chuỗi, do đó hàm `type(x)` trả về `&lt;class 'str'&gt;`.</t>
         </is>
       </c>
       <c r="I23" s="3" t="inlineStr">
         <is>
-          <t>`result` có giá trị là `"x = -3, y = 9"`. Nguyên nhân do toán tử chia lấy phần dư `%` và chia lấy phần nguyên `//` có độ ưu tiên cao hơn toán tử nhân `*`.</t>
+          <t>Chương trình in ra `&lt;class 'type'&gt;`, đại diện cho kiểu dữ liệu gốc của mọi đối tượng trong môi trường thực thi Python 3.12.</t>
         </is>
       </c>
       <c r="J23" s="3" t="inlineStr">
         <is>
-          <t>Phân tích sai lầm: Đáp án này mắc bẫy sai thứ tự ưu tiên giữa các toán tử nhân/chia. Trong Python, các toán tử số học `*`, `/`, `//`, `%` có độ ưu tiên ngang nhau và tuân theo tính kết hợp từ trái sang phải (left-to-right). Do đó `15 % 4 * 2` được tính là `(15 % 4) * 2 = 3 * 2 = 6`, chứ không phải `15 % (4 * 2) = 15 % 8 = 7` làm cho `y = 9 + 0` hay `9`.</t>
+          <t>Hàm `type(x)` trả về kiểu dữ liệu cụ thể của đối tượng mà biến `x` đang tham chiếu đến ở thời điểm hiện tại (`str`), chứ không trả về đối tượng lớp gốc `&lt;class 'type'&gt;`.</t>
         </is>
       </c>
       <c r="K23" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L23" s="2" t="n">
         <v>10</v>
@@ -2082,54 +1965,54 @@
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>Xem xét đoạn mã Python 3.12 thực hiện các phép chia lấy phần nguyên `//` và chia lấy phần dư `%` với số âm dưới đây:
+          <t>Trong quá trình thiết lập các biến lưu trữ thông tin hệ thống, người phát triển cần tuân thủ đúng quy tắc đặt tên định danh trong Python 3.12. Xét 4 khai báo biến dưới đây:
 ```python
-a = -13 // 4
-b = -13 % 4
-c = 13 % -4
-result = f"{a=}, {b=}, {c=}"
+(1) 2nd_user_score = 95
+(2) _user_score_2 = 95
+(3) user-score = 95
+(4) user score = 95
 ```
-Giá trị chính xác của chuỗi `result` thu được là gì và quy tắc hoạt động của phép toán `%` và `//` với số âm trong Python được định nghĩa như thế nào?</t>
+Phát biểu nào sau đây đánh giá chính xác về tính hợp lệ của các khai báo trên?</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>`result` có giá trị là `"a=-3, b=-1, c=1"`. Python cắt bỏ phần thập phân hướng về 0 khi thực hiện phép chia `//`, và toán tử `%` trả về kết quả mang cùng dấu với số bị chia (dividend).</t>
+          <t>Cả khai báo (2) và (4) đều hợp lệ, vì khoảng trắng giữa các ký tự sẽ tự động được trình biên dịch Python 3.12 bỏ qua khi gán giá trị.</t>
         </is>
       </c>
       <c r="D24" s="3" t="inlineStr">
         <is>
-          <t>Phân tích sai lầm: Đây là bẫy tư duy của lập trình viên chuyển sang từ các ngôn ngữ như C/C++ hoặc Java. Trong C/C++, phép chia số nguyên bị cắt bỏ phần thập phân về phía số `0` (`-13 / 4 = -3`), và toán tử `%` lấy dấu theo số bị chia. Tuy nhiên, Python thiết kế toán tử `//` theo cơ chế floor division và toán tử `%` lấy dấu theo số chia.</t>
+          <t>Tên biến không được phép chứa khoảng trắng; khai báo (4) (`user score = 95`) sẽ gây ra lỗi cú pháp (`SyntaxError`) ngay khi khởi chạy.</t>
         </is>
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>`result` có giá trị là `"a=-3, b=3, c=-3"`. Phép chia `//` làm tròn tới số nguyên gần 0 nhất, trong khi toán tử `%` tính phần dư theo giá trị tuyệt đối.</t>
+          <t>Cả khai báo (1) và (2) đều hợp lệ, vì Python cho phép dùng chữ số ở bất kỳ vị trí nào trong tên biến miễn là chứa ký tự gạch dưới.</t>
         </is>
       </c>
       <c r="F24" s="3" t="inlineStr">
         <is>
-          <t>Phân tích sai lầm: Đáp án này sai ở giá trị của `a = -3`. Học viên hiểu nhầm rằng `-3.25` được làm tròn tiến về `0` thành `-3`. Trong toán học máy tính của Python, làm tròn xuống (floor) của `-3.25` phải là `-4` vì `-4 &lt; -3.25`.</t>
+          <t>Khai báo (1) vi phạm quy tắc không được bắt đầu tên biến bằng chữ số (`2nd_user_score`), dẫn đến lỗi cú pháp (`SyntaxError`).</t>
         </is>
       </c>
       <c r="G24" s="3" t="inlineStr">
         <is>
-          <t>`result` có giá trị là `"a=-4, b=-1, c=1"`. Phép chia nguyên `//` làm tròn về âm vô cực, nhưng toán tử `%` trong Python ưu tiên trả về dấu của số bị chia (dividend).</t>
+          <t>Cả khai báo (2) và (3) đều hợp lệ, vì dấu gạch ngang (`-`) và dấu gạch dưới (`_`) có vai trò hoàn toàn tương đương trong quy tắc đặt tên.</t>
         </is>
       </c>
       <c r="H24" s="3" t="inlineStr">
         <is>
-          <t>Phân tích sai lầm: Đáp án này tính đúng `a = -4` nhưng lại sai quy tắc dấu của toán tử phần dư `%`. Toán tử `%` trong Python không lấy dấu từ số bị chia (dividend `-13` hay `13`), mà kết quả `x % y` luôn guaranteed nằm trong khoảng giữa `0` và `y` (tức là cùng dấu với số chia `y`).</t>
+          <t>Ký tự dấu gạch ngang (`-`) không được phép xuất hiện trong tên biến vì trình thông dịch Python sẽ xử lý đó là ký tự không hợp lệ trong tên định danh.</t>
         </is>
       </c>
       <c r="I24" s="3" t="inlineStr">
         <is>
-          <t>`result` có giá trị là `"a=-4, b=3, c=-3"`. Python quy định phép chia lấy phần nguyên `//` luôn làm tròn về phía âm vô cực (floor), và toán tử `%` trả về kết quả mang cùng dấu với số chia (divisor).</t>
+          <t>Chỉ có khai báo (2) là hợp lệ, vì tên biến có thể bắt đầu bằng dấu gạch dưới (`_`), trong khi (1) bắt đầu bằng chữ số, (3) chứa dấu gạch ngang và (4) chứa khoảng trắng.</t>
         </is>
       </c>
       <c r="J24" s="3" t="inlineStr">
         <is>
-          <t>Đáp án đúng. Phép chia `//` trong Python là floor division (làm tròn xuống số nguyên nhỏ hơn hoặc bằng). Ta có `-13 / 4 = -3.25`, làm tròn xuống âm vô cực thu được `a = -4`. Toán tử modulo `%` trong Python tuân theo công thức đại số `r = x - (y * (x // y))`. Với `b = -13 % 4`: `-13 - (4 * (-13 // 4)) = -13 - (4 * -4) = -13 + 16 = 3` (mang dấu dương của số chia `4`). Với `c = 13 % -4`: `13 - (-4 * (13 // -4)) = 13 - (-4 * -4) = 13 - 16 = -3` (mang dấu âm của số chia `-4`). F-string `=` xuất đúng `"a=-4, b=3, c=-3"`.</t>
+          <t>Theo quy tắc đặt tên định danh trong Python, tên biến chỉ bao gồm chữ cái, chữ số và dấu gạch dưới (`_`), không được bắt đầu bằng chữ số và không chứa khoảng trắng hay ký tự đặc biệt như dấu gạch ngang (`-`). Khai báo (2) tuân thủ đầy đủ các quy tắc này.</t>
         </is>
       </c>
       <c r="K24" s="2" t="n">
@@ -2150,55 +2033,54 @@
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>Một lập trình viên viết đoạn mã xử lý toán tử gán mở rộng và định dạng f-string debug trong Python 3.12 như sau:
+          <t>Cho đoạn mã nguồn Python 3.12 thực hiện hiển thị thông tin hệ thống ra màn hình console như sau:
 ```python
-item_code = "PY"
-count = 2 + 1
-item_code += str(count * 2)
-display_text = item_code * 2
-final_output = f"{display_text=}"
+title = "Python"
+version = 3.12
+is_active = True
+print(title, version, str(is_active), sep=" - ", end=" | END")
 ```
-Giá trị chính xác của biến `final_output` thu được là gì và cơ chế biểu diễn chuỗi ký tự của cú pháp f-string `=` trong Python 3.12 hoạt động như thế nào?</t>
+Kết quả hiển thị chính xác trên màn hình console khi chạy đoạn mã trên là gì?</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>`final_output` có giá trị là `"display_text='PY6PY6'"`. Cú pháp `=` trong f-string mặc định gọi hàm `repr()` trên giá trị của biểu thức, làm cho chuỗi ký tự được bao bọc bởi cặp dấu nháy đơn `'...'`.</t>
+          <t>Chương trình in ra `Python - 3.12 - True | END`, trong đó các đối số được phân tách bởi chuỗi `" - "` và kết thúc dòng bằng chuỗi `" | END"` thay vì xuống dòng mặc định.</t>
         </is>
       </c>
       <c r="D25" s="3" t="inlineStr">
         <is>
-          <t>Đáp án đúng. Từng bước thực thi: `count = 3`, `count * 2 = 6`, `str(6) = "6"`. Toán tử `+=` thực hiện nối chuỗi `item_code = "PY" + "6" = "PY6"`. Toán tử nhân chuỗi `*` lặp lại chuỗi `display_text = "PY6" * 2 = "PY6PY6"`. Cuối cùng, cú pháp f-string debug `f"{display_text=}"` trong Python mặc định chuyển đổi giá trị biểu thức bằng hàm `repr()` chứ không phải `str()`. Hàm `repr()` đối với một chuỗi sẽ trả về chuỗi đó nằm trong cặp dấu nháy đơn, tạo nên giá trị hoàn chỉnh `"display_text='PY6PY6'"`.</t>
+          <t>Trong hàm `print()` của Python, tham số `sep` quy định chuỗi phân tách giữa các giá trị xuất ra (mặc định là khoảng trắng), còn `end` quy định chuỗi kết thúc lệnh in (mặc định là `\n`). Do đó kết quả hiển thị chính xác là `Python - 3.12 - True | END`.</t>
         </is>
       </c>
       <c r="E25" s="3" t="inlineStr">
         <is>
-          <t>`final_output` có giá trị là `"display_text='PY12'"`. Do phép toán `count * 2` thực hiện nhân giá trị số với chuỗi `item_code` trước khi thực hiện phép gán.</t>
+          <t>Chương trình xuất hiện lỗi thực thi (`TypeError`) vì các biến thuộc nhiều kiểu dữ liệu khác nhau (`str`, `float`, `bool`) không thể in chung trong một hàm `print()`.</t>
         </is>
       </c>
       <c r="F25" s="3" t="inlineStr">
         <is>
-          <t>Phân tích sai lầm: Đáp án này sai ở tư duy thứ tự toán tử và kiểu dữ liệu. Phép toán `count * 2` được thực thi hoàn toàn giữa 2 số nguyên (`3 * 2 = 6`), sau đó mới được ép thành chuỗi `"6"` rồi nối vào `"PY"` tạo thành `"PY6"`. Không có cơ chế nào biến phép toán thành `2 * 6 = 12` hay nhân trực tiếp chuỗi trước khi ép kiểu.</t>
+          <t>Hàm `print()` trong Python hỗ trợ nhận nhiều đối số thuộc các kiểu dữ liệu cơ bản khác nhau và tự động chuyển đổi biểu diễn chuỗi để in ra mà không gây lỗi kiểu dữ liệu.</t>
         </is>
       </c>
       <c r="G25" s="3" t="inlineStr">
         <is>
-          <t>`final_output` có giá trị là `"display_text=PY6PY6"`. Cú pháp `=` trong f-string chỉ gọi hàm `str()` trên giá trị của biểu thức nên không xuất hiện dấu nháy đơn bao bọc.</t>
+          <t>Chương trình in ra `Python 3.12 True - | END`, vì tham số `sep` chỉ áp dụng phân tách giữa phần tử cuối cùng và tham số `end`.</t>
         </is>
       </c>
       <c r="H25" s="3" t="inlineStr">
         <is>
-          <t>Phân tích sai lầm: Học viên nhầm lẫn rằng f-string debug `=` chuyển đổi giá trị bằng hàm `str()`. Thực tế, để hỗ trợ mục đích debug trực quan và phân biệt kiểu dữ liệu (ví dụ chuỗi `"6"` khác với số `6`), Python tự động áp dụng `repr()` cho các biểu thức sau dấu `=`, do đó kết quả chuỗi bắt buộc phải có dấu nháy bao bọc.</t>
+          <t>Tham số `sep=" - "` sẽ chèn chuỗi `" - "` vào giữa mọi cặp đối số được truyền vào hàm `print()`, chứ không chỉ chèn vào vị trí phần tử cuối cùng.</t>
         </is>
       </c>
       <c r="I25" s="3" t="inlineStr">
         <is>
-          <t>Đoạn mã phát sinh lỗi `TypeError` tại dòng `item_code += str(count * 2)` do toán tử `+=` không hỗ trợ nối chuỗi với kết quả trả về từ hàm `str()`.</t>
+          <t>Chương trình in ra `Python - 3.12 - True\n | END`, vì tham số `end` luôn tự động nối tiếp sau ký tự xuống dòng mặc định của hàm `print()`.</t>
         </is>
       </c>
       <c r="J25" s="3" t="inlineStr">
         <is>
-          <t>Phân tích sai lầm: Đây là bẫy về kiểu dữ liệu. Toán tử `+=` trên kiểu chuỗi (`str`) thực chất gọi phương thức nối chuỗi. Hàm `str(count * 2)` trả về kiểu chuỗi hợp lệ (`"6"`), do đó hai chuỗi nối với nhau hoàn toàn hợp lệ và không gây ra `TypeError`.</t>
+          <t>Tham số `end` ghi đè hoàn toàn ký tự xuống dòng mặc định `\n`, do đó không xuất hiện ký tự `\n` trước chuỗi `" | END"`.</t>
         </is>
       </c>
       <c r="K25" s="2" t="n">
@@ -2219,52 +2101,47 @@
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>Trong phiên bản Python 3.12, đoạn mã nguồn xử lý các toán tử số học cơ bản dưới đây sẽ trả về kết quả hiển thị ra màn hình là gì?
-```python
-x = -3 ** 2 + 17 // -5
-y = 17 % -5
-print(f"{x}_{y}")
-```</t>
+          <t>Trong ngôn ngữ lập trình Python, một lập trình viên cần khởi tạo các biến lưu trữ thông tin hệ thống. Cú pháp khai báo biến nào dưới đây là hợp lệ theo quy tắc đặt tên định danh (identifier) và không gây ra lỗi cú pháp (```SyntaxError```)?</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>"5_-3"</t>
+          <t>Khai báo tên biến ```2024_user_count = 50``` đúng quy tắc do bắt đầu bằng số nguyên và chỉ chứa chữ cái, chữ số.</t>
         </is>
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>Đáp án sai. Lập trình viên đã xác định đúng cơ chế phép chia lấy dư `%` với số âm trong Python (`y = -3`) và phép chia nguyên (`17 // -5 = -4`), nhưng lại mắc lỗi kinh điển về độ ưu tiên toán tử khi cho rằng `-3 ** 2` tương đương `(-3) ** 2 = 9`, dẫn đến `x = 9 + (-4) = 5`.</t>
+          <t>Trong Python, tên biến không được phép bắt đầu bằng một chữ số. Việc khai báo ```2024_user_count = 50``` sẽ khiến trình thông dịch báo lỗi cú pháp ```SyntaxError: invalid decimal literal``` ngay khi khởi tạo chương trình.</t>
         </is>
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>"-13_-3"</t>
+          <t>Khai báo tên biến ```_user_count_2024 = 50``` đúng quy tắc do bắt đầu bằng ký tự gạch dưới và chỉ chứa chữ cái, chữ số.</t>
         </is>
       </c>
       <c r="F26" s="3" t="inlineStr">
         <is>
-          <t>Đáp án đúng. Trong Python, toán tử lũy thừa `**` có độ ưu tiên cao hơn toán tử đổi dấu âm `-_unary`. Do đó, `-3 ** 2` được tính là `-(3 ** 2) = -9`. Tiếp theo, phép chia lấy phần nguyên `17 // -5` làm tròn xuống về phía âm vô cực (floor), cho kết quả là `-4` (vì `-5 * -4 = 20`, còn `-5 * -3 = 15`). Tổng `x = -9 + (-4) = -13`. Đối với phép chia lấy phần dư `17 % -5`, công thức chuẩn của Python là `r = a - (b * (a // b))`, suy ra `17 - (-5 * -4) = 17 - 20 = -3`. Kết quả chuỗi f-string thu được là `"-13_-3"`.</t>
+          <t>Quy tắc đặt tên biến trong Python cho phép tên biến bắt đầu bằng một chữ cái hoặc dấu gạch dưới (```_```), theo sau là các chữ cái, chữ số hoặc dấu gạch dưới. Do đó, khai báo ```_user_count_2024 = 50``` hoàn toàn hợp lệ và chương trình thực thi thành công.</t>
         </is>
       </c>
       <c r="G26" s="3" t="inlineStr">
         <is>
-          <t>"-12_2"</t>
+          <t>Khai báo tên biến ```user-count-2024 = 50``` đúng quy tắc do sử dụng dấu gạch nối nối các thành phần tên biến.</t>
         </is>
       </c>
       <c r="H26" s="3" t="inlineStr">
         <is>
-          <t>Đáp án sai. Nguyên nhân do học viên tính đúng phần lũy thừa `-3 ** 2 = -9`, nhưng lại tính sai phép chia nguyên `17 // -5 = -3` (do cắt bỏ phần thập phân thay vì làm tròn xuống âm vô cực) dẫn tới `x = -9 + (-3) = -12`, đồng thời xác định sai phần dư `17 % -5 = 2` (do lấy dư theo dấu của số bị chia thay vì theo số chia như quy chuẩn Python).</t>
+          <t>Ký tự gạch nối (```-```) không thuộc tập ký tự hợp lệ khi đặt tên biến trong Python (chỉ bao gồm chữ cái, chữ số và dấu gạch dưới ```_```). Khai báo ```user-count-2024 = 50``` sẽ gây ra lỗi cú pháp ```SyntaxError: cannot assign to expression```.</t>
         </is>
       </c>
       <c r="I26" s="3" t="inlineStr">
         <is>
-          <t>"5_2"</t>
+          <t>Khai báo tên biến ```user count 2024 = 50``` đúng quy tắc do chứa khoảng trắng ngăn cách giữa các chữ cái.</t>
         </is>
       </c>
       <c r="J26" s="3" t="inlineStr">
         <is>
-          <t>Đáp án sai. Học viên mắc phải hai bẫy tư duy sai lầm: (1) Nhầm lẫn độ ưu tiên toán tử khi cho rằng `-3 ** 2` bằng `(-3) ** 2 = 9`; (2) Lập luận phép chia nguyên `17 // -5` làm tròn về 0 giống C/Java ra `-3` và phần dư `17 % -5` ra `2`. Từ đó tính sai `x = 9 + (-4) = 5` hoặc `9 + (-3) = 6` và `y = 2`.</t>
+          <t>Tên biến trong Python không được chứa khoảng trắng. Việc khai báo ```user count 2024 = 50``` khiến trình thông dịch không thể phân tích cấu trúc câu lệnh và phát sinh lỗi ```SyntaxError: invalid syntax```.</t>
         </is>
       </c>
       <c r="K26" s="2" t="n">
@@ -2285,59 +2162,57 @@
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>Phân tích đoạn mã Python 3.12 thực thi các toán tử gán kết hợp và toán tử trên chuỗi/số thực dưới đây. Cho biết giá trị biến `result` thu được là gì?
+          <t>Khi thực thi chương trình Python nhập xuất dữ liệu console, lập trình viên sử dụng đoạn mã sau:
 ```python
-text_data = "py"
-multiplier = 2
-text_data *= multiplier + 1
-numeric_val = 10.0
-numeric_val %= 4
-result = f"{text_data}_{numeric_val}"
-```</t>
+raw_val = input()
+converted_val = bool(raw_val)
+print(converted_val)
+```
+Khi người dùng nhập chuỗi ký tự ```0``` từ màn hình console và nhấn Enter, kết quả hiển thị ra màn hình và bản chất kiểu dữ liệu của biến ```converted_val``` là gì?</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>"pypypy_2.0"</t>
+          <t>Hiển thị giá trị ```0``` thuộc kiểu dữ liệu ```int``` do hàm ```bool()``` tự động ép kiểu dữ liệu về số nguyên.</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>Đáp án đúng. Trong biểu thức gán mở rộng `text_data *= multiplier + 1`, vế phải `multiplier + 1` (giá trị bằng `3`) được ưu tiên tính toán trước hoàn toàn, sau đó mới thực hiện toán tử lặp chuỗi `text_data = "py" * 3`, trả về `"pypypy"`. Với `numeric_val %= 4`, do `numeric_val` ban đầu có kiểu `float` (`10.0`), kết quả của phép chia lấy dư `%` với số nguyên `4` vẫn bảo toàn kiểu `float` là `2.0`. Do đó `result` có giá trị chuỗi là `"pypypy_2.0"`.</t>
+          <t>Hàm ```bool()``` thực hiện chuyển đổi dữ liệu sang kiểu boolean với giá trị ```True``` hoặc ```False```, không thực hiện chuyển đổi về kiểu số nguyên ```int```.</t>
         </is>
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
-          <t>"pypypy_2"</t>
+          <t>Hiển thị giá trị ```False``` thuộc kiểu dữ liệu ```bool``` do hàm ```input()``` tự động nhận diện ký tự ```0``` là số zero.</t>
         </is>
       </c>
       <c r="F27" s="3" t="inlineStr">
         <is>
-          <t>Đáp án sai. Học viên tính đúng phần nhân chuỗi `"pypypy"`, nhưng hiểu sai cơ chế ép kiểu tự động của toán tử số học trong Python khi cho rằng phép chia lấy dư `10.0 % 4` sẽ tự động chuyển kết quả về kiểu số nguyên `int` (`2`) thay vì giữ nguyên kiểu số thực `float` (`2.0`).</t>
+          <t>Giá trị ```False``` khi ép kiểu chuỗi sang boolean chỉ xảy ra với chuỗi rỗng ```""```. Chuỗi ```"0"``` là chuỗi ký tự chứa một ký tự nên hàm ```bool()``` trả về giá trị ```True```.</t>
         </is>
       </c>
       <c r="G27" s="3" t="inlineStr">
         <is>
-          <t>"pypy_2.0"</t>
+          <t>Hiển thị giá trị ```"0"``` thuộc kiểu dữ liệu ```str``` do hàm ```bool()``` giữ nguyên dạng chuỗi ký tự ban đầu.</t>
         </is>
       </c>
       <c r="H27" s="3" t="inlineStr">
         <is>
-          <t>Đáp án sai. Bẫy tư duy xuất hiện khi học viên cho rằng toán tử `*=` được thực hiện với `multiplier` trước (`"py" * 2 = "pypy"`), sau đó bỏ qua phép cộng `+ 1` hoặc hiểu sai quy tắc đồng nhất biểu thức vế phải trong phép gán kết hợp.</t>
+          <t>Kết quả thu được từ hàm ```bool()``` luôn là một giá trị thuộc kiểu dữ liệu boolean (```bool```), không thể duy trì kiểu chuỗi ký tự (```str```).</t>
         </is>
       </c>
       <c r="I27" s="3" t="inlineStr">
         <is>
-          <t>"pypy1_2.0"</t>
+          <t>Hiển thị giá trị ```True``` thuộc kiểu dữ liệu ```bool``` do hàm ```input()``` nhận về chuỗi ký tự không rỗng.</t>
         </is>
       </c>
       <c r="J27" s="3" t="inlineStr">
         <is>
-          <t>Đáp án sai. Học viên suy luận sai lầm rằng `text_data *= multiplier + 1` sẽ được phân tách thành `(text_data * multiplier) + 1` làm phát sinh việc cộng chuỗi `"pypy"` với số nguyên `1`. Trong thực tế nếu viết như vậy Python sẽ báo lỗi `TypeError`, nhưng biểu thức gán kết hợp `a *= b + c` luôn tương đương `a = a * (b + c)`.</t>
+          <t>Hàm ```input()``` luôn trả về dữ liệu thuộc kiểu chuỗi ký tự (```str```). Khi người dùng nhập ```0```, biến ```raw_val``` mang giá trị là chuỗi ```"0"```. Hàm ép kiểu ```bool("0")``` đánh giá một chuỗi có độ dài lớn hơn 0 là có giá trị đúng, do đó biến ```converted_val``` nhận giá trị boolean ```True```.</t>
         </is>
       </c>
       <c r="K27" s="2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="L27" s="2" t="n">
         <v>10</v>
@@ -2354,56 +2229,53 @@
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>Xem xét thứ tự ưu tiên của các toán tử số học trong đoạn mã Python 3.12 sau. Giá trị của biến `total_score` sau khi hoàn thành tính toán là bao nhiêu?
+          <t>Trong môi trường Python 3.12, một lập trình viên thực hiện ép kiểu và in dữ liệu ra màn hình console bằng đoạn mã sau:
 ```python
-initial_val = 5
-initial_val += 3 * 2 ** 2
-ratio_val = 25 / 2 // 2
-total_score = initial_val - ratio_val
-```</t>
+price_text = "100.75"
+price_num = int(float(price_text))
+print(price_num)
+```
+Kết quả hiển thị trên màn hình console và cơ chế chuyển đổi dữ liệu của đoạn mã trên là gì?</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>-8.0</t>
+          <t>Hiển thị giá trị ```100.75``` do hàm ```int()``` tự động bảo toàn giá trị thập phân ban đầu của chuỗi ký tự.</t>
         </is>
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>Đáp án sai. Học viên mắc bẫy thứ tự ưu tiên toán tử từ trái sang phải của `/` và `//`, nhầm tưởng rằng `2 // 2` có độ ưu tiên cao hơn nên được thực hiện trước ra `1`, sau đó lấy `25 / 1 = 25.0`. Khi đó `ratio_val = 25.0`, dẫn đến `total_score = 17 - 25.0 = -8.0`.</t>
+          <t>Hàm ```int()``` luôn trả về một số nguyên kiểu ```int``` và cắt bỏ hoàn toàn phần thập phân, do đó kết quả hiển thị không thể giữ lại phần thập phân ```100.75```.</t>
         </is>
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t>36.0</t>
+          <t>Báo lỗi ```ValueError``` do trình thông dịch Python 3.12 không cho phép thực hiện ép kiểu dữ liệu lồng nhau.</t>
         </is>
       </c>
       <c r="F28" s="3" t="inlineStr">
         <is>
-          <t>Đáp án sai. Học viên mắc lỗi nghiêm trọng về độ ưu tiên toán tử khi thực hiện phép nhân trước lũy thừa ở vế `3 * 2 ** 2` -&gt; `(3 * 2) ** 2 = 36`. Điều này khiến `initial_val` tính sai thành `5 + 36 = 41`, sau đó trừ cho `ratio_val` (`6.0`) ra kết quả sai lệch hoàn toàn.</t>
+          <t>Python 3.12 cho phép gọi lồng các hàm chuyển đổi kiểu dữ liệu hợp lệ. Việc thực hiện ```int(float("100.75"))``` là hoàn toàn hợp lệ và chương trình thực thi bình thường mà không phát sinh lỗi ```ValueError```.</t>
         </is>
       </c>
       <c r="G28" s="3" t="inlineStr">
         <is>
-          <t>11.0</t>
+          <t>Hiển thị giá trị ```100``` do chuỗi được chuyển sang kiểu ```float``` trước rồi mới ép kiểu thành ```int``` làm mất phần thập phân.</t>
         </is>
       </c>
       <c r="H28" s="3" t="inlineStr">
         <is>
-          <t>Đáp án đúng. Thứ tự thực thi được phân tích chi tiết như sau:
-1. Biểu thức `3 * 2 ** 2`: Toán tử lũy thừa `**` có độ ưu tiên cao nhất -&gt; `2 ** 2 = 4`. Phép nhân thực hiện tiếp -&gt; `3 * 4 = 12`. Phép gán kết hợp `initial_val += 12` -&gt; `initial_val = 5 + 12 = 17`.
-2. Biểu thức `25 / 2 // 2`: Các toán tử `/` và `//` có cùng độ ưu tiên nên được tính từ trái sang phải. `25 / 2` cho kết quả số thực `12.5`. Sau đó `12.5 // 2` thực hiện chia lấy phần nguyên trên số thực, trả về `6.0`.
-3. Biểu thức `total_score = 17 - 6.0`: Phép trừ giữa `int` và `float` tự động nâng kiểu lên `float`, cho kết quả chính xác là `11.0`.</t>
+          <t>Hàm ```float("100.75")``` chuyển đổi chuỗi ký tự thành số thực ```100.75```. Sau đó, hàm ```int(100.75)``` tiếp nhận số thực và thực hiện cắt bỏ toàn bộ phần thập phân (chỉ giữ phần nguyên), trả về giá trị số nguyên ```100``` để hàm ```print()``` xuất ra màn hình console.</t>
         </is>
       </c>
       <c r="I28" s="3" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>Hiển thị giá trị ```101``` do hàm ```int()``` tự động làm tròn lên số nguyên gần nhất khi ép kiểu từ ```float```.</t>
         </is>
       </c>
       <c r="J28" s="3" t="inlineStr">
         <is>
-          <t>Đáp án sai. Học viên đã tính đúng giá trị số học (11) nhưng bỏ qua quy tắc chuyển đổi kiểu dữ liệu tự động trong Python. Phép chia `/` luôn trả về kiểu `float` (`12.5`), khiến kết quả của `//` tiếp theo là `6.0` (`float`). Khi lấy số nguyên `17` trừ cho `6.0`, kết quả bắt buộc phải là số thực `11.0` chứ không phải số nguyên `11`.</t>
+          <t>Hàm ```int()``` khi chuyển đổi số thực sang số nguyên chỉ thực hiện cơ chế cắt bỏ phần thập phân (truncation) chứ không thực hiện quy tắc làm tròn (rounding), vì vậy kết quả nhận được là ```100```.</t>
         </is>
       </c>
       <c r="K28" s="2" t="n">
@@ -2424,57 +2296,57 @@
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>Trong một mô-đun tính toán tài chính của ứng dụng Python 3.12, nhà phát triển gặp sự cố sai lệch kết quả khi thực hiện phép toán lũy thừa và chia lấy phần nguyên với số âm. Xét đoạn mã nguồn sau:
+          <t>Xét đoạn mã xử lý kiểu dữ liệu logic trong Python 3.12 sau:
 ```python
-initial_val = -3 ** 2 // 2
-corrected_val = (-3) ** 2 // 2
-print(f"{initial_val}_{corrected_val}")
+data_a = bool("False")
+data_b = bool("")
+print(data_a, data_b)
 ```
-Kết quả in ra màn hình console là gì và tại sao lại có sự khác biệt này?</t>
+Kết quả hiển thị chính xác ra màn hình console khi thực thi đoạn mã trên là gì?</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>"-4_4"</t>
+          <t>Giá trị `False` cho `data_a` và giá trị `True` cho `data_b`</t>
         </is>
       </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
-          <t>Đáp án sai: Người học thường nhầm lẫn rằng phép chia lấy phần nguyên `//` với số âm sẽ cắt bỏ phần thập phân (truncate toward zero) như trong một số ngôn ngữ lập trình khác (như C/C++ hay Java) khiến `-9 // 2` thành `-4`. Thực tế, Python sử dụng nguyên tắc làm tròn xuống (floor toward negative infinity) nên `-9 // 2` phải là `-5`.</t>
+          <t>Phương án này không chính xác vì chuỗi `"False"` không rỗng nên `data_a` nhận giá trị `True`, còn chuỗi rỗng `""` không chứa ký tự nào nên `data_b` nhận giá trị `False`.</t>
         </is>
       </c>
       <c r="E29" s="3" t="inlineStr">
         <is>
-          <t>"4_4"</t>
+          <t>Giá trị `True` cho `data_a` và giá trị `True` cho `data_b`</t>
         </is>
       </c>
       <c r="F29" s="3" t="inlineStr">
         <is>
-          <t>Đáp án sai: Đây là bẫy phổ biến khi cho rằng dấu âm `-` sẽ được kết hợp với cơ số `3` trước khi thực hiện phép lũy thừa `**` (tức hiểu nhầm `-3 ** 2` là `(-3) ** 2 = 9`). Trên thực tế, toán tử `**` có độ ưu tiên toán tử cao hơn toán tử dấu âm một ngôi `-`.</t>
+          <t>Phương án này không chính xác vì chuỗi rỗng `""` được Python đánh giá là giá trị falsy, khi chuyển đổi bằng hàm `bool()` sẽ cho kết quả là `False` chứ không phải `True`.</t>
         </is>
       </c>
       <c r="G29" s="3" t="inlineStr">
         <is>
-          <t>"-5_4.5"</t>
+          <t>Giá trị `True` cho `data_a` và giá trị `False` cho `data_b`</t>
         </is>
       </c>
       <c r="H29" s="3" t="inlineStr">
         <is>
-          <t>Đáp án sai: Nhầm lẫn rằng phép chia lấy phần nguyên `//` khi áp dụng trên các số nguyên vẫn trả về số thực kiểu `float`. Toán tử `//` giữa hai số nguyên (`int`) luôn trả về kết quả thuộc kiểu số nguyên (`int`), do đó `9 // 2` trả về `4` chứ không phải `4.5`.</t>
+          <t>Trong Python, hàm `bool()` chuyển đổi một chuỗi ký tự thành `True` nếu chuỗi đó không rỗng (chứa ít nhất một ký tự, kể cả chuỗi `"False"`). Hàm `bool("")` trả về `False` vì chuỗi truyền vào là chuỗi rỗng.</t>
         </is>
       </c>
       <c r="I29" s="3" t="inlineStr">
         <is>
-          <t>"-5_4"</t>
+          <t>Giá trị `False` cho `data_a` và giá trị `False` cho `data_b`</t>
         </is>
       </c>
       <c r="J29" s="3" t="inlineStr">
         <is>
-          <t>Đáp án đúng: Khi không có ngoặc, toán tử lũy thừa `**` có độ ưu tiên cao hơn toán tử dấu âm một ngôi (unary `-`). Do đó, `-3 ** 2` được tính là `-(3 ** 2) = -9`. Tiếp theo, phép chia lấy phần nguyên `//` trong Python làm tròn xuống phía âm vô cùng (floor), nên `-9 // 2` cho kết quả `-5`. Ngược lại, đối với `(-3) ** 2`, biểu thức trong ngoặc được tính trước thành `9`, và `9 // 2` bằng `4`.</t>
+          <t>Phương án này không chính xác vì chuỗi `"False"` có độ dài bằng 5 ký tự (chuỗi không rỗng), do đó hàm `bool("False")` trả về `True` chứ không đánh giá theo nội dung văn bản của chuỗi.</t>
         </is>
       </c>
       <c r="K29" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L29" s="2" t="n">
         <v>10</v>
@@ -2491,57 +2363,51 @@
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>Trong quá trình tối ưu hóa thuật toán xử lý dữ liệu xoay vòng (ring buffer), một lập trình viên Python 3.12 thực hiện phép toán chia lấy phần dư `%` với các số nguyên âm. Hãy phân tích đoạn mã sau:
-```python
-val_a = -13 % 4
-val_b = 13 % -4
-print(f"{val_a}:{val_b}")
-```
-Kết quả hiển thị trên màn hình console là gì?</t>
+          <t>Trong ngôn ngữ lập trình Python, việc khai báo biến phải tuân theo các quy tắc định danh chuẩn xác. Cách khai báo biến nào sau đây hoàn toàn hợp lệ?</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>"-1:-3"</t>
+          <t>Khai báo biến dạng `sys-user-2024`</t>
         </is>
       </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
-          <t>Đáp án sai: Giả định sai lầm rằng dấu của số dư luôn phụ thuộc vào số bị chia `a` đối với `val_a` và phụ thuộc số chia `b` đối với `val_b`. Thực chất trong Python, dấu của phép chia lấy phần dư `%` luôn luôn tuân theo dấu của số chia `b`.</t>
+          <t>Phương án này không chính xác vì ký tự gạch nối `-` được trình biên dịch/phiên dịch Python hiểu là toán tử trừ chứ không phải ký tự hợp lệ nằm trong tên biến.</t>
         </is>
       </c>
       <c r="E30" s="3" t="inlineStr">
         <is>
-          <t>"-1:1"</t>
+          <t>Khai báo biến dạng `_sys_user_2024`</t>
         </is>
       </c>
       <c r="F30" s="3" t="inlineStr">
         <is>
-          <t>Đáp án sai: Đây là kết quả thu được nếu áp dụng định nghĩa phần dư của ngôn ngữ C/C++ hoặc Java (nơi phép chia cắt bỏ phần thập phân hướng về 0 - truncate toward zero, khiến phần dư cùng dấu với số bị chia `a`). Học viên nhầm lẫn giữa cơ chế của Python và C sẽ tính nhầm `-13 % 4` thành `-1`.</t>
+          <t>Tên biến trong Python hợp lệ khi bắt đầu bằng một chữ cái hoặc dấu gạch dưới `_`, theo sau có thể là chữ cái, chữ số hoặc dấu gạch dưới. Do đó `_sys_user_2024` là định danh hoàn toàn hợp lệ.</t>
         </is>
       </c>
       <c r="G30" s="3" t="inlineStr">
         <is>
-          <t>"3:1"</t>
+          <t>Khai báo biến dạng `sys user 2024`</t>
         </is>
       </c>
       <c r="H30" s="3" t="inlineStr">
         <is>
-          <t>Đáp án sai: Nhầm lẫn trong tính toán phép chia phần nguyên `13 // -4` thành `-3` (tính sai theo kiểu cắt bỏ phần thập phân hướng về 0) dẫn đến `r = 13 - (-3 * -4) = 1`, khiến kết quả `val_b` bị tính sai dấu từ `-3` thành `1`.</t>
+          <t>Phương án này không chính xác vì tên biến trong Python không được phép chứa khoảng trắng phân tách giữa các từ, việc đặt khoảng trắng sẽ dẫn đến lỗi cú pháp (`SyntaxError`).</t>
         </is>
       </c>
       <c r="I30" s="3" t="inlineStr">
         <is>
-          <t>"3:-3"</t>
+          <t>Khai báo biến dạng `2024_sys_user`</t>
         </is>
       </c>
       <c r="J30" s="3" t="inlineStr">
         <is>
-          <t>Đáp án đúng: Trong Python, kết quả của toán tử chia lấy phần dư `%` luôn cùng dấu với số chia (divisor `b`). Công thức nền tảng trong Python là `r = a - (a // b) * b`. Với `val_a`: `-13 // 4 = -4` (làm tròn xuống), do đó `-13 - (-4 * 4) = 3`. Với `val_b`: `13 // -4 = -4`, do đó `13 - (-4 * -4) = -3`.</t>
+          <t>Phương án này không chính xác vì quy tắc định danh của Python không cho phép tên biến bắt đầu bằng một chữ số (như `2024`), việc này sẽ gây ra lỗi cú pháp (`SyntaxError`).</t>
         </is>
       </c>
       <c r="K30" s="2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L30" s="2" t="n">
         <v>10</v>
@@ -2558,53 +2424,54 @@
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>Phân tích thứ tự ưu tiên của toán tử số học và toán tử bitwise trong Python 3.12. Cho đoạn mã nguồn sau:
+          <t>Xét đoạn mã nhập và xử lý dữ liệu từ bàn phím trong Python như sau:
 ```python
-base_val = 5
-result_val = ~base_val &lt;&lt; 2 + 1
-print(result_val)
+val_a = input()
+val_b = input()
+result = val_a + val_b
+print(type(result), result)
 ```
-Giá trị của biến `result_val` được in ra màn hình là bao nhiêu?</t>
+Nếu người dùng lần lượt nhập vào từ màn hình console hai giá trị là `10` và `20`, kết quả xuất ra màn hình là gì?</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>"32"</t>
+          <t>Kiểu dữ liệu `&lt;class 'str'&gt;` cùng giá trị kết quả là `30`</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>Đáp án sai: Bẫy nhầm lẫn toán tử `~` với phép tính bù 1 hoặc đảo thành số dương `4`, dẫn đến việc lấy `4 &lt;&lt; 3 = 32`. Trong Python, số nguyên có độ chính xác vô hạn và bit dấu luôn được bảo toàn theo dạng số bù 2.</t>
+          <t>Phương án này không chính xác vì mặc dù kiểu dữ liệu trả về đúng là `str`, nhưng toán tử `+` trên hai chuỗi `"10"` và `"20"` ghép nối hai chuỗi thành `"1020"` chứ không thực hiện phép cộng số học ra `30`.</t>
         </is>
       </c>
       <c r="E31" s="3" t="inlineStr">
         <is>
-          <t>"-48"</t>
+          <t>Kiểu dữ liệu `&lt;class 'str'&gt;` cùng giá trị kết quả là `1020`</t>
         </is>
       </c>
       <c r="F31" s="3" t="inlineStr">
         <is>
-          <t>Đáp án đúng: Thứ tự ưu tiên toán tử trong Python được thực hiện như sau: 1. Toán tử một ngôi `~` (bitwise NOT) thực hiện trước: `~5` bằng `-(5 + 1) = -6`. 2. Toán tử số học cộng `+` có độ ưu tiên cao hơn toán tử dịch bit `&lt;&lt;`, nên `2 + 1` được tính trước thành `3`. 3. Cuối cùng, thực hiện phép dịch trái `-6 &lt;&lt; 3`, tương đương với `-6 * (2**3) = -6 * 8 = -48`.</t>
+          <t>Hàm `input()` trong Python luôn trả về dữ liệu thuộc kiểu chuỗi ký tự (`str`). Khi sử dụng toán tử `+` giữa hai chuỗi `"10"` và `"20"`, Python thực hiện thao tác nối chuỗi tạo thành `"1020"` với kiểu dữ liệu là `&lt;class 'str'&gt;`.</t>
         </is>
       </c>
       <c r="G31" s="3" t="inlineStr">
         <is>
-          <t>"-40"</t>
+          <t>Kiểu dữ liệu `&lt;class 'int'&gt;` cùng giá trị kết quả là `30`</t>
         </is>
       </c>
       <c r="H31" s="3" t="inlineStr">
         <is>
-          <t>Đáp án sai: Bẫy về cách hoạt động của toán tử đảo bit `~`. Người học nhầm lẫn cho rằng `~5` chỉ đơn thuần là đổi dấu thành `-5` (thay vì biểu diễn bù 2 là `-(x + 1)` tức `-(5 + 1) = -6`), dẫn đến phép tính sai `-5 &lt;&lt; 3 = -40`.</t>
+          <t>Phương án này không chính xác vì hàm `input()` không tự động chuyển đổi dữ liệu nhập vào thành kiểu số nguyên (`int`), trừ khi gọi hàm ép kiểu `int(input())` một cách rõ ràng.</t>
         </is>
       </c>
       <c r="I31" s="3" t="inlineStr">
         <is>
-          <t>"-23"</t>
+          <t>Kiểu dữ liệu `&lt;class 'float'&gt;` cùng giá trị kết quả là `30.0`</t>
         </is>
       </c>
       <c r="J31" s="3" t="inlineStr">
         <is>
-          <t>Đáp án sai: Bẫy về thứ tự ưu tiên toán tử. Người học thường lầm tưởng toán tử dịch bit `&lt;&lt;` có độ ưu tiên cao hơn toán tử cộng `+`, dẫn đến việc tính toán sai thứ tự thành `(~5 &lt;&lt; 2) + 1` = `(-6 &lt;&lt; 2) + 1` = `-24 + 1 = -23`.</t>
+          <t>Phương án này không chính xác vì dữ liệu nhận từ `input()` là kiểu `str`, toán tử `+` sẽ tiến hành nối hai chuỗi lại với nhau chứ không ép kiểu thành số thực để tính toán số học.</t>
         </is>
       </c>
       <c r="K31" s="2" t="n">
@@ -2625,64 +2492,57 @@
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>Phân tích đoạn mã nguồn Python 3.12 dưới đây sử dụng các toán tử số học cơ bản:
+          <t>Cho đoạn mã Python 3.12 xử lý chuyển đổi kiểu dữ liệu như sau:
 ```python
-base_val = 2
-exp_val = 3
-mod_val = 5
-result = -base_val ** exp_val ** 2 // mod_val
+user_status = "False"
+is_active = bool(user_status)
+print(type(is_active), is_active)
 ```
-Cho biết giá trị và kiểu dữ liệu của biến `result` sau khi đoạn mã trên được thực thi thành công?</t>
+Kết quả xuất ra màn hình console khi thực thi đoạn mã trên là gì?</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>`result` có giá trị là `-103` kiểu `int`, do toán tử `**` kết hợp từ phải qua trái (`3 ** 2 = 9`, `2 ** 9 = 512`), unary `-` biến thành `-512`, và chia lấy nguyên `//` làm tròn xuống số nguyên âm gần nhất.</t>
+          <t>Kết quả là `&lt;class 'str'&gt; False` vì hàm `bool()` giữ nguyên kiểu dữ liệu ban đầu và chỉ biến đổi định dạng.</t>
         </is>
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>Đáp án đúng là A. Phân tích thứ tự ưu tiên (Precedence) và chiều kết hợp (Associativity) của các toán tử trong Python:
-1. Toán tử lũy thừa `**` có chiều kết hợp từ phải sang trái (right-to-left associativity). Do đó biểu thức `exp_val ** 2` được tính trước: `3 ** 2 = 9`. Tiếp theo, `base_val ** 9` được tính: `2 ** 9 = 512`.
-2. Toán tử âm một ngôi (unary minus) `-` có độ ưu tiên thấp hơn toán tử lũy thừa `**`. Do đó `-base_val ** ...` được hiểu là `-(2 ** 9) = -512`.
-3. Toán tử chia lấy nguyên `//` có cùng độ ưu tiên với phép nhân/chia và thực hiện cơ chế floor division (làm tròn xuống về phía âm vô cực). Phép tính `-512 // 5` cho kết quả thực tế là `-102.4`, làm tròn xuống số nguyên gần nhất là `-103`.
-Vì hai toán hạng `-512` và `5` đều thuộc kiểu `int`, kết quả `result` mang giá trị `-103` kiểu `int`.</t>
+          <t>Hàm `bool()` khởi tạo một đối tượng mới thuộc kiểu dữ liệu `bool`, không giữ nguyên kiểu dữ liệu chuỗi `str` của biến đầu vào.</t>
         </is>
       </c>
       <c r="E32" s="3" t="inlineStr">
         <is>
-          <t>`result` có giá trị là `12` kiểu `int`, do biểu thức `(-2 ** 3)` được tính trước bằng `-8`, sau đó `(-8) ** 2 = 64`, và cuối cùng `64 // 5 = 12`.</t>
+          <t>Chương trình dừng và báo lỗi `ValueError` vì chuỗi `"False"` không thể chuyển đổi trực tiếp sang kiểu `bool`.</t>
         </is>
       </c>
       <c r="F32" s="3" t="inlineStr">
         <is>
-          <t>Đáp án B sai vì hai lý do nghiêm trọng về mặt cú pháp toán tử:
-1. Toán tử âm một ngôi `-` KHÔNG được tính gộp vào cơ số nếu không có dấu ngoặc đơn `(-2)`. Do đó `-2 ** 3` trong Python được hiểu là `-(2 ** 3) = -8`, không phải toán tử âm gắn liền với biến.
-2. Quan trọng hơn, toán tử lũy thừa `**` kết hợp từ PHẢI sang TRÁI (right-associative). Biểu thức `2 ** 3 ** 2` phải được tính là `2 ** (3 ** 2) = 2 ** 9 = 512`, chứ không tính từ trái sang phải `(2 ** 3) ** 2 = 64`.</t>
+          <t>Cú pháp `bool("False")` hoàn toàn hợp lệ trong Python và không gây ra lỗi `ValueError` trong quá trình thực thi.</t>
         </is>
       </c>
       <c r="G32" s="3" t="inlineStr">
         <is>
-          <t>`result` có giá trị là `-102.4` kiểu `float`, do toán tử `//` khi kết hợp với toán tử âm một ngôi sẽ tự động ép kiểu kết quả về `float`.</t>
+          <t>Kết quả là `&lt;class 'bool'&gt; False` vì hàm `bool()` tự động nhận diện giá trị ngữ nghĩa của chuỗi `"False"`.</t>
         </is>
       </c>
       <c r="H32" s="3" t="inlineStr">
         <is>
-          <t>Đáp án D sai vì toán tử chia lấy nguyên `//` giữa hai toán hạng kiểu nguyên (`int // int`) BẮT BUỘC luôn trả về một số nguyên kiểu `int`. Toán tử `//` không bao giờ tự động biến kết quả thành `float` chỉ vì sự xuất hiện của toán tử âm một ngôi `-`. Phép chia `/` mới là toán tử luôn trả về kiểu `float`.</t>
+          <t>Hàm `bool()` không phân tích cú pháp giá trị chữ bên trong chuỗi để hiểu ngữ nghĩa. Việc cho rằng chuỗi `"False"` chuyển thành `False` là sai lầm phổ biến do nhầm lẫn giữa kiểu boolean và string.</t>
         </is>
       </c>
       <c r="I32" s="3" t="inlineStr">
         <is>
-          <t>`result` có giá trị là `-102` kiểu `int`, do phép chia lấy nguyên `//` cắt bỏ phần thập phân (truncation towards zero) của `-102.4`.</t>
+          <t>Kết quả là `&lt;class 'bool'&gt; True` vì hàm `bool()` đánh giá mọi chuỗi ký tự khác rỗng là `True`.</t>
         </is>
       </c>
       <c r="J32" s="3" t="inlineStr">
         <is>
-          <t>Đáp án C sai do nhầm lẫn về cơ chế hoạt động của toán tử chia lấy nguyên `//` trong Python. Khác với các ngôn ngữ như C/C++ hay Java thực hiện cắt bỏ phần thập phân (truncation towards zero, biến `-102.4` thành `-102`), toán tử `//` trong Python thực hiện phép làm tròn sàn (floor division - làm tròn xuống số nguyên nhỏ hơn hoặc bằng nó gần nhất trên trục số). Đối với giá trị `-102.4`, số nguyên nhỏ hơn gần nhất về phía âm vô cực là `-103`.</t>
+          <t>Trong Python, hàm khởi tạo `bool()` khi nhận vào một chuỗi ký tự sẽ kiểm tra độ dài của chuỗi đó. Chuỗi `"False"` có độ dài 5 ký tự (khác rỗng) nên kết quả trả về là đối tượng luận lý `True` thuộc lớp `&lt;class 'bool'&gt;`.</t>
         </is>
       </c>
       <c r="K32" s="2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="L32" s="2" t="n">
         <v>10</v>
@@ -2699,64 +2559,57 @@
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>Xét đoạn mã Python 3.12 thực hiện các toán tử chia lấy nguyên `//`, chia lấy dư `%` trên số âm và toán tử nhân chuỗi `*` như sau:
+          <t>Cho đoạn mã Python 3.12 thực hiện khai báo và khởi tạo các biến như sau:
 ```python
-dividend_val = -19
-divisor_val = 4
-quotient_val = dividend_val // divisor_val
-remainder_val = dividend_val % divisor_val
-pattern_str = "*" * remainder_val
-output_text = f"{quotient_val}|{pattern_str}"
+item_price = 50_000
+_discount_rate = 0.15
+1st_buyer_flag = True
 ```
-Kết quả của biến `output_text` sau khi chạy chương trình là gì?</t>
+Phát biểu nào sau đây phản ánh đúng nhất về tính hợp lệ cú pháp của đoạn mã trên?</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>Chương trình phát sinh lỗi `TypeError` tại dòng `pattern_str = "*" * remainder_val` do không thể nhân chuỗi với kết quả của phép chia lấy dư từ một số bị chia âm.</t>
+          <t>Dòng lệnh `item_price = 50_000` gây lỗi `ValueError` vì cú pháp số nguyên không được phép chứa dấu gạch dưới `_`.</t>
         </is>
       </c>
       <c r="D33" s="3" t="inlineStr">
         <is>
-          <t>Đáp án C sai vì phép toán chia lấy dư `-19 % 4` trả về kết quả là một số nguyên dương hợp lệ (`1`). Toán tử nhân chuỗi `*` với một số nguyên dương là một thao tác hoàn toàn hợp lệ trong Python (chuỗi được lặp lại số lần tương ứng). Không có lỗi `TypeError` nào xảy ra.</t>
+          <t>Python cho phép sử dụng dấu gạch dưới `_` trong các hằng số số học (như `50_000`) để tăng tính dễ đọc của mã nguồn, giá trị lưu trữ vẫn là số nguyên `50000` hợp lệ.</t>
         </is>
       </c>
       <c r="E33" s="3" t="inlineStr">
         <is>
-          <t>Giá trị của `output_text` là `"-5|*"`, do `quotient_val` bằng `-5` (làm tròn xuống âm vô cực) và `remainder_val` bằng `1` (số dư luôn cùng dấu với số chia trong Python).</t>
+          <t>Tất cả các dòng lệnh trên đều hợp lệ về mặt cú pháp và chương trình sẽ thực thi bình thường mà không báo lỗi.</t>
         </is>
       </c>
       <c r="F33" s="3" t="inlineStr">
         <is>
-          <t>Đáp án đúng là A. Phân tích từng toán tử cơ bản với toán hạng âm trong Python:
-1. Phép chia lấy nguyên `dividend_val // divisor_val` = `-19 // 4`: Phép chia số thực cho ra `-4.75`. Toán tử `//` làm tròn xuống (floor) về số nguyên nhỏ hơn gần nhất, thu được `quotient_val = -5`.
-2. Phép chia lấy dư `dividend_val % divisor_val` = `-19 % 4`: Trong Python, toán tử `%` tuân theo công thức `r = a - (b * (a // b))`. Thay số ta có: `r = -19 - (4 * -5) = -19 - (-20) = 1`. Do đó `remainder_val = 1` (luôn cùng dấu với số chia `divisor_val = 4`).
-3. Toán tử nhân chuỗi `pattern_str = "*" * 1` trả về chuỗi `"*"`.
-4. Định dạng f-string ghép hai giá trị lại tạo thành chuỗi `"-5|*"`.</t>
+          <t>Phát biểu này sai vì khai báo `1st_buyer_flag = True` bắt đầu bằng chữ số `1` làm trình dịch báo lỗi `SyntaxError` ngay khi phân tích mã.</t>
         </is>
       </c>
       <c r="G33" s="3" t="inlineStr">
         <is>
-          <t>Giá trị của `output_text` là `"-5|"`, do `remainder_val` bằng `-3` và toán tử nhân chuỗi với số nguyên âm trả về chuỗi rỗng `""`.</t>
+          <t>Dòng lệnh `_discount_rate = 0.15` gây lỗi `NameError` vì tên biến bắt đầu bằng dấu gạch dưới là ký tự bất hợp lệ.</t>
         </is>
       </c>
       <c r="H33" s="3" t="inlineStr">
         <is>
-          <t>Đáp án D sai vì xác định sai giá trị của `remainder_val`. Đúng là trong Python, khi nhân một chuỗi với số nguyên âm hoặc `0` (ví dụ `"*" * -3`), kết quả sẽ là chuỗi rỗng `""`. Tuy nhiên, kết quả của phép tính `-19 % 4` trong Python là `1` (số dương), KHÔNG PHẢI `-3`. Nguyên nhân vì toán tử `%` trong Python luôn trả về số dư cùng dấu với số chia (`divisor_val = 4` là số dương).</t>
+          <t>Dấu gạch dưới `_` là ký tự bắt đầu hoàn toàn hợp lệ cho tên biến trong Python và thường được dùng cho các biến nội bộ hoặc biến riêng tư.</t>
         </is>
       </c>
       <c r="I33" s="3" t="inlineStr">
         <is>
-          <t>Giá trị của `output_text` là `"-4|***"`, do `quotient_val` bằng `-4` (cắt phần thập phân của `-4.75`) và `remainder_val` bằng `-3` nhưng toán tử nhân chuỗi tự động đổi dấu thành `3`.</t>
+          <t>Dòng lệnh `1st_buyer_flag = True` gây lỗi `SyntaxError` vì tên biến trong Python cấm bắt đầu bằng chữ số.</t>
         </is>
       </c>
       <c r="J33" s="3" t="inlineStr">
         <is>
-          <t>Đáp án B sai vì áp dụng sai cơ chế chia số âm trong Python. Học viên bị ảnh hưởng bởi tư duy của ngôn ngữ C/C++/Java (nơi `-19 / 4 = -4` và phần dư là `-3`). Trong Python, phép chia lấy nguyên `//` luôn làm tròn về phía âm vô cực (`-4.75` tròn xuống thành `-5`), và phép toán `%` không bao giờ tự đổi dấu số dư theo cách thủ công mà tính theo công thức chuẩn của toán tử Python.</t>
+          <t>Theo quy tắc đặt tên định danh (identifier) trong Python, tên biến chỉ được bắt đầu bằng một chữ cái (a-z, A-Z) hoặc dấu gạch dưới `_`. Việc bắt đầu tên biến bằng chữ số như `1st_buyer_flag` vi phạm quy tắc cú pháp và dẫn đến `SyntaxError`.</t>
         </is>
       </c>
       <c r="K33" s="2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L33" s="2" t="n">
         <v>10</v>
@@ -2773,62 +2626,53 @@
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>Đánh giá đoạn mã Python 3.12 sau đây về thao tác chuyển đổi kiểu dữ liệu ngầm định và độ ưu tiên của các toán tử số học:
+          <t>Cho đoạn mã Python 3.12 thực hiện thao tác ép kiểu dữ liệu như sau:
 ```python
-num_x = 7.0
-num_y = 2
-res_a = num_x // num_y
-res_b = num_x / num_y
-res_c = int(num_x) % num_y
-final_val = res_a + res_b * res_c
-output_str = f"Val: {final_val:.2f} | Type: {type(final_val).__name__}"
+user_input = "45.7"
+result = int(user_input)
+print(result)
 ```
-Giá trị chính xác của chuỗi `output_str` thu được sau khi đoạn mã thực thi là gì?</t>
+Hành vi thực thi của đoạn mã trên trên hệ thống là gì?</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>Giá trị của `output_str` là `"Val: 6.00 | Type: float"`, do `res_a` bằng `3.0` và `res_b` bằng `3.0` (phép chia `/` bị tự động ép thành chia nguyên vì cả hai giá trị đều được làm tròn).</t>
+          <t>Chương trình in ra giá trị `45` vì hàm `int()` tự động loại bỏ phần thập phân của chuỗi truyền vào.</t>
         </is>
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t>Đáp án C sai vì hiểu sai bản chất của toán tử chia thực `/`. Trong Python 3, toán tử `/` BẤT KỂ toán hạng là nguyên hay thực, luôn thực hiện phép chia chính xác và trả về số thực `float`. Do đó `7.0 / 2` cho kết quả chính xác là `3.5`, không bao giờ bị cắt phần thập phân thành `3.0`.</t>
+          <t>Hàm `int()` chỉ cắt bỏ phần thập phân khi đối số truyền vào là một số thực (ví dụ `int(45.7)`). Nếu đối số là chuỗi ký tự số thực `"45.7"`, hàm sẽ báo lỗi `ValueError` chứ không tự động cắt bỏ.</t>
         </is>
       </c>
       <c r="E34" s="3" t="inlineStr">
         <is>
-          <t>Chương trình phát sinh lỗi `TypeError` tại dòng `res_a = num_x // num_y` vì toán tử chia lấy nguyên `//` chỉ chấp nhận các toán hạng là số nguyên `int`.</t>
+          <t>Chương trình in ra giá trị `46` vì hàm `int()` tự động thực hiện quy tắc làm tròn số nguyên gần nhất.</t>
         </is>
       </c>
       <c r="F34" s="3" t="inlineStr">
         <is>
-          <t>Đáp án D sai vì toán tử chia lấy nguyên `//` trong Python hoàn toàn hỗ trợ cả số nguyên `int` lẫn số thực `float` (ví dụ `7.0 // 2`, `7.5 // 2.5`). Ngoại lệ `TypeError` sẽ không bao giờ xảy ra trong tình huống này.</t>
+          <t>Hàm `int()` không thực hiện phép làm tròn số học (round) đối với dữ liệu đầu vào. Việc truyền chuỗi `"45.7"` trực tiếp vào `int()` gây lỗi `ValueError`.</t>
         </is>
       </c>
       <c r="G34" s="3" t="inlineStr">
         <is>
-          <t>Giá trị của `output_str` là `"Val: 6.50 | Type: int"`, vì phép chia lấy nguyên `//` đã ép `res_a` về kiểu `int` (`3`), kết hợp với `res_c` kiểu `int` làm cho tổng thể bị ép kiểu ngược lại thành `int`.</t>
+          <t>Chương trình in ra giá trị `45.7` vì kiểu dữ liệu của `result` tự động chuyển thành kiểu `float`.</t>
         </is>
       </c>
       <c r="H34" s="3" t="inlineStr">
         <is>
-          <t>Đáp án B sai vì hiểu sai quy tắc kiểu dữ liệu của toán tử `//`. Toán tử chia lấy nguyên `//` KHÔNG bắt buộc trả về kiểu `int`. Nếu toán hạng tham gia chứa số thực `float` (`num_x = 7.0`), kết quả của `//` sẽ là `float` (`3.0`). Ngoài ra, trong biểu thức toán học chứa cả `float` và `int`, Python luôn ưu tiên thúc đẩy kiểu dữ liệu lên `float` (type promotion) chứ không bao giờ ép ngược về `int`.</t>
+          <t>Python là ngôn ngữ định kiểu động nhưng không tự động thay đổi kiểu trả về của hàm `int()` thành `float` để tránh lỗi; lệnh gán sẽ dừng lại do phát sinh ngoại lệ `ValueError`.</t>
         </is>
       </c>
       <c r="I34" s="3" t="inlineStr">
         <is>
-          <t>Giá trị của `output_str` là `"Val: 6.50 | Type: float"`, do `res_a` bằng `3.0` (float), `res_b` bằng `3.5` (float), `res_c` bằng `1` (int), và biểu thức hỗn hợp giữa float và int luôn tự động ép kiểu ngầm định về `float`.</t>
+          <t>Chương trình báo lỗi `ValueError` vì hàm `int()` không thể ép trực tiếp một chuỗi biểu diễn số thực.</t>
         </is>
       </c>
       <c r="J34" s="3" t="inlineStr">
         <is>
-          <t>Đáp án đúng là A. Phân tích chi tiết quy tắc ép kiểu và toán tử trong Python:
-1. `res_a = 7.0 // 2`: Khi có ít nhất một toán hạng là `float`, toán tử chia lấy nguyên `//` vẫn thực hiện làm tròn xuống nhưng trả về kết quả kiểu `float` là `3.0`.
-2. `res_b = 7.0 / 2`: Toán tử chia thực `/` luôn trả về kết quả kiểu `float` là `3.5`.
-3. `res_c = int(7.0) % 2` = `7 % 2 = 1` kiểu `int`.
-4. Phép tính `final_val = res_a + res_b * res_c`: Phép nhân `res_b * res_c` (`3.5 * 1`) được thực hiện trước, thu được `3.5` kiểu `float` (do thúc đẩy kiểu giữa float và int). Tiếp đó `res_a + 3.5` (`3.0 + 3.5`) thu được `6.5` kiểu `float`.
-5. F-string `{final_val:.2f}` định dạng `6.5` thành `"6.50"` và `type(final_val).__name__` trả về tên kiểu dữ liệu `"float"`. Tổng hợp thành `"Val: 6.50 | Type: float"`.</t>
+          <t>Hàm `int()` khi nhận đối tượng đầu vào là chuỗi ký tự thì chuỗi đó phải là biểu diễn của một số nguyên hợp lệ (như `"45"`). Khi truyền chuỗi chứa dấu chấm thập phân `"45.7"`, Python không tự động chuyển đổi trung gian mà phát sinh ngay lỗi `ValueError`. Để xử lý đúng cần qua hai bước: `int(float(user_input))`.</t>
         </is>
       </c>
       <c r="K34" s="2" t="n">
@@ -2849,58 +2693,56 @@
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>Trong phiên bản Python 3.12, đoạn mã xử lý tính toán thứ tự ưu tiên của toán tử số học dưới đây sẽ cho kết quả biến `final_value` là bao nhiêu?
+          <t>Xét đoạn mã nguồn Python xử lý nhập dữ liệu từ console sau:
 ```python
-initial_cost = 3
-final_value = -initial_cost ** 2 + 17 % 5 * 3 // 2
-```</t>
+age = input("Nhập tuổi của bạn: ")
+print(type(age))
+```
+Khi người dùng nhập giá trị `25` từ màn hình console, kết quả kiểm tra kiểu dữ liệu của biến `age` và lý do là gì?</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>Kiểu `str`, vì hàm `input()` luôn đọc dữ liệu vào dưới dạng một chuỗi văn bản từ console bất kể nội dung người dùng nhập vào.</t>
         </is>
       </c>
       <c r="D35" s="3" t="inlineStr">
         <is>
-          <t>Đáp án sai. Lỗi này xảy ra khi tính sai kết quả phép chia lấy dư `17 % 5` hoặc nhầm lẫn quy tắc dấu làm phép toán cộng/trừ số âm bị sai lệch kết quả.</t>
+          <t>Hàm `input()` trong Python luôn trả về một giá trị thuộc kiểu dữ liệu chuỗi (`str`), ngay cả khi nội dung người dùng nhập vào toàn các chữ số như `25`.</t>
         </is>
       </c>
       <c r="E35" s="3" t="inlineStr">
         <is>
-          <t>-7.5</t>
+          <t>Kiểu `float`, vì các dữ liệu số nhập từ màn hình console mặc định được quy đổi về dạng số thực để đảm bảo độ chính xác.</t>
         </is>
       </c>
       <c r="F35" s="3" t="inlineStr">
         <is>
-          <t>Đáp án sai. Nguyên nhân xuất phát từ việc hiểu sai toán tử chia lấy phần nguyên `//` thành toán tử chia thực `/` (`6 / 2 = 3.0`), hoặc tính sai thứ tự ưu tiên nhóm toán tử nhân/chia/chia lấy dư làm kết quả chuyển thành số thực `float`.</t>
+          <t>Hàm `input()` không tự động quy đổi dữ liệu nhập vào thành kiểu số thực (`float`), người dùng phải thực hiện việc chuyển kiểu dữ liệu rõ ràng.</t>
         </is>
       </c>
       <c r="G35" s="3" t="inlineStr">
         <is>
-          <t>-6</t>
+          <t>Kiểu `int`, vì cú pháp `input()` tự động nhận diện các ký tự chữ số và chuyển đổi thành số nguyên trong Python 3.12.</t>
         </is>
       </c>
       <c r="H35" s="3" t="inlineStr">
         <is>
-          <t>Đáp án đúng. Thứ tự ưu tiên của các toán tử số học trong Python được thực hiện như sau:
-1. Toán tử lũy thừa `**` có độ ưu tiên cao hơn toán tử đổi dấu `-` (unary minus). Do đó `-initial_cost ** 2` được tính là `-(3 ** 2) = -9` chứ không phải `(-3) ** 2 = 9`.
-2. Nhóm toán tử `%`, `*`, `//` có cùng độ ưu tiên và được tính từ trái sang phải: `17 % 5 = 2`, tiếp theo `2 * 3 = 6`, cuối cùng `6 // 2 = 3`.
-3. Phép cộng `+` thực hiện cuối cùng giữa hai kết quả: `-9 + 3 = -6`.</t>
+          <t>Python không tự động ép kiểu dữ liệu từ chuỗi sang số nguyên (`int`) khi thu thập dữ liệu bằng hàm `input()`, nhà phát triển cần gọi hàm `int()` thủ công nếu muốn chuyển đổi.</t>
         </is>
       </c>
       <c r="I35" s="3" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>Kiểu `bool`, vì các giá trị nhập vào từ bàn phím được đánh giá thành một trạng thái luận lý ngay khi người dùng nhấn phím Enter.</t>
         </is>
       </c>
       <c r="J35" s="3" t="inlineStr">
         <is>
-          <t>Đáp án sai. Đây là lỗi phổ biến khi lập trình viên nhầm lẫn thứ tự ưu tiên của toán tử đổi dấu `-` (unary minus) cao hơn toán tử lũy thừa `**`, dẫn đến tính `(-3) ** 2 = 9`, sau đó cộng với `3` thành `12`.</t>
+          <t>Giá trị thu được từ `input()` là chuỗi văn bản chứ không bị ép kiểu thành `bool` trừ khi có thao tác ép kiểu chủ động.</t>
         </is>
       </c>
       <c r="K35" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="L35" s="2" t="n">
         <v>11</v>
@@ -2917,56 +2759,47 @@
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>Đoạn mã Python 3.12 dưới đây sử dụng f-string kết hợp với các toán tử trên chuỗi và số học. Giá trị in ra màn hình của biến `result` là gì?
-```python
-raw_count = "2"
-multiplier = 3
-base_val = 10
-result = f"{raw_count * multiplier + str(base_val // 4)}"
-```</t>
+          <t>Khi khởi tạo và quản lý biến trong chương trình Python, phát biểu nào sau đây mô tả đúng tên biến hợp lệ `bonus_2024` theo quy tắc đặt tên định danh?</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>"62"</t>
+          <t>Tên biến `bonus-2024` hợp lệ vì sử dụng dấu gạch nối để phân tách các từ trong cú pháp khai báo của Python.</t>
         </is>
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>Đáp án sai. Đây là bẫy khi nghĩ rằng toán tử `*` giữa chuỗi `"2"` và số `3` sẽ nhân giá trị số học trước thành `6` rồi ép thành chuỗi `"6"`, sau đó mới nối với chuỗi `"2"` tạo thành `"62"`.</t>
+          <t>Tên biến `bonus-2024` không hợp lệ vì dấu gạch nối `-` được hiểu là toán tử trừ chứ không phải ký tự hợp lệ trong tên định danh.</t>
         </is>
       </c>
       <c r="E36" s="3" t="inlineStr">
         <is>
-          <t>"2222"</t>
+          <t>Tên biến `bonus_2024` hợp lệ vì chứa chữ cái, chữ số, dấu gạch dưới và không bắt đầu bằng một chữ số.</t>
         </is>
       </c>
       <c r="F36" s="3" t="inlineStr">
         <is>
-          <t>Đáp án đúng. Quy tắc xử lý biểu thức bên trong f-string của Python 3.12 diễn ra theo các bước:
-1. Biểu thức `raw_count * multiplier` thực hiện toán tử lặp chuỗi `*` giữa `"2"` và `3`, tạo ra chuỗi `"222"`.
-2. Biểu thức `base_val // 4` thực hiện toán tử chia lấy phần nguyên số học `10 // 4 = 2`. Sau đó hàm `str(2)` ép kiểu thành chuỗi `"2"`.
-3. Toán tử `+` giữa hai chuỗi `"222" + "2"` đóng vai trò là toán tử nối chuỗi, tạo ra chuỗi kết quả cuối cùng là `"2222"`.</t>
+          <t>Trong Python, tên biến hợp lệ phải bắt đầu bằng một chữ cái hoặc dấu gạch dưới `_`, theo sau là các chữ cái, chữ số hoặc dấu gạch dưới. Tên `bonus_2024` đáp ứng đầy đủ các quy tắc này.</t>
         </is>
       </c>
       <c r="G36" s="3" t="inlineStr">
         <is>
-          <t>"8"</t>
+          <t>Tên biến `bonus score` hợp lệ vì sử dụng khoảng trắng giữa các từ để tăng tính rõ ràng khi đọc mã nguồn.</t>
         </is>
       </c>
       <c r="H36" s="3" t="inlineStr">
         <is>
-          <t>Đáp án sai. Lỗi này xảy ra do giả định sai rằng Python sẽ tự động ép kiểu chuỗi `"2"` thành số nguyên `2` để thực hiện phép nhân số học `2 * 3 = 6`, rồi cộng với `2` để ra `8`.</t>
+          <t>Tên biến `bonus score` không hợp lệ vì tên biến trong Python không được phép chứa khoảng trắng giữa các ký tự.</t>
         </is>
       </c>
       <c r="I36" s="3" t="inlineStr">
         <is>
-          <t>"2222.5"</t>
+          <t>Tên biến `2024_bonus` hợp lệ vì chứa chữ cái, chữ số, dấu gạch dưới và được phép bắt đầu bằng một chữ số.</t>
         </is>
       </c>
       <c r="J36" s="3" t="inlineStr">
         <is>
-          <t>Đáp án sai. Lỗi này do nhầm lẫn toán tử chia lấy phần nguyên `//` thành toán tử chia thực `/` (`10 / 4 = 2.5`), khiến kết quả ép chuỗi thành `"2.5"` và nối ra chuỗi `"2222.5"`.</t>
+          <t>Tên biến `2024_bonus` không hợp lệ vì quy tắc cú pháp của Python nghiêm cấm đặt tên biến bắt đầu bằng một chữ số.</t>
         </is>
       </c>
       <c r="K36" s="2" t="n">
@@ -2987,60 +2820,58 @@
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>Cho đoạn mã Python 3.12 thực hiện chuỗi phép toán gán phức hợp (compound assignment operators) dưới đây. Giá trị cuối cùng của biến `score_val` sau khi in ra bằng lệnh `print(score_val)` sẽ là bao nhiêu?
+          <t>Xét đoạn mã nguồn thực hiện chuyển đổi kiểu dữ liệu và tính toán cơ bản sau:
 ```python
-score_val = 50
-score_val /= 2
-score_val //= 4
-score_val %= 3
-```</t>
+price_input = "150.5"
+quantity_input = "2"
+total = float(price_input) * int(quantity_input)
+print(total)
+```
+Kết quả hiển thị trên màn hình console và kiểu dữ liệu của biến `total` sau khi thực thi là gì?</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>0.0</t>
+          <t>Giá trị `"301.0"` với kiểu dữ liệu `str`, vì các biến ban đầu là chuỗi nên kết quả thực thi vẫn giữ nguyên định dạng chuỗi.</t>
         </is>
       </c>
       <c r="D37" s="3" t="inlineStr">
         <is>
-          <t>Đáp án đúng. Phân tích tiến trình biến đổi kiểu dữ liệu và giá trị qua từng toán tử gán phức hợp:
-1. `score_val /= 2`: Toán tử chia thực `/` trong Python luôn trả về kiểu `float`. Giá trị `50 / 2` bằng `25.0` (chuyển biến `score_val` từ `int` sang `float`).
-2. `score_val //= 4`: Toán tử chia lấy phần nguyên `//` khi thực hiện với một số thực (`25.0 // 4`) vẫn trả về kiểu `float`, cho kết quả `6.0`.
-3. `score_val %= 3`: Phép chia lấy dư trên số thực `6.0 % 3` trả về `0.0` (kiểu `float`). Do đó hàm `print(score_val)` sẽ hiển thị `0.0`.</t>
+          <t>Các hàm `float()` và `int()` đã thực hiện ép kiểu từ `str` sang số, nên phép toán kết quả tạo ra giá trị số thực chứ không phải chuỗi.</t>
         </is>
       </c>
       <c r="E37" s="3" t="inlineStr">
         <is>
-          <t>2.0</t>
+          <t>Giá trị `301.0` với kiểu dữ liệu `float`, vì phép nhân giữa một số thực và một số nguyên luôn trả về kết quả thuộc kiểu số thực.</t>
         </is>
       </c>
       <c r="F37" s="3" t="inlineStr">
         <is>
-          <t>Đáp án sai. Lỗi này xuất phát từ việc tính sai kết quả phép chia lấy phần nguyên `25.0 // 4` (tính nhầm thành `7.0`), dẫn đến phép chia lấy dư `7.0 % 3` ra `1.0` hoặc `2.0`.</t>
+          <t>Hàm `float("150.5")` chuyển đổi thành `150.5` (kiểu `float`) và `int("2")` thành `2` (kiểu `int`). Khi thực hiện phép nhân giữa `float` và `int`, Python tự động nâng cấp kiểu dữ liệu kết quả thành `float`, tạo ra giá trị `301.0`.</t>
         </is>
       </c>
       <c r="G37" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Lỗi cú pháp thực thi, vì Python không cho phép thực hiện phép nhân trực tiếp giữa kiểu số thực `float` và kiểu số nguyên `int`.</t>
         </is>
       </c>
       <c r="H37" s="3" t="inlineStr">
         <is>
-          <t>Đáp án sai. Đây là lỗi phổ biến do không nắm vững cơ chế chuyển đổi kiểu dữ liệu ngầm định (implicit type coercion) của toán tử chia `/`. Học viên lầm tưởng `50 / 2` cho ra số nguyên `25` (kiểu `int`), dẫn tới tính toán các bước sau đều ra kiểu `int` và chọn nhầm `0`.</t>
+          <t>Phép nhân giữa kiểu `float` và `int` hoàn toàn hợp lệ trong Python và không gây ra bất kỳ lỗi thực thi nào.</t>
         </is>
       </c>
       <c r="I37" s="3" t="inlineStr">
         <is>
-          <t>6.0</t>
+          <t>Giá trị `301` với kiểu dữ liệu `int`, vì kết quả của phép tính là số tròn nên Python tự động đơn giản hóa về kiểu số nguyên.</t>
         </is>
       </c>
       <c r="J37" s="3" t="inlineStr">
         <is>
-          <t>Đáp án sai. Bẫy tư duy khi giả định toán tử `%=` không làm thay đổi giá trị của biến khi số bị chia chia hết cho số chia, hoặc bỏ qua không thực hiện bước gán cuối cùng `score_val %= 3`.</t>
+          <t>Python không tự động chuyển kết quả từ `float` về `int` ngay cả khi phần thập phân bằng 0, do đó giá trị giữ nguyên kiểu số thực `301.0`.</t>
         </is>
       </c>
       <c r="K37" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L37" s="2" t="n">
         <v>11</v>
@@ -3057,64 +2888,51 @@
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>Trong một mô-đun tối ưu hóa số học của hệ thống Python 3.12, lập trình viên thực hiện tính toán chỉ số phân bổ bộ nhớ bằng các toán tử số học cơ bản. Cho đoạn mã nguồn Python sau:
-```python
-buffer_size = 25
-block_size = 4
-calculated_val = buffer_size // block_size * block_size + buffer_size % block_size ** 2 / 2
-```
-Hãy xác định giá trị và kiểu dữ liệu của biến `calculated_val` thu được sau khi thực thi đoạn mã trên.</t>
+          <t>Trong ngôn ngữ lập trình Python 3.12, quy tắc đặt tên biến (identifier) yêu cầu tuân thủ đúng cú pháp chuẩn của ngôn ngữ. Xét các tập hợp khai báo biến dưới đây, tập hợp nào hoàn toàn hợp lệ và không tạo ra lỗi cú pháp ```SyntaxError``` khi thực thi?</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>`28` thuộc kiểu `int`</t>
+          <t>```user_name = "Alice"```, ```_user_age = 25```, ```is_active = True```</t>
         </is>
       </c>
       <c r="D38" s="3" t="inlineStr">
         <is>
-          <t>Phương án nhiễu sai. Học viên chọn phương án này thường do nhầm lẫn rằng phép chia `9 / 2` kết hợp với toán tử `//` ở đầu sẽ tự động ép toàn bộ biểu thức về kiểu `int` và làm tròn xuống `4`, dẫn đến phép tính `24 + 4 = 28`. Thực tế trong Python 3.12, phép chia `/` luôn trả về kết quả kiểu `float` làm cho toàn bộ biểu thức chứa nó nâng cấp sang kiểu `float` (implicit type promotion).</t>
+          <t>Khai báo này hoàn toàn hợp lệ theo quy tắc đặt tên biến của Python: tên biến có thể bắt đầu bằng chữ cái hoặc dấu gạch dưới (```_```), theo sau là chữ cái, chữ số hoặc dấu gạch dưới, không chứa khoảng trắng hay ký tự đặc biệt.</t>
         </is>
       </c>
       <c r="E38" s="3" t="inlineStr">
         <is>
-          <t>`26.0` thuộc kiểu `float`</t>
+          <t>```user name = "Alice"```, ```user#age = 25```, ```is_active = True```</t>
         </is>
       </c>
       <c r="F38" s="3" t="inlineStr">
         <is>
-          <t>Phương án nhiễu sai. Mẫu thuẫn này phát sinh khi học viên hiểu sai quy tắc kết hợp từ trái sang phải của phép chia lấy phần nguyên `//` và phép nhân `*`, tự ý nhóm `block_size * block_size` lại thành `25 // (4 * 4) = 1`, sau đó cộng với `25.0` dẫn đến kết quả `26.0`. Đúng ra `25 // 4` phải được tính trước ra `6` rồi mới nhân với `4` thành `24`.</t>
+          <t>Khai báo này vi phạm quy tắc do tên biến ```user name``` chứa khoảng trắng và tên biến ```user#age``` chứa ký tự đặc biệt ```#``` (ký tự này bắt đầu một ghi chú trong Python).</t>
         </is>
       </c>
       <c r="G38" s="3" t="inlineStr">
         <is>
-          <t>`24.5` thuộc kiểu `float`</t>
+          <t>```2user_name = "Alice"```, ```user-age = 25```, ```is_active = True```</t>
         </is>
       </c>
       <c r="H38" s="3" t="inlineStr">
         <is>
-          <t>Phương án nhiễu sai. Học viên mắc bẫy khi cho rằng toán tử chia lấy phần dư `%` được thực hiện trước toán tử lũy thừa `**`. Khi đó học viên tính `buffer_size % block_size` trước thành `25 % 4 = 1`, sau đó mới lấy `1 ** 2 = 1`, tiếp theo lấy `1 / 2 = 0.5` và cộng với `24` ra `24.5`. Điều này sai quy tắc ưu tiên toán tử vì `**` có độ ưu tiên cao hơn `%`.</t>
+          <t>Khai báo này thất bại và báo lỗi cú pháp vì tên biến ```2user_name``` bắt đầu bằng chữ số (vi phạm quy tắc) và tên biến ```user-age``` chứa ký tự dấu gạch ngang (```-```).</t>
         </is>
       </c>
       <c r="I38" s="3" t="inlineStr">
         <is>
-          <t>`28.5` thuộc kiểu `float`</t>
+          <t>```user@name = "Alice"```, ```$user_age = 25```, ```is_active = True```</t>
         </is>
       </c>
       <c r="J38" s="3" t="inlineStr">
         <is>
-          <t>Đáp án đúng A. Thứ tự ưu tiên của các toán tử số học trong Python được thực hiện theo quy tắc chuẩn:
-1. Toán tử lũy thừa `**` có độ ưu tiên cao nhất: `block_size ** 2` tương đương `4 ** 2 = 16`.
-2. Phép chia lấy phần nguyên `//`, phép nhân `*`, phép chia lấy phần dư `%` và phép chia số thực `/` có cùng độ ưu tiên và thực hiện từ trái sang phải:
-- `buffer_size // block_size` tương đương `25 // 4 = 6`.
-- `6 * block_size` tương đương `6 * 4 = 24`.
-- `buffer_size % 16` tương đương `25 % 16 = 9`.
-- `9 / 2` cho kết quả `4.5` (phép chia `/` trong Python luôn trả về kết quả kiểu `float`).
-3. Cuối cùng thực hiện phép cộng `+`: `24 + 4.5 = 28.5` (kết quả chuyển sang kiểu `float`).</t>
+          <t>Khai báo này vi phạm cú pháp do tên biến ```user@name``` chứa ký tự đặc biệt ```@``` và tên biến ```$user_age``` bắt đầu bằng ký tự đặc biệt ```$```.</t>
         </is>
       </c>
       <c r="K38" s="2" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="L38" s="2" t="n">
         <v>11</v>
@@ -3131,59 +2949,53 @@
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>Trong một kịch bản xử lý mã định danh dữ liệu console, lập trình viên kết hợp toán tử số học và chuyển đổi kiểu dữ liệu cơ bản trong Python 3.12 như sau:
+          <t>Xét đoạn mã nguồn Python 3.12 xử lý dữ liệu nhập vào từ bàn phím như sau:
 ```python
-unit_code = "8"
-multiplier = 3
-offset = 5
-result_val = int(unit_code * multiplier) // offset + float(unit_code) * 2
+raw_data = input("Nhập số lượng sản phẩm: ")
+converted_data = int(raw_data)
+print(type(converted_data))
 ```
-Giá trị và kiểu dữ liệu của biến `result_val` sau khi hoàn tất dòng lệnh là bao nhiêu?</t>
+Nếu người dùng nhập vào chuỗi chữ số ```"150"``` từ màn hình console, kết quả hiển thị kiểu dữ liệu thực tế trên console là gì?</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>`193.0` thuộc kiểu `float`</t>
+          <t>Kiểu dữ liệu hiển thị là `int` do hàm `int()` đã thực hiện chuyển đổi kiểu thành công từ chuỗi chữ số sang số nguyên.</t>
         </is>
       </c>
       <c r="D39" s="3" t="inlineStr">
         <is>
-          <t>Đáp án đúng A. Quá trình tính toán diễn ra theo từng bước quy chuẩn:
-1. Phép nhân chuỗi `unit_code * multiplier` tương đương `"8" * 3` tạo ra chuỗi lặp `"888"`.
-2. Hàm `int("888")` chuyển đổi chuỗi thành số nguyên `888`.
-3. Phép chia lấy phần nguyên `888 // 5` cho kết quả số nguyên `177` (vì `177 * 5 = 885`, dư `3`).
-4. Phép toán `float("8") * 2` thực hiện chuyển `"8"` thành `8.0` và nhân với `2` được `16.0`.
-5. Phép cộng giữa số nguyên và số thực `177 + 16.0` trả về kết quả số thực `193.0`.</t>
+          <t>Hàm `input()` luôn trả về dữ liệu kiểu chuỗi (`str`). Việc sử dụng hàm `int()` bọc ngoài giá trị `raw_data` đã chủ động chuyển đổi chuỗi `"150"` thành giá trị số nguyên `150`, do đó hàm `type(converted_data)` trả về kết quả là kiểu `int`.</t>
         </is>
       </c>
       <c r="E39" s="3" t="inlineStr">
         <is>
-          <t>`193` thuộc kiểu `int`</t>
+          <t>Kiểu dữ liệu hiển thị là `bool` do kết quả của thao tác ép kiểu dữ liệu từ bàn phím trả về trạng thái kiểm định logic.</t>
         </is>
       </c>
       <c r="F39" s="3" t="inlineStr">
         <is>
-          <t>Phương án nhiễu sai. Học viên chọn đáp án này do nhầm tưởng rằng vì `16.0` không có phần thập phân lẻ (phần thập phân bằng 0) nên Python sẽ tự động ép kiểu kết quả của phép cộng `177 + 16.0` về số nguyên `int`. Trong thực tế, khi thực hiện phép cộng giữa `int` và `float`, Python luôn tự động chuyển đổi kiểu dữ liệu thành `float`.</t>
+          <t>Đáp án này không chính xác vì hàm `int()` chuyển đổi chuỗi chữ số thành số nguyên chứ không biến đổi dữ liệu thành kiểu boolean (`bool`).</t>
         </is>
       </c>
       <c r="G39" s="3" t="inlineStr">
         <is>
-          <t>`20.8` thuộc kiểu `float`</t>
+          <t>Kiểu dữ liệu hiển thị là `str` do hàm `input()` mặc định trả về chuỗi văn bản và không thể bị thay đổi bởi hàm ép kiểu.</t>
         </is>
       </c>
       <c r="H39" s="3" t="inlineStr">
         <is>
-          <t>Phương án nhiễu sai. Học viên mắc sai lầm căn bản khi nghĩ rằng phép toán `unit_code * multiplier` thực hiện phép nhân số học `8 * 3 = 24` thay vì lặp chuỗi. Khi đó `int(24) // 5 = 4`, sau đó cộng với `16.8` hoặc tính sai toán tử dẫn tới đáp án `20.8`.</t>
+          <t>Đáp án này không chính xác vì hàm ép kiểu `int()` hoàn toàn có khả năng chuyển đổi một chuỗi ký tự chứa các chữ số hợp lệ thành kiểu số nguyên thực sự.</t>
         </is>
       </c>
       <c r="I39" s="3" t="inlineStr">
         <is>
-          <t>`177.6` thuộc kiểu `float`</t>
+          <t>Kiểu dữ liệu hiển thị là `float` do mọi dữ liệu số sau khi nhận qua giao diện console đều chuyển hóa tự động thành số thực.</t>
         </is>
       </c>
       <c r="J39" s="3" t="inlineStr">
         <is>
-          <t>Phương án nhiễu sai. Bẫy này xuất hiện khi học viên nhầm lẫn toán tử chia lấy phần nguyên `//` thành toán tử chia số thực `/`. Học viên tính `888 / 5 = 177.6` nhưng lại bỏ qua hoặc tính sai vế cộng `float(unit_code) * 2` ở phía sau.</t>
+          <t>Đáp án này không chính xác vì việc chuyển đổi sang kiểu số thực chỉ xảy ra khi sử dụng hàm `float()`, không tự động diễn ra khi dùng hàm `int()`.</t>
         </is>
       </c>
       <c r="K39" s="2" t="n">
@@ -3204,62 +3016,58 @@
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>Xét đoạn mã nguồn Python 3.12 sử dụng các toán tử gán gộp (augmented assignment operators) để cập nhật biến số như sau:
+          <t>Khi xây dựng ứng dụng giao diện console trong Python 3.12, thao tác xuất dữ liệu định dạng chuẩn được thực hiện qua hàm `print()`. Phân tích đoạn mã nguồn sau:
 ```python
-counter = 10
-scale = 2.5
-counter *= scale
-counter //= 3
-counter **= 2
+system_name = "Rikkei"
+sys_version = "3.12"
+sys_status = "Active"
+print(system_name, sys_version, sys_status, sep=" | ")
 ```
-Sau khi chạy đoạn mã trên, giá trị và kiểu dữ liệu của biến `counter` sẽ là gì?</t>
+Kết quả hiển thị chính xác của đoạn mã trên trên màn hình console là gì?</t>
         </is>
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>`64.0` thuộc kiểu `float`</t>
+          <t>Chuỗi văn bản `Rikkei | 3.12 | Active | ` xuất hiện trên một dòng kèm ký tự gạch đứng ` | ` bổ sung ở vị trí cuối cùng.</t>
         </is>
       </c>
       <c r="D40" s="3" t="inlineStr">
         <is>
-          <t>Đáp án đúng A. Diễn biến thay đổi giá trị và kiểu dữ liệu của biến `counter` qua từng dòng lệnh:
-1. `counter *= scale`: tương đương `counter = 10 * 2.5 = 25.0` (biến `counter` chuyển từ kiểu `int` sang kiểu `float`).
-2. `counter //= 3`: tương đương `counter = 25.0 // 3`. Do vế trái `25.0` mang kiểu `float`, toán tử `//` thực hiện chia lấy phần nguyên nhưng vẫn duy trì kiểu `float`, thu được `8.0`.
-3. `counter **= 2`: tương đương `counter = 8.0 ** 2 = 64.0` (kết quả giữ nguyên kiểu `float`).</t>
+          <t>Đáp án này không đúng vì tham số `sep` chỉ chèn ký tự phân cách giữa các đối số xuất ra, không chèn ký tự phân cách vào cuối chuỗi hiển thị.</t>
         </is>
       </c>
       <c r="E40" s="3" t="inlineStr">
         <is>
-          <t>`72.25` thuộc kiểu `float`</t>
+          <t>Ba chuỗi văn bản `Rikkei`, `3.12` và `Active` xuất hiện xuống dòng lần lượt trên ba dòng màn hình console khác nhau.</t>
         </is>
       </c>
       <c r="F40" s="3" t="inlineStr">
         <is>
-          <t>Phương án nhiễu sai. Nguyên nhân do học viên tính toán sai bước chia lấy phần nguyên: thay vì tính `25.0 // 3 = 8.0`, học viên thực hiện phép chia thường `25.0 / 3` ra `8.5` (nhầm dữ liệu toán tử), rồi lấy `8.5 ** 2 = 72.25`.</t>
+          <t>Đáp án này không đúng vì việc xuống dòng tự động sau từng đối số chỉ xảy ra nếu tham số `sep` được truyền vào ký tự xuống dòng `\n`.</t>
         </is>
       </c>
       <c r="G40" s="3" t="inlineStr">
         <is>
-          <t>`64.25` thuộc kiểu `float`</t>
+          <t>Chuỗi văn bản `Rikkei | 3.12 | Active` xuất hiện trên một dòng duy nhất với ký tự nối ` | ` nằm giữa các giá trị.</t>
         </is>
       </c>
       <c r="H40" s="3" t="inlineStr">
         <is>
-          <t>Phương án nhiễu sai. Bẫy này xảy ra khi học viên nhầm lẫn giữa toán tử chia lấy phần nguyên `//` và toán tử chia số thực `/`. Học viên tính `25.0 / 3` ra `8.333...`, sau đó lũy thừa hoặc làm tròn sai dẫn tới giá trị `64.25`.</t>
+          <t>Trong hàm `print()`, tham số `sep` (separator) quy định ký tự phân cách nằm giữa các đối số được truyền vào. Giá trị `sep=" | "` sẽ chèn chuỗi `" | "` vào giữa các giá trị `system_name`, `sys_version` và `sys_status` mà không thêm vào cuối dòng.</t>
         </is>
       </c>
       <c r="I40" s="3" t="inlineStr">
         <is>
-          <t>`64` thuộc kiểu `int`</t>
+          <t>Chuỗi văn bản `Rikkei 3.12 Active` xuất hiện trên một dòng duy nhất và tham số `sep=" | "` bị trình biên dịch bỏ qua.</t>
         </is>
       </c>
       <c r="J40" s="3" t="inlineStr">
         <is>
-          <t>Phương án nhiễu sai. Học viên hiểu sai cơ chế của toán tử gán gộp chia lấy phần nguyên `//=`. Học viên cho rằng toán tử `//` luôn ép kết quả về kiểu số nguyên `int`. Tuy nhiên trong Python, nếu toán hạng là `float`, kết quả của phép `//` vẫn là một số thực `float` với phần thập phân là `.0` (ví dụ `25.0 // 3` ra `8.0`).</t>
+          <t>Đáp án này không đúng vì tham số `sep` ghi đè ký tự khoảng trắng mặc định thành chuỗi phân cách được chỉ định là `" | "`.</t>
         </is>
       </c>
       <c r="K40" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="L40" s="2" t="n">
         <v>11</v>
@@ -3276,61 +3084,57 @@
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>Xét đoạn mã Python 3.12 thực hiện các phép toán trên số nguyên dưới đây:
+          <t>Trong Python 3.12, một nhà phát triển thực hiện đoạn mã xử lý dữ liệu đầu vào và kiểm tra kiểu như sau:
 ```python
-initial_value = -3 ** 2 % 4 // 2
-print(f"Result: {initial_value}")
+data = "100"
+data = int(data) + 50
+result_type = type(data)
 ```
-Kết quả màn hình Console hiển thị là gì?</t>
+Giá trị thực tế của biến `result_type` lưu trữ thông tin kiểu dữ liệu là gì?</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>Result: -1</t>
+          <t>Phát sinh lỗi `TypeError`, vì Python là ngôn ngữ định kiểu tĩnh không cho phép gán kiểu dữ liệu khác cho biến đã tạo.</t>
         </is>
       </c>
       <c r="D41" s="3" t="inlineStr">
         <is>
-          <t>ĐÁP ÁN SAI. Lỗi sai xảy ra khi học viên áp dụng quy tắc phép dư `%` của ngôn ngữ C/C++ (trong C: `-9 % 4 = -1`). Sau đó lấy `-1 // 2` và cho rằng kết quả bằng `-1`. Thực tế Python quy định `a % b` luôn mang dấu của số chia `b`, nên `-9 % 4` bằng `3`, dẫn tới `3 // 2 = 1`.</t>
+          <t>Python là ngôn ngữ định kiểu động (dynamic typing), cho phép một biến có thể gán lại các giá trị mang kiểu dữ liệu khác nhau ở các thời điểm khác nhau mà không gây ra lỗi `TypeError`.</t>
         </is>
       </c>
       <c r="E41" s="3" t="inlineStr">
         <is>
-          <t>Result: 1</t>
+          <t>Kiểu `&lt;class 'float'&gt;`, vì phép cộng số học trong Python tự động ép kiểu dữ liệu kết quả về dạng số thực.</t>
         </is>
       </c>
       <c r="F41" s="3" t="inlineStr">
         <is>
-          <t>ĐÁP ÁN ĐÚNG. Trong Python, thứ tự ưu tiên của các toán tử số học được quy định rất chặt chẽ:
-1. Toán tử lũy thừa `**` có độ ưu tiên cao hơn toán tử âm một ngôi `-`. Do đó `-3 ** 2` được thực hiện là `-(3 ** 2) = -9` (chứ không phải `(-3)**2 = 9`).
-2. Tiếp theo, các toán tử chia lấy dư `%` và chia lấy phần nguyên `//` có cùng độ ưu tiên, thực hiện lần lượt từ trái sang phải.
-3. Phép tính `-9 % 4`: Trong Python, kết quả của phép chia lấy dư `%` luôn cùng dấu với số chia (`4`). Ta có `-9 = -3 * 4 + 3`, do đó `-9 % 4` trả về `3`.
-4. Phép tính `3 // 2`: Phép chia lấy phần nguyên của `3` cho `2` trả về `1`.
-Do đó, biến `initial_value` nhận giá trị `1` và màn hình in ra `Result: 1`.</t>
+          <t>Phép cộng giữa hai số nguyên (`100` và `50`) trong Python tạo ra một kết quả số nguyên (`int`), không tự động biểu diễn thành số thực (`float`).</t>
         </is>
       </c>
       <c r="G41" s="3" t="inlineStr">
         <is>
-          <t>Result: 0</t>
+          <t>Kiểu `&lt;class 'int'&gt;`, vì chuỗi `"100"` đã được chuyển đổi thành số nguyên trước khi thực hiện phép cộng với `50`.</t>
         </is>
       </c>
       <c r="H41" s="3" t="inlineStr">
         <is>
-          <t>ĐÁP ÁN SAI. Lỗi sai này xuất phát từ việc hiểu sai thứ tự ưu tiên của toán tử âm một ngôi `-` và toán tử lũy thừa `**`. Người học lầm tưởng `-3 ** 2` tính ra `(-3)**2 = 9`. Khi đó: `9 % 4 = 1`, sau đó `1 // 2 = 0`. Tuy nhiên trong Python, `**` ưu tiên cao hơn `-` nên `-3 ** 2` phải là `-9`.</t>
+          <t>Hàm `int("100")` chuyển đổi thành công chuỗi `"100"` thành giá trị số nguyên `100`. Khi thực hiện phép cộng với số nguyên `50`, kết quả thu được là `150` thuộc kiểu `int`. Do đó, `type(data)` trả về `&lt;class 'int'&gt;`.</t>
         </is>
       </c>
       <c r="I41" s="3" t="inlineStr">
         <is>
-          <t>Result: -4</t>
+          <t>Kiểu `&lt;class 'str'&gt;`, vì biến `data` ban đầu được khởi tạo dưới dạng một chuỗi ký tự.</t>
         </is>
       </c>
       <c r="J41" s="3" t="inlineStr">
         <is>
-          <t>ĐÁP ÁN SAI. Lỗi sai này do người học áp dụng sai quy tắc tính toán của toán tử chia lấy phần nguyên `//` và chia lấy dư `%` khi làm việc với số âm, dẫn tới việc tính toán sai lệch kết quả trung gian.</t>
+          <t>Python là ngôn ngữ sử dụng cơ chế định kiểu động (dynamic typing). Khi gán lại `data = int(data) + 50`, kiểu dữ liệu của `data` đã thay đổi từ `str` sang `int`, không giữ lại kiểu ban đầu.</t>
         </is>
       </c>
       <c r="K41" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L41" s="2" t="n">
         <v>11</v>
@@ -3347,67 +3151,57 @@
       </c>
       <c r="B42" s="3" t="inlineStr">
         <is>
-          <t>Cho đoạn mã Python 3.12 xử lý chuỗi và số học như sau:
+          <t>Trong quá trình khai báo các biến để lưu trữ thông tin hệ thống bằng Python 3.12, đoạn mã sau được thực thi:
 ```python
-item_code = "A"
-repeat_count = 5 // 2 + 3 * 2 % 4
-item_code *= repeat_count
-item_code += str(10 / 2)
-print(f"Output: {item_code}")
+_user_id = 101
+user_name = "Alice"
+2nd_score = 95.5
 ```
-Kết quả in ra màn hình Console là gì?</t>
+Dòng mã nào sẽ gây ra lỗi cú pháp `SyntaxError` do vi phạm quy tắc đặt tên biến?</t>
         </is>
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>Output: AAAAA5</t>
+          <t>Dòng `_user_id = 101`, vì tên biến trong Python không được phép chứa dấu gạch dưới `_` ở vị trí đầu tiên.</t>
         </is>
       </c>
       <c r="D42" s="3" t="inlineStr">
         <is>
-          <t>ĐÁP ÁN SAI. Học viên mắc đồng thời 2 lỗi tư duy: (1) Tính sai `repeat_count = 5` dẫn tới chuỗi `"AAAAA"` và (2) Nhầm lẫn toán tử chia `/` trả về kiểu `int` (`5`) thay vì `float` (`5.0`), dẫn tới kết quả ghép chuỗi bị thiếu phần thập phân.</t>
+          <t>Tên biến bắt đầu bằng dấu gạch dưới `_` như `_user_id` là hoàn toàn hợp lệ trong cú pháp Python và thường được dùng theo quy ước định danh.</t>
         </is>
       </c>
       <c r="E42" s="3" t="inlineStr">
         <is>
-          <t>Output: AAAAA5.0</t>
+          <t>Cả ba dòng mã trên đều vi phạm quy tắc đặt tên biến và làm cho trình thông dịch dừng hoạt động.</t>
         </is>
       </c>
       <c r="F42" s="3" t="inlineStr">
         <is>
-          <t>ĐÁP ÁN SAI. Lỗi do tính sai giá trị của `repeat_count`. Học viên nhầm lẫn phép chia phần nguyên `5 // 2` ra `2.5` rồi làm tròn lên `3`, dẫn đến `repeat_count = 5`, khiến chuỗi `"A"` bị nhân bản thành 5 lần `"AAAAA"`.</t>
+          <t>Hai dòng mã `_user_id = 101` và `user_name = "Alice"` hoàn toàn hợp lệ theo quy tắc cú pháp Python, chỉ có dòng `2nd_score = 95.5` vi phạm.</t>
         </is>
       </c>
       <c r="G42" s="3" t="inlineStr">
         <is>
-          <t>Output: AAAA5</t>
+          <t>Dòng `2nd_score = 95.5`, vì tên biến trong Python tuyệt đối không được phép bắt đầu bằng một chữ số.</t>
         </is>
       </c>
       <c r="H42" s="3" t="inlineStr">
         <is>
-          <t>ĐÁP ÁN SAI. Học viên mắc bẫy khi cho rằng phép chia `/` với hai số nguyên chia hết (`10 / 2`) sẽ trả về số nguyên `5` (`int`). Thực tế trong Python 3, toán tử `/` luôn trả về số thực (`float`), do đó `str(10 / 2)` cho kết quả `"5.0"` chứ không phải `"5"`.</t>
+          <t>Theo quy tắc đặt tên biến chuẩn của Python, tên biến chỉ có thể bắt đầu bằng một chữ cái (a-z, A-Z) hoặc dấu gạch dưới `_`. Tên biến `2nd_score` bắt đầu bằng chữ số `2` nên trình thông dịch báo lỗi `SyntaxError`.</t>
         </is>
       </c>
       <c r="I42" s="3" t="inlineStr">
         <is>
-          <t>Output: AAAA5.0</t>
+          <t>Dòng `user_name = "Alice"`, vì dấu gạch dưới `_` nối giữa các từ bị cấm sử dụng trong khai báo biến.</t>
         </is>
       </c>
       <c r="J42" s="3" t="inlineStr">
         <is>
-          <t>ĐÁP ÁN ĐÚNG. Phân tích chi tiết từng bước thực thi:
-1. Phép tính `repeat_count = 5 // 2 + 3 * 2 % 4`:
-   - `5 // 2` (chia lấy phần nguyên) = `2`.
-   - `3 * 2 % 4`: Toán tử `*` và `%` có cùng độ ưu tiên nên tính từ trái sang phải: `3 * 2 = 6`, sau đó `6 % 4 = 2`.
-   - `repeat_count = 2 + 2 = 4`.
-2. `item_code *= 4`: Toán tử `*` giữa chuỗi `"A"` và số nguyên `4` thực hiện nhân bản chuỗi 4 lần -&gt; `item_code` trở thành `"AAAA"`.
-3. `10 / 2`: Trong Python, toán tử chia trôi `/` LUÔN LUÔN trả về kiểu dữ liệu số thực (`float`), nên `10 / 2` cho kết quả `5.0`.
-4. `str(5.0)` chuyển đổi số thực thành chuỗi `"5.0"`.
-5. `item_code += "5.0"` thực hiện phép nối chuỗi -&gt; `"AAAA5.0"`.</t>
+          <t>Tên biến `user_name` sử dụng dấu gạch dưới để phân tách các từ tuân thủ đúng cú pháp Python và chuẩn trình bày snake_case.</t>
         </is>
       </c>
       <c r="K42" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L42" s="2" t="n">
         <v>11</v>
@@ -3424,70 +3218,58 @@
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>Xét đoạn mã Python 3.12 thực thi các phép toán so sánh và ép kiểu ngầm định dưới đây:
+          <t>Giả sử người dùng nhập vào từ bàn phím lần lượt hai giá trị là `10` và `20` khi trình thông dịch Python 3.12 thực thi đoạn mã sau:
 ```python
-base_num = 15
-is_even = base_num % 2 == 0
-multiplier = (base_num &gt; 10) + (base_num == 15) * 2
-result_value = base_num * multiplier + is_even
-print(f"Result: {result_value}")
+val1 = input("Nhập số thứ nhất: ")
+val2 = input("Nhập số thứ hai: ")
+result = val1 + val2
+print(result)
 ```
-Kết quả hiển thị trên màn hình Console là gì?</t>
+Kết quả hiển thị ra màn hình console của câu lệnh `print(result)` là gì?</t>
         </is>
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>Result: 46</t>
+          <t>`30`, vì trình thông dịch tự động nhận diện chuỗi ký tự chứa chữ số và thực hiện phép tính cộng số học.</t>
         </is>
       </c>
       <c r="D43" s="3" t="inlineStr">
         <is>
-          <t>ĐÁP ÁN SAI. Lỗi sai do học viên hiểu nhầm giá trị số nguyên ngầm định của biến kiểu boolean `is_even`. Học viên nghĩ `False` khi tham gia phép cộng số học sẽ được chuyển thành `1` (hoặc nhầm kết quả `15 % 2 == 0` thành `True`), dẫn đến phép tính `45 + 1 = 46`.</t>
+          <t>Python không tự động chuyển đổi dữ liệu kiểu `str` nhận từ `input()` sang kiểu `int`. Để thu được kết quả số học `30`, cần thực hiện ép kiểu rõ ràng như `int(input())`.</t>
         </is>
       </c>
       <c r="E43" s="3" t="inlineStr">
         <is>
-          <t>Result: 31</t>
+          <t>`1020`, vì hàm `input()` luôn trả về kiểu dữ liệu chuỗi (`str`), dẫn đến toán tử `+` thực hiện phép nối chuỗi.</t>
         </is>
       </c>
       <c r="F43" s="3" t="inlineStr">
         <is>
-          <t>ĐÁP ÁN SAI. Lỗi sai này xảy ra khi học viên tính sai thứ tự ưu tiên toán tử trong biểu thức `multiplier`, thực hiện phép cộng trước phép nhân: `(True + True) * 2` = `(1 + 1) * 2 = 4`, dẫn tới `15 * 2 + 1 = 31` do tính toán sai biến `multiplier` và cấu trúc biểu thức.</t>
+          <t>Dữ liệu trả về từ hàm `input()` mặc định luôn thuộc kiểu chuỗi (`str`). Khi áp dụng toán tử `+` giữa hai chuỗi `"10"` và `"20"`, Python thực hiện phép nối chuỗi tạo ra kết quả `"1020"`.</t>
         </is>
       </c>
       <c r="G43" s="3" t="inlineStr">
         <is>
-          <t>Result: 16</t>
+          <t>`30.0`, vì toàn bộ dữ liệu nhập vào từ bàn phím qua `input()` tự động chuyển về kiểu số thực (`float`).</t>
         </is>
       </c>
       <c r="H43" s="3" t="inlineStr">
         <is>
-          <t>ĐÁP ÁN SAI. Lỗi sai xuất phát từ tư duy cho rằng giá trị kiểu `bool` (`True`/`False`) không thể trực tiếp tham gia tính toán số học (`+`, `*`) với số nguyên trong Python, dẫn tới việc bỏ qua các biểu thức so sánh và tính sai toàn bộ giá trị của `multiplier`.</t>
+          <t>Hàm `input()` không tự động ép kiểu dữ liệu về `float`. Giá trị nhận được nguyên bản từ console luôn là một chuỗi ký tự (`str`).</t>
         </is>
       </c>
       <c r="I43" s="3" t="inlineStr">
         <is>
-          <t>Result: 45</t>
+          <t>Phát sinh lỗi `TypeError`, vì toán tử `+` không được hỗ trợ để làm việc với các biến nhận từ hàm `input()`.</t>
         </is>
       </c>
       <c r="J43" s="3" t="inlineStr">
         <is>
-          <t>ĐÁP ÁN ĐÚNG. Phân tích chi tiết từng bước thực thi:
-1. `is_even = 15 % 2 == 0`: Phép toán chia lấy dư `%` được ưu tiên trước phép so sánh `==`. `15 % 2` bằng `1`, `1 == 0` trả về giá trị kiểu boolean là `False`.
-2. `multiplier = (base_num &gt; 10) + (base_num == 15) * 2`:
-   - `(15 &gt; 10)` trả về `True`.
-   - `(15 == 15)` trả về `True`.
-   - Phép nhân `*` ưu tiên hơn phép cộng `+`: `(True) * 2` ép kiểu ngầm định `True` thành `1`, tính ra `1 * 2 = 2`.
-   - Tiếp theo `True + 2` ép kiểu `True` thành `1`, tính ra `1 + 2 = 3`.
-   - Do đó `multiplier = 3`.
-3. `result_value = 15 * 3 + False`:
-   - `15 * 3 = 45`.
-   - Trong phép cộng số học, `False` được ép kiểu ngầm định thành số `0` (`45 + 0 = 45`).
-Kết quả in ra màn hình là `Result: 45`.</t>
+          <t>Toán tử `+` hoạt động hoàn toàn hợp lệ đối với hai đối tượng kiểu chuỗi (`str`) dưới cơ chế nối chuỗi, do đó chương trình không phát sinh lỗi `TypeError`.</t>
         </is>
       </c>
       <c r="K43" s="2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L43" s="2" t="n">
         <v>11</v>
@@ -3504,62 +3286,51 @@
       </c>
       <c r="B44" s="3" t="inlineStr">
         <is>
-          <t>Phân tích thứ tự ưu tiên toán tử và cơ chế xử lý số âm của phép chia lấy phần nguyên `//`, phép chia lấy dư `%`, toán tử lũy thừa `**` và toán tử đổi dấu một ngôi `-` trong Python 3.12 qua đoạn mã sau:
-```python
-initial_val = 5
-result_a = -initial_val ** 2 // 3 % 4
-result_b = (-initial_val) ** 2 // 3 % 4
-final_output = f"{result_a}_{result_b}"
-print(final_output)
-```
-Giá trị được in ra màn hình của biến `final_output` là bao nhiêu?</t>
+          <t>Khi thực hiện lưu trữ giá trị doanh thu hàng tháng trong ứng dụng Python 3.12, khai báo biến nào sau đây tuân thủ đúng quy tắc đặt tên định danh (identifier) và chuẩn snake_case?</t>
         </is>
       </c>
       <c r="C44" s="3" t="inlineStr">
         <is>
-          <t>-1_0</t>
+          <t>`1st_monthly_revenue = 150000.5`</t>
         </is>
       </c>
       <c r="D44" s="3" t="inlineStr">
         <is>
-          <t>Sai. Học viên gặp bẫy ở toán tử chia lấy dư `%` với số âm. Trong nhiều ngôn ngữ lập trình khác, biểu thức `-9 % 4` trả về kết quả âm là `-1`. Tuy nhiên trong Python, kết quả của toán tử `%` luôn cùng dấu với số chia `b` (ở đây `b = 4` là số dương), nên `-9 % 4` phải trả về `3`. Chọn `-1_0` phản ánh tư duy sai lầm do áp dụng quy tắc toán tử của ngôn ngữ khác vào Python.</t>
+          <t>Khai báo `1st_monthly_revenue = 150000.5` vi phạm quy tắc đặt tên trong Python do tên định danh không được phép bắt đầu bằng chữ số (`1`), gây ra lỗi `SyntaxError` khi chương trình thực thi.</t>
         </is>
       </c>
       <c r="E44" s="3" t="inlineStr">
         <is>
-          <t>3_0</t>
+          <t>`monthly revenue = 150000.5`</t>
         </is>
       </c>
       <c r="F44" s="3" t="inlineStr">
         <is>
-          <t>Chính xác. Phương án này tính toán hoàn toàn đúng theo quy tắc ưu tiên toán tử trong Python:
-- Với `result_a`: Toán tử lũy thừa `**` có độ ưu tiên cao hơn toán tử đổi dấu một ngôi `-`. Do đó, `-initial_val ** 2` được tính thành `-(5 ** 2) = -25`. Tiếp theo, phép chia lấy phần nguyên `-25 // 3` trong Python luôn làm tròn xuống về phía âm vô cực (floor towards negative infinity), thu được `-9` (vì `-9 * 3 = -27 &lt;= -25`). Sau đó, phép chia lấy dư `-9 % 4` áp dụng công thức `r = a - (b * (a // b))` trả về kết quả `-9 - (4 * (-9 // 4)) = -9 - (4 * (-3)) = 3`.
-- Với `result_b`: Cặp dấu ngoặc đơn ép buộc thực hiện `(-5) ** 2 = 25` trước. Tiếp theo `25 // 3 = 8` và `8 % 4 = 0`.
-- Kết hợp chuỗi f-string tạo thành giá trị `"3_0"`.</t>
+          <t>Khai báo `monthly revenue = 150000.5` vi phạm quy tắc định danh vì tên biến trong Python tuyệt đối không được chứa khoảng trắng, dẫn đến lỗi cú pháp `SyntaxError`.</t>
         </is>
       </c>
       <c r="G44" s="3" t="inlineStr">
         <is>
-          <t>-8_0</t>
+          <t>`monthly-revenue = 150000.5`</t>
         </is>
       </c>
       <c r="H44" s="3" t="inlineStr">
         <is>
-          <t>Sai. Học viên chọn đáp án này do hiểu sai quy tắc làm tròn của toán tử chia lấy phần nguyên `//` đối với số âm trong Python. Học viên đã tính `-25 // 3 = -8` (làm tròn cắt phần thập phân về phía số 0 giống như các ngôn ngữ C/C++/Java) thay vì `-9` (làm tròn về phía âm vô cực trong Python). Nếu `-25 // 3` ra `-8`, phép toán tiếp theo `-8 % 4` sẽ ra `0`, dẫn đến kết quả sai lệch hoàn toàn là `-8_0`.</t>
+          <t>Khai báo `monthly-revenue = 150000.5` không hợp lệ vì chứa dấu gạch nối `-`, trình biên dịch Python sẽ hiểu nhầm đây là phép toán trừ giữa hai biến `monthly` và `revenue` thay vì một tên biến duy nhất.</t>
         </is>
       </c>
       <c r="I44" s="3" t="inlineStr">
         <is>
-          <t>3_2</t>
+          <t>`monthly_revenue = 150000.5`</t>
         </is>
       </c>
       <c r="J44" s="3" t="inlineStr">
         <is>
-          <t>Sai. Học viên đã tính chính xác giá trị của `result_a` (`3`) nhưng lại tính sai ở `result_b`. Trong biểu thức `8 % 4`, do 8 chia hết hoàn toàn cho 4 nên phần dư đúng phải là `0` chứ không phải `2`.</t>
+          <t>Khai báo `monthly_revenue = 150000.5` hợp lệ vì tên biến bắt đầu bằng chữ cái, chỉ chứa chữ cái, chữ số và dấu gạch dưới `_`, đồng thời tuân thủ chuẩn quy ước đặt tên snake_case trong Python.</t>
         </is>
       </c>
       <c r="K44" s="2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L44" s="2" t="n">
         <v>11</v>
@@ -3576,62 +3347,57 @@
       </c>
       <c r="B45" s="3" t="inlineStr">
         <is>
-          <t>Phân tích độ ưu tiên giữa toán tử số học (`+`) và các toán tử thao tác bit (bitwise operators: `&lt;&lt;`, `^`) trong Python 3.12 thông qua chương trình dưới đây:
+          <t>Xem xét đoạn mã nguồn Python xử lý dữ liệu nhập từ người dùng như sau:
 ```python
-raw_bits = 5
-step_a = raw_bits &lt;&lt; 2 + 1
-step_b = step_a ^ 15
-output_data = f"{step_a}:{step_b}"
-print(output_data)
+user_input = input("Nhập tuổi của bạn: ")
+age = int(user_input)
+print(type(age))
 ```
-Kết quả xuất ra màn hình console của biến `output_data` là gì?</t>
+Khi người dùng nhập chuỗi `"25"` từ giao diện console, kết quả hiển thị của lệnh `print(type(age))` là gì?</t>
         </is>
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t>40:39</t>
+          <t>`&lt;class 'bool'&gt;`</t>
         </is>
       </c>
       <c r="D45" s="3" t="inlineStr">
         <is>
-          <t>Chính xác. Phân tích từng bước thực thi toán tử:
-- Trong Python, toán tử số học cộng `+` có độ ưu tiên CAO HƠN toán tử dịch trái bit `&lt;&lt;`. Do đó, biểu thức `raw_bits &lt;&lt; 2 + 1` sẽ thực hiện phép cộng `2 + 1 = 3` trước, sau đó mới thực hiện phép dịch bit `5 &lt;&lt; 3`. Phép dịch trái `5 &lt;&lt; 3` tương đương với `5 * (2 ** 3) = 40`, nên `step_a = 40`.
-- Tiếp theo, tính `step_b = 40 ^ 15`: Chuyển đổi sang hệ nhị phân, 40 là `0010 1000`, 15 là `0000 1111`. Toán tử XOR `^` trả về bit `1` khi hai bit thành phần khác nhau, kết quả thu được là `0010 0111` (giá trị thập phân tương ứng là `39`).
-- Kết hợp f-string trả về chuỗi `"40:39"`.</t>
+          <t>Hàm `int()` chỉ chuyển đổi dữ liệu chuỗi chữ số thành số nguyên, không phải kiểu dữ liệu luận lý (Boolean) `&lt;class 'bool'&gt;`.</t>
         </is>
       </c>
       <c r="E45" s="3" t="inlineStr">
         <is>
-          <t>21:26</t>
+          <t>`&lt;class 'float'&gt;`</t>
         </is>
       </c>
       <c r="F45" s="3" t="inlineStr">
         <is>
-          <t>Sai. Đây là bẫy phổ biến khi học viên nhầm lẫn rằng toán tử dịch bit `&lt;&lt;` có độ ưu tiên cao hơn toán tử số học `+`. Nếu tính toán sai thứ tự thành `(5 &lt;&lt; 2) + 1`, ta sẽ thu được `20 + 1 = 21` cho `step_a`. Sau đó tính `21 ^ 15` (nhị phân `0001 0101 ^ 0000 1111`) ra `0001 1010` (tức `26`), dẫn đến đáp án nhiễu `21:26`.</t>
+          <t>Hàm `int()` thực hiện chuyển đổi dữ liệu sang kiểu số nguyên, không phải kiểu số thực `&lt;class 'float'&gt;`.</t>
         </is>
       </c>
       <c r="G45" s="3" t="inlineStr">
         <is>
-          <t>40:55</t>
+          <t>`&lt;class 'int'&gt;`</t>
         </is>
       </c>
       <c r="H45" s="3" t="inlineStr">
         <is>
-          <t>Sai. Học viên chọn đáp án này đã nắm vững độ ưu tiên để tính đúng `step_a = 40`, nhưng lại nhầm lẫn toán tử Bitwise XOR `^` với toán tử Bitwise OR `|` ở bước `step_b`. Phép tính `40 | 15` (nhị phân `0010 1000 | 0000 1111`) mới cho ra kết quả `0010 1111` (tương ứng `47`) hoặc thực hiện sai phép tính bitwise.</t>
+          <t>Hàm `input()` mặc định trả về dữ liệu kiểu chuỗi `str`. Khi gọi hàm `int(user_input)`, giá trị chuỗi `"25"` được chuyển đổi thành số nguyên, do đó kết quả kiểm tra kiểu bằng `type(age)` trả về `&lt;class 'int'&gt;`.</t>
         </is>
       </c>
       <c r="I45" s="3" t="inlineStr">
         <is>
-          <t>20:27</t>
+          <t>`&lt;class 'str'&gt;`</t>
         </is>
       </c>
       <c r="J45" s="3" t="inlineStr">
         <is>
-          <t>Sai. Học viên mắc sai lầm khi bỏ qua toán tử `+ 1` trong biểu thức (chỉ tính `5 &lt;&lt; 2 = 20`) hoặc tính sai hoàn toàn quy tắc chuyển đổi nhị phân của toán tử dịch bit và toán tử XOR.</t>
+          <t>Mặc dù hàm `input()` trả về kiểu `str`, nhưng giá trị đã được thực hiện ép kiểu thông qua hàm `int()`, nên biến `age` không còn giữ kiểu chuỗi `&lt;class 'str'&gt;`.</t>
         </is>
       </c>
       <c r="K45" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="L45" s="2" t="n">
         <v>11</v>
@@ -3648,61 +3414,54 @@
       </c>
       <c r="B46" s="3" t="inlineStr">
         <is>
-          <t>Trong Python 3.12, việc kết hợp giữa kiểu dữ liệu số thực (`float`), toán tử chia phần nguyên `//`, toán tử chia lấy dư `%` và toán tử gán phức hợp `/=` tạo ra kết quả và kiểu dữ liệu như thế nào? Xét đoạn mã sau:
+          <t>Cho đoạn mã nguồn Python thu thập hai giá trị từ bàn phím và in ra màn hình console:
 ```python
-initial_score = 17.5
-divisor = 4.0
-part_1 = initial_score // divisor
-part_2 = initial_score % divisor
-initial_score /= divisor
-summary = f"{part_1}_{part_2}_{initial_score}"
-print(summary)
+val1 = input("Nhập số thứ nhất: ")
+val2 = input("Nhập số thứ hai: ")
+result = val1 + val2
+print(result)
 ```
-Giá trị của biến `summary` được in ra console là gì?</t>
+Nếu người dùng nhập lần lượt `10` cho `val1` và `20` cho `val2`, kết quả in ra màn hình console là gì và vì sao?</t>
         </is>
       </c>
       <c r="C46" s="3" t="inlineStr">
         <is>
-          <t>4.375_1.5_4.375</t>
+          <t>Báo lỗi `TypeError` vì không thể dùng toán tử `+` tác động lên các giá trị dữ liệu được thu thập từ hàm `input()`.</t>
         </is>
       </c>
       <c r="D46" s="3" t="inlineStr">
         <is>
-          <t>Sai. Học viên nhầm lẫn giữa toán tử chia lấy phần nguyên `//` và toán tử chia số thực thông thường `/`. Phép tính `17.5 // 4.0` bị tính sai thành phép chia thông thường `17.5 / 4.0 = 4.375`.</t>
+          <t>Toán tử `+` là hợp lệ đối với kiểu chuỗi `str` trong Python để thực hiện ghép chuỗi, do đó không phát sinh lỗi `TypeError`.</t>
         </is>
       </c>
       <c r="E46" s="3" t="inlineStr">
         <is>
-          <t>4.0_1.5_4.375</t>
+          <t>Hiển thị `1020` vì hàm `input()` luôn trả về dữ liệu kiểu chuỗi `str`, toán tử `+` giữa hai chuỗi sẽ thực hiện phép nối chuỗi.</t>
         </is>
       </c>
       <c r="F46" s="3" t="inlineStr">
         <is>
-          <t>Chính xác. Phân tích kiểu dữ liệu và toán tử số thực trong Python:
-- Với `part_1`: Khi thực hiện phép chia lấy phần nguyên `//` mà có ít nhất một toán hạng là kiểu số thực `float` (`17.5` và `4.0`), kết quả trả về bắt buộc mang kiểu `float` (`4.0` chứ không phải số nguyên `4`).
-- Với `part_2`: Phép chia lấy dư `%` giữa hai số thực `17.5 % 4.0` tính toán phần dư thực tế: `17.5 - (4.0 * 4.0) = 1.5` mang kiểu `float`.
-- Với `initial_score /= divisor`: Toán tử gán phức hợp `/=` thực hiện phép chia số thực thông thường `17.5 / 4.0 = 4.375` và gán lại cho `initial_score`.
-- Kết hợp f-string thu được kết quả chính xác: `"4.0_1.5_4.375"`.</t>
+          <t>Hàm `input()` luôn trả về dữ liệu kiểu chuỗi `str`. Khi áp dụng toán tử `+` giữa hai chuỗi `"10"` và `"20"`, Python thực hiện thao tác ghép chuỗi tạo thành chuỗi mới là `"1020"`.</t>
         </is>
       </c>
       <c r="G46" s="3" t="inlineStr">
         <is>
-          <t>4_1.5_4.375</t>
+          <t>Hiển thị `30.0` vì Python mặc định ép kiểu các giá trị dữ liệu nhập vào từ console thành số thực `float`.</t>
         </is>
       </c>
       <c r="H46" s="3" t="inlineStr">
         <is>
-          <t>Sai. Học viên mắc bẫy khi nghĩ rằng toán tử chia phần nguyên `//` luôn luôn ép kiểu kết quả về số nguyên `int`. Trong Python, nếu một trong các toán hạng tham gia phép tính `//` là `float`, kết quả vẫn giữ nguyên dạng `float` (tức `4.0` chứ không phải `4`).</t>
+          <t>Python không tự động ép kiểu dữ liệu từ `input()` sang số thực `float` mà giữ nguyên giá trị dưới dạng chuỗi ký tự `str`.</t>
         </is>
       </c>
       <c r="I46" s="3" t="inlineStr">
         <is>
-          <t>4.0_1.5_4</t>
+          <t>Hiển thị `30` vì Python tự động nhận diện các ký tự số `10` và `20` để thực hiện phép cộng số nguyên `int`.</t>
         </is>
       </c>
       <c r="J46" s="3" t="inlineStr">
         <is>
-          <t>Sai. Học viên hiểu đúng cơ chế của toán tử `//` và `%` nhưng lại hiểu sai toán tử gán phức hợp `/=`. Học viên đã nhầm lẫn toán tử `/=` là toán tử chia lấy phần nguyên (tương tự `//=`), làm cho biến `initial_score` bị cắt mất phần thập phân và thành `4` (hoặc `4.0`) thay vì `4.375`.</t>
+          <t>Python là ngôn ngữ định kiểu mạnh (strongly typed), không tự động chuyển đổi kiểu dữ liệu chuỗi chữ số từ `input()` thành số nguyên `int` để thực hiện phép cộng toán học.</t>
         </is>
       </c>
       <c r="K46" s="2" t="n">

</xml_diff>